<commit_message>
docs(knowledge): map validated Bungalov 4KK client facts
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 02.xlsx
+++ b/docs/knowledge/znalostní báze – mustr 02.xlsx
@@ -8278,13 +8278,17 @@
       </c>
       <c r="F384" s="11" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="G384" s="13" t="n"/>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G384" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Aktuální klientská konfigurace používá elektrické topné fólie.</t>
+        </is>
+      </c>
       <c r="H384" s="12" t="inlineStr">
         <is>
-          <t>B Souhrnná technická zpráva 11/2023, str. 24</t>
+          <t>B Souhrnná technická zpráva 11/2023, str. 24 / Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
         </is>
       </c>
       <c r="O384" s="13" t="n"/>
@@ -8371,13 +8375,17 @@
       </c>
       <c r="F387" s="11" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="G387" s="13" t="n"/>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G387" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Aktuální řešení používá systém řízeného větrání s rekuperací Zehnder ve výkonnější konfiguraci.</t>
+        </is>
+      </c>
       <c r="H387" s="12" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / Validace autora domu / CURRENT / 2026-09-09</t>
         </is>
       </c>
       <c r="O387" s="13" t="n"/>
@@ -9035,22 +9043,10 @@
           <t>Do jaké výšky jsou v koupelně obklady?</t>
         </is>
       </c>
-      <c r="E417" s="13" t="inlineStr">
-        <is>
-          <t>Koupelna má světle šedý obklad a dlažbu; zadní stěna sprchového koutu je v imitaci dřevěných latí.</t>
-        </is>
-      </c>
-      <c r="F417" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E417" s="13" t="n"/>
+      <c r="F417" s="11" t="n"/>
       <c r="G417" s="13" t="n"/>
-      <c r="H417" s="13" t="inlineStr">
-        <is>
-          <t>Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
-        </is>
-      </c>
+      <c r="H417" s="13" t="n"/>
       <c r="O417" s="13" t="n"/>
     </row>
     <row r="418" ht="15.75" customHeight="1" s="15">
@@ -10257,10 +10253,22 @@
           <t>Je možné vytvořit u ložnice samostatnou šatnu?</t>
         </is>
       </c>
-      <c r="E481" s="13" t="n"/>
-      <c r="F481" s="11" t="n"/>
+      <c r="E481" s="13" t="inlineStr">
+        <is>
+          <t>Ano. U ložnice je řešena integrovaná šatna bez sníženého podhledu.</t>
+        </is>
+      </c>
+      <c r="F481" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G481" s="13" t="n"/>
-      <c r="H481" s="13" t="n"/>
+      <c r="H481" s="13" t="inlineStr">
+        <is>
+          <t>Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
+        </is>
+      </c>
       <c r="O481" s="13" t="n"/>
     </row>
     <row r="482" ht="15.75" customHeight="1" s="15">
@@ -10937,10 +10945,22 @@
           <t>Co všechno je umístěné v technické místnosti?</t>
         </is>
       </c>
-      <c r="E517" s="13" t="n"/>
-      <c r="F517" s="11" t="n"/>
+      <c r="E517" s="13" t="inlineStr">
+        <is>
+          <t>V technické místnosti je v nice boiler, vzadu pod stropem technologická jednotka a před nimi prostor pro rozvaděč.</t>
+        </is>
+      </c>
+      <c r="F517" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G517" s="13" t="n"/>
-      <c r="H517" s="13" t="n"/>
+      <c r="H517" s="13" t="inlineStr">
+        <is>
+          <t>Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
+        </is>
+      </c>
       <c r="O517" s="13" t="n"/>
     </row>
     <row r="518" ht="15.75" customHeight="1" s="15">
@@ -12423,10 +12443,22 @@
           <t>Je možné terasu zastřešit?</t>
         </is>
       </c>
-      <c r="E595" s="13" t="n"/>
-      <c r="F595" s="11" t="n"/>
+      <c r="E595" s="13" t="inlineStr">
+        <is>
+          <t>Ano. U referenční realizace byla zastřešená plocha terasy klientskou změnou rozšířena.</t>
+        </is>
+      </c>
+      <c r="F595" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G595" s="13" t="n"/>
-      <c r="H595" s="13" t="n"/>
+      <c r="H595" s="13" t="inlineStr">
+        <is>
+          <t>Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
+        </is>
+      </c>
       <c r="O595" s="13" t="n"/>
     </row>
     <row r="596" ht="15.75" customHeight="1" s="15">

</xml_diff>

<commit_message>
docs(knowledge): ingest Bungalov 4KK visual study facts
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 02.xlsx
+++ b/docs/knowledge/znalostní báze – mustr 02.xlsx
@@ -1310,9 +1310,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Studie uvádí, že dům lze osadit také do svahu, zejména při umístění po vrstevnici.</t>
+        </is>
+      </c>
       <c r="H42" s="12" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 1 a 26</t>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 1 a 26 / Studie Bungalov 4KK / 01.11.2022</t>
         </is>
       </c>
       <c r="O42" s="13" t="n"/>
@@ -7896,10 +7901,22 @@
           <t>Je dům připravený pro nabíjení elektromobilu?</t>
         </is>
       </c>
-      <c r="E368" s="13" t="n"/>
-      <c r="F368" s="11" t="n"/>
+      <c r="E368" s="13" t="inlineStr">
+        <is>
+          <t>Studie počítá s možností dobíjení elektromobilu z dobíjecí stanice umístěné v zahradním domku.</t>
+        </is>
+      </c>
+      <c r="F368" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G368" s="13" t="n"/>
-      <c r="H368" s="13" t="n"/>
+      <c r="H368" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O368" s="13" t="n"/>
     </row>
     <row r="369" ht="15.75" customHeight="1" s="15">
@@ -9666,10 +9683,22 @@
           <t>Je možné mít v kuchyni ostrůvek?</t>
         </is>
       </c>
-      <c r="E450" s="13" t="n"/>
-      <c r="F450" s="11" t="n"/>
+      <c r="E450" s="13" t="inlineStr">
+        <is>
+          <t>Kuchyň je ve studii řešena s centrálním ostrůvkem.</t>
+        </is>
+      </c>
+      <c r="F450" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G450" s="13" t="n"/>
-      <c r="H450" s="13" t="n"/>
+      <c r="H450" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O450" s="13" t="n"/>
     </row>
     <row r="451" ht="15.75" customHeight="1" s="15">

</xml_diff>

<commit_message>
docs(knowledge): map additional Bungalov 4KK study facts
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 02.xlsx
+++ b/docs/knowledge/znalostní báze – mustr 02.xlsx
@@ -1310,7 +1310,7 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G42" s="0" t="inlineStr">
         <is>
           <t>Studie uvádí, že dům lze osadit také do svahu, zejména při umístění po vrstevnici.</t>
         </is>
@@ -2330,10 +2330,22 @@
           <t>Je kuchyň propojená s obývacím pokojem?</t>
         </is>
       </c>
-      <c r="E92" s="13" t="n"/>
-      <c r="F92" s="11" t="n"/>
+      <c r="E92" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Kuchyň je přímo propojená s obývacím pokojem a jídelnou do jednoho hlavního obytného prostoru.</t>
+        </is>
+      </c>
+      <c r="F92" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G92" s="13" t="n"/>
-      <c r="H92" s="13" t="n"/>
+      <c r="H92" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O92" s="13" t="n"/>
     </row>
     <row r="93" ht="15.75" customHeight="1" s="15">
@@ -2841,10 +2853,22 @@
           <t>Je možné k domu přidat pergolu nebo zastřešení terasy?</t>
         </is>
       </c>
-      <c r="E119" s="13" t="n"/>
-      <c r="F119" s="11" t="n"/>
+      <c r="E119" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Koncept domu pracuje s velkou krytou terasou navázanou na zahradní stranu domu.</t>
+        </is>
+      </c>
+      <c r="F119" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G119" s="13" t="n"/>
-      <c r="H119" s="13" t="n"/>
+      <c r="H119" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O119" s="13" t="n"/>
     </row>
     <row r="120" ht="15.75" customHeight="1" s="15">
@@ -6328,10 +6352,14 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="G293" s="13" t="n"/>
+      <c r="G293" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Studie navrhuje střechu se sklonem 30° jako vhodnou pro integrovanou fotovoltaiku.</t>
+        </is>
+      </c>
       <c r="H293" s="12" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / Studie Bungalov 4KK / 01.11.2022</t>
         </is>
       </c>
       <c r="O293" s="13" t="n"/>
@@ -10206,10 +10234,22 @@
           <t>Je možné jeden dětský pokoj využít jako pracovnu?</t>
         </is>
       </c>
-      <c r="E477" s="13" t="n"/>
-      <c r="F477" s="11" t="n"/>
+      <c r="E477" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Jeden z pokojů je koncipován flexibilně pro využití jako dětský pokoj nebo pracovna.</t>
+        </is>
+      </c>
+      <c r="F477" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G477" s="13" t="n"/>
-      <c r="H477" s="13" t="n"/>
+      <c r="H477" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O477" s="13" t="n"/>
     </row>
     <row r="478" ht="15.75" customHeight="1" s="15">

</xml_diff>

<commit_message>
docs(knowledge): ingest DSE ebook knowledge into Bungalov 4KK
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 02.xlsx
+++ b/docs/knowledge/znalostní báze – mustr 02.xlsx
@@ -2494,10 +2494,22 @@
           <t>Je v zádveří dostatek prostoru pro běžný provoz rodiny?</t>
         </is>
       </c>
-      <c r="E100" s="13" t="n"/>
-      <c r="F100" s="11" t="n"/>
+      <c r="E100" s="13" t="inlineStr">
+        <is>
+          <t>Zádveří je navrženo s místem pro odkládání bot a svršků, věšákovým panelem a úložným prostorem pro sezónní věci.</t>
+        </is>
+      </c>
+      <c r="F100" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G100" s="13" t="n"/>
-      <c r="H100" s="13" t="n"/>
+      <c r="H100" s="13" t="inlineStr">
+        <is>
+          <t>E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O100" s="13" t="n"/>
     </row>
     <row r="101" ht="15.75" customHeight="1" s="15">
@@ -5545,10 +5557,22 @@
           <t>Jak přesně jsou skladby obvodových stěn řešené?</t>
         </is>
       </c>
-      <c r="E256" s="13" t="n"/>
-      <c r="F256" s="11" t="n"/>
+      <c r="E256" s="13" t="inlineStr">
+        <is>
+          <t>Koncepční skladba obvodového pláště je: sádrová omítka, Ekopanel, tepelná izolace Climatizer Plus mezi rámy, difuzní fólie, kontralatě, kotvící latě, odvětrávaná mezera a fasádní prvek.</t>
+        </is>
+      </c>
+      <c r="F256" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G256" s="13" t="n"/>
-      <c r="H256" s="13" t="n"/>
+      <c r="H256" s="13" t="inlineStr">
+        <is>
+          <t>E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O256" s="13" t="n"/>
     </row>
     <row r="257" ht="15.75" customHeight="1" s="15">
@@ -5733,10 +5757,22 @@
           <t>Je konstrukční systém difuzně otevřený, nebo uzavřený?</t>
         </is>
       </c>
-      <c r="E264" s="13" t="n"/>
-      <c r="F264" s="11" t="n"/>
+      <c r="E264" s="13" t="inlineStr">
+        <is>
+          <t>Dům používá difuzně otevřený konstrukční princip, ve kterém jsou vrstvy směrem k exteriéru stále propustnější a vnější plášť je odvětrávaný.</t>
+        </is>
+      </c>
+      <c r="F264" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G264" s="13" t="n"/>
-      <c r="H264" s="13" t="n"/>
+      <c r="H264" s="13" t="inlineStr">
+        <is>
+          <t>E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O264" s="13" t="n"/>
     </row>
     <row r="265" ht="15.75" customHeight="1" s="15">
@@ -6716,10 +6752,22 @@
           <t>Jsou terasové dveře posuvné?</t>
         </is>
       </c>
-      <c r="E308" s="13" t="n"/>
-      <c r="F308" s="11" t="n"/>
+      <c r="E308" s="13" t="inlineStr">
+        <is>
+          <t>Koncept využívá posuvné dveře, které šetří prostor potřebný pro otevírací křídlo.</t>
+        </is>
+      </c>
+      <c r="F308" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G308" s="13" t="n"/>
-      <c r="H308" s="13" t="n"/>
+      <c r="H308" s="13" t="inlineStr">
+        <is>
+          <t>E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O308" s="13" t="n"/>
     </row>
     <row r="309" ht="15.75" customHeight="1" s="15">
@@ -9718,13 +9766,17 @@
       </c>
       <c r="F450" s="11" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="G450" s="13" t="n"/>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G450" s="13" t="inlineStr">
+        <is>
+          <t>Kuchyňský koncept používá ostrůvek orientovaný do hlavního obytného prostoru.</t>
+        </is>
+      </c>
       <c r="H450" s="13" t="inlineStr">
         <is>
-          <t>Studie Bungalov 4KK / 01.11.2022</t>
+          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
         </is>
       </c>
       <c r="O450" s="13" t="n"/>
@@ -14173,10 +14225,22 @@
           <t>Vyžaduje dřevostavba jinou údržbu než zděný dům?</t>
         </is>
       </c>
-      <c r="E672" s="13" t="n"/>
-      <c r="F672" s="11" t="n"/>
+      <c r="E672" s="13" t="inlineStr">
+        <is>
+          <t>Dřevěné fasádní prvky vyžadují pravidelnou povrchovou údržbu; interval závisí na zvoleném ochranném systému.</t>
+        </is>
+      </c>
+      <c r="F672" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G672" s="13" t="n"/>
-      <c r="H672" s="13" t="n"/>
+      <c r="H672" s="13" t="inlineStr">
+        <is>
+          <t>E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O672" s="13" t="n"/>
     </row>
     <row r="673" ht="15.75" customHeight="1" s="15">

</xml_diff>

<commit_message>
docs(knowledge): apply current spatial validations to Bungalov 4KK
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 02.xlsx
+++ b/docs/knowledge/znalostní báze – mustr 02.xlsx
@@ -2496,18 +2496,18 @@
       </c>
       <c r="E100" s="13" t="inlineStr">
         <is>
-          <t>Zádveří je navrženo s místem pro odkládání bot a svršků, věšákovým panelem a úložným prostorem pro sezónní věci.</t>
+          <t>Ano. V zádveří je dostatek prostoru pro běžný provoz rodiny.</t>
         </is>
       </c>
       <c r="F100" s="11" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="G100" s="13" t="n"/>
       <c r="H100" s="13" t="inlineStr">
         <is>
-          <t>E-book Jak se staví Domy s energií / KOMPLET</t>
+          <t>E-book Jak se staví Domy s energií / KOMPLET / Validace autora domu / CURRENT / 2026-09-09</t>
         </is>
       </c>
       <c r="O100" s="13" t="n"/>
@@ -6754,18 +6754,18 @@
       </c>
       <c r="E308" s="13" t="inlineStr">
         <is>
-          <t>Koncept využívá posuvné dveře, které šetří prostor potřebný pro otevírací křídlo.</t>
+          <t>Ne. Terasové dveře nejsou řešeny jako posuvné. Exteriérové posuvné dveře by bylo možné použít pouze ve štítových stěnách, ale toto řešení je vyhodnoceno jako nepraktické a s velmi slabým poměrem ceny a užitku.</t>
         </is>
       </c>
       <c r="F308" s="11" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="G308" s="13" t="n"/>
       <c r="H308" s="13" t="inlineStr">
         <is>
-          <t>E-book Jak se staví Domy s energií / KOMPLET</t>
+          <t>E-book Jak se staví Domy s energií / KOMPLET / Validace autora domu / CURRENT / 2026-09-09</t>
         </is>
       </c>
       <c r="O308" s="13" t="n"/>
@@ -9362,10 +9362,22 @@
           <t>Je z obývacího pokoje přímý vstup na terasu?</t>
         </is>
       </c>
-      <c r="E429" s="13" t="n"/>
-      <c r="F429" s="11" t="n"/>
+      <c r="E429" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Z hlavního obytného prostoru je přímý vstup na terasu a zahradu.</t>
+        </is>
+      </c>
+      <c r="F429" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G429" s="13" t="n"/>
-      <c r="H429" s="13" t="n"/>
+      <c r="H429" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O429" s="13" t="n"/>
     </row>
     <row r="430" ht="15.75" customHeight="1" s="15">
@@ -9761,22 +9773,18 @@
       </c>
       <c r="E450" s="13" t="inlineStr">
         <is>
-          <t>Kuchyň je ve studii řešena s centrálním ostrůvkem.</t>
+          <t>Ano. Kuchyň je navržena s centrálním ostrůvkem orientovaným do hlavního obytného prostoru.</t>
         </is>
       </c>
       <c r="F450" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G450" s="13" t="inlineStr">
-        <is>
-          <t>Kuchyňský koncept používá ostrůvek orientovaný do hlavního obytného prostoru.</t>
-        </is>
-      </c>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="G450" s="13" t="n"/>
       <c r="H450" s="13" t="inlineStr">
         <is>
-          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
+          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET / Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
         </is>
       </c>
       <c r="O450" s="13" t="n"/>
@@ -12495,10 +12503,22 @@
           <t>Jak je terasa propojená s obývacím pokojem?</t>
         </is>
       </c>
-      <c r="E592" s="13" t="n"/>
-      <c r="F592" s="11" t="n"/>
+      <c r="E592" s="13" t="inlineStr">
+        <is>
+          <t>Terasa přímo navazuje na hlavní obytný prostor; velké prosklení a přímý vstup vytvářejí intenzivní propojení interiéru se zahradou.</t>
+        </is>
+      </c>
+      <c r="F592" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G592" s="13" t="n"/>
-      <c r="H592" s="13" t="n"/>
+      <c r="H592" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O592" s="13" t="n"/>
     </row>
     <row r="593" ht="15.75" customHeight="1" s="15">

</xml_diff>

<commit_message>
docs(knowledge): map final DSE ebook facts to Bungalov 4KK
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 02.xlsx
+++ b/docs/knowledge/znalostní báze – mustr 02.xlsx
@@ -7228,10 +7228,22 @@
           <t>Jak rychle dům v zimě vychladne při vypnutí vytápění?</t>
         </is>
       </c>
-      <c r="E330" s="13" t="n"/>
-      <c r="F330" s="11" t="n"/>
+      <c r="E330" s="13" t="inlineStr">
+        <is>
+          <t>Lehká konstrukce má menší tepelnou akumulaci, takže na změnu topného režimu reaguje rychleji než těžká zděná konstrukce.</t>
+        </is>
+      </c>
+      <c r="F330" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G330" s="13" t="n"/>
-      <c r="H330" s="13" t="n"/>
+      <c r="H330" s="13" t="inlineStr">
+        <is>
+          <t>E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O330" s="13" t="n"/>
     </row>
     <row r="331" ht="15.75" customHeight="1" s="15">
@@ -7247,10 +7259,22 @@
           <t>Jak rychle se dá dům znovu vytopit?</t>
         </is>
       </c>
-      <c r="E331" s="13" t="n"/>
-      <c r="F331" s="11" t="n"/>
+      <c r="E331" s="13" t="inlineStr">
+        <is>
+          <t>Díky lehké konstrukci s malou tepelnou akumulací lze dům po změně topného režimu znovu tepelně stabilizovat relativně rychle.</t>
+        </is>
+      </c>
+      <c r="F331" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G331" s="13" t="n"/>
-      <c r="H331" s="13" t="n"/>
+      <c r="H331" s="13" t="inlineStr">
+        <is>
+          <t>E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O331" s="13" t="n"/>
     </row>
     <row r="332" ht="15.75" customHeight="1" s="15">
@@ -10922,10 +10946,22 @@
           <t>Kam se dávají kabáty a boty po příchodu do domu?</t>
         </is>
       </c>
-      <c r="E509" s="13" t="n"/>
-      <c r="F509" s="11" t="n"/>
+      <c r="E509" s="13" t="inlineStr">
+        <is>
+          <t>Zádveří je řešeno s místem pro boty a svrchní oděvy; počítá s botníkem, věšákovým panelem a úložným prostorem pro sezónní věci.</t>
+        </is>
+      </c>
+      <c r="F509" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G509" s="13" t="n"/>
-      <c r="H509" s="13" t="n"/>
+      <c r="H509" s="13" t="inlineStr">
+        <is>
+          <t>E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O509" s="13" t="n"/>
     </row>
     <row r="510" ht="15.75" customHeight="1" s="15">
@@ -11238,10 +11274,22 @@
           <t>Lze v domě vytvořit vestavěné skříně bez omezení průchodů?</t>
         </is>
       </c>
-      <c r="E525" s="13" t="n"/>
-      <c r="F525" s="11" t="n"/>
+      <c r="E525" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Koncept využívá vestavěné a integrované úložné prostory tak, aby nezabíraly zbytečně komunikační plochu.</t>
+        </is>
+      </c>
+      <c r="F525" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G525" s="13" t="n"/>
-      <c r="H525" s="13" t="n"/>
+      <c r="H525" s="13" t="inlineStr">
+        <is>
+          <t>E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O525" s="13" t="n"/>
     </row>
     <row r="526" ht="15.75" customHeight="1" s="15">
@@ -12391,10 +12439,22 @@
           <t>Jak velká okna ovlivňují pocit prostoru uvnitř domu?</t>
         </is>
       </c>
-      <c r="E586" s="13" t="n"/>
-      <c r="F586" s="11" t="n"/>
+      <c r="E586" s="13" t="inlineStr">
+        <is>
+          <t>Velké prosklené a francouzské okenní plochy opticky propojují interiér se zahradou a zvyšují pocit otevřenosti a velikosti prostoru.</t>
+        </is>
+      </c>
+      <c r="F586" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G586" s="13" t="n"/>
-      <c r="H586" s="13" t="n"/>
+      <c r="H586" s="13" t="inlineStr">
+        <is>
+          <t>E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O586" s="13" t="n"/>
     </row>
     <row r="587" ht="15.75" customHeight="1" s="15">

</xml_diff>

<commit_message>
docs(knowledge): ingest Bungalov 4KK fire and structural facts
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 02.xlsx
+++ b/docs/knowledge/znalostní báze – mustr 02.xlsx
@@ -5178,10 +5178,22 @@
           <t>Jak je konstrukce domu staticky navržená?</t>
         </is>
       </c>
-      <c r="E237" s="13" t="n"/>
-      <c r="F237" s="11" t="n"/>
+      <c r="E237" s="13" t="inlineStr">
+        <is>
+          <t>Hlavní nosnou konstrukci tvoří dřevěné rámy a ztužující stěny. Hlavní rámy jsou z profilů 60 × 240 mm C24 v osové vzdálenosti 1 200 mm; konstrukce byla posouzena prostorovým statickým modelem.</t>
+        </is>
+      </c>
+      <c r="F237" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G237" s="13" t="n"/>
-      <c r="H237" s="13" t="n"/>
+      <c r="H237" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O237" s="13" t="n"/>
     </row>
     <row r="238" ht="15.75" customHeight="1" s="15">
@@ -5197,10 +5209,22 @@
           <t>Jakou životnost má nosná konstrukce domu?</t>
         </is>
       </c>
-      <c r="E238" s="13" t="n"/>
-      <c r="F238" s="11" t="n"/>
+      <c r="E238" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek řadí konstrukci do 4. kategorie návrhové životnosti podle ČSN EN 1990, tedy 50 let.</t>
+        </is>
+      </c>
+      <c r="F238" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G238" s="13" t="n"/>
-      <c r="H238" s="13" t="n"/>
+      <c r="H238" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O238" s="13" t="n"/>
     </row>
     <row r="239" ht="15.75" customHeight="1" s="15">
@@ -5216,10 +5240,22 @@
           <t>Jak odolná je konstrukce proti větru a sněhu?</t>
         </is>
       </c>
-      <c r="E239" s="13" t="n"/>
-      <c r="F239" s="11" t="n"/>
+      <c r="E239" s="13" t="inlineStr">
+        <is>
+          <t>Konstrukce je staticky posouzena na sníh i vítr; výpočet uvažuje charakteristické zatížení sněhem 1,00 kN/m² a II. větrnou zónu, II. kategorii terénu. Konstrukce vyhovuje na únosnost, použitelnost i stabilitu.</t>
+        </is>
+      </c>
+      <c r="F239" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G239" s="13" t="n"/>
-      <c r="H239" s="13" t="n"/>
+      <c r="H239" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O239" s="13" t="n"/>
     </row>
     <row r="240" ht="15.75" customHeight="1" s="15">
@@ -5292,10 +5328,22 @@
           <t>Jak se konstrukce přizpůsobuje větrné oblasti?</t>
         </is>
       </c>
-      <c r="E243" s="13" t="n"/>
-      <c r="F243" s="11" t="n"/>
+      <c r="E243" s="13" t="inlineStr">
+        <is>
+          <t>Statický návrh pracuje s konkrétní větrnou oblastí stavby: II. větrná zóna a II. kategorie terénu. Stabilitu proti bočnímu tlaku větru zajišťují ztužující stěny a ocelová křížová táhla.</t>
+        </is>
+      </c>
+      <c r="F243" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G243" s="13" t="n"/>
-      <c r="H243" s="13" t="n"/>
+      <c r="H243" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O243" s="13" t="n"/>
     </row>
     <row r="244" ht="15.75" customHeight="1" s="15">
@@ -5523,8 +5571,16 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="G254" s="13" t="n"/>
-      <c r="H254" s="13" t="n"/>
+      <c r="G254" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek pracuje s prostorovým výpočtovým modelem a posouzením podle příslušných Eurokódů; závěr uvádí, že všechny navržené konstrukce vyhovují na I. i II. mezní stav, včetně stability a lokálního vzpěru.</t>
+        </is>
+      </c>
+      <c r="H254" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O254" s="13" t="n"/>
     </row>
     <row r="255" ht="15.75" customHeight="1" s="15">
@@ -5736,10 +5792,14 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="G263" s="13" t="n"/>
+      <c r="G263" s="13" t="inlineStr">
+        <is>
+          <t>Nosná konstrukce používá zejména konstrukční dřevo C22 a C24; součástí zavětrování jsou také ocelové prvky S235.</t>
+        </is>
+      </c>
       <c r="H263" s="12" t="inlineStr">
         <is>
-          <t>B Souhrnná technická zpráva 11/2023, str. 22</t>
+          <t>B Souhrnná technická zpráva 11/2023, str. 22 / Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
         </is>
       </c>
       <c r="O263" s="13" t="n"/>
@@ -5819,10 +5879,22 @@
           <t>Jak jsou řešené spoje jednotlivých konstrukčních částí?</t>
         </is>
       </c>
-      <c r="E266" s="13" t="n"/>
-      <c r="F266" s="11" t="n"/>
+      <c r="E266" s="13" t="inlineStr">
+        <is>
+          <t>Spoje hlavních rámů jsou zesíleny příložkami X-LVL tloušťky 24 mm a zajištěny dubovými kolíky průměru 20 mm; další stabilitu zajišťují ztužující prvky a ocelová táhla.</t>
+        </is>
+      </c>
+      <c r="F266" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G266" s="13" t="n"/>
-      <c r="H266" s="13" t="n"/>
+      <c r="H266" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O266" s="13" t="n"/>
     </row>
     <row r="267" ht="15.75" customHeight="1" s="15">
@@ -7459,8 +7531,22 @@
           <t>Jakou požární odolnost mají stěny a další konstrukce domu?</t>
         </is>
       </c>
-      <c r="F341" s="11" t="n"/>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>PBŘ uvádí pro obvodovou nosnou stěnu požární odolnost REI 45 z vnitřní strany. Požární stěna technické místnosti a požární stropy mají požadavek EI 15 a požární dveře mezi požárními úseky EW 15 DP3.</t>
+        </is>
+      </c>
+      <c r="F341" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G341" s="13" t="n"/>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>PBŘ SO 2.1 / Ing. Jan Kabot / 08-2023</t>
+        </is>
+      </c>
       <c r="O341" s="13" t="n"/>
     </row>
     <row r="342" ht="15.75" customHeight="1" s="15">
@@ -7514,10 +7600,22 @@
           <t>Jaké materiály v konstrukci zajišťují požární odolnost?</t>
         </is>
       </c>
-      <c r="E344" s="13" t="n"/>
-      <c r="F344" s="11" t="n"/>
+      <c r="E344" s="13" t="inlineStr">
+        <is>
+          <t>Na vnitřní straně obvodového pláště a pod střechou je použit Ekopanel 60. Požární řešení dále využívá certifikované sádrokartonové požární konstrukce podle konkrétního místa a požadované odolnosti.</t>
+        </is>
+      </c>
+      <c r="F344" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G344" s="13" t="n"/>
-      <c r="H344" s="13" t="n"/>
+      <c r="H344" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-09</t>
+        </is>
+      </c>
       <c r="O344" s="13" t="n"/>
     </row>
     <row r="345" ht="15.75" customHeight="1" s="15">

</xml_diff>

<commit_message>
docs(knowledge): ingest Bungalov 4KK PENB envelope facts
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 02.xlsx
+++ b/docs/knowledge/znalostní báze – mustr 02.xlsx
@@ -7141,10 +7141,14 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="G323" s="13" t="n"/>
+      <c r="G323" s="13" t="inlineStr">
+        <is>
+          <t>Obvodový plášť je podle PENB zateplen foukanou izolací Climatizer; energetický výpočet pracuje s tloušťkou 280 mm.</t>
+        </is>
+      </c>
       <c r="H323" s="12" t="inlineStr">
         <is>
-          <t>B Souhrnná technická zpráva 11/2023, str. 22</t>
+          <t>B Souhrnná technická zpráva 11/2023, str. 22 / PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
         </is>
       </c>
       <c r="O323" s="13" t="n"/>
@@ -7172,10 +7176,14 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="G324" s="13" t="n"/>
+      <c r="G324" s="13" t="inlineStr">
+        <is>
+          <t>Střecha je podle PENB zateplena foukanou izolací Climatizer tloušťky 220 mm.</t>
+        </is>
+      </c>
       <c r="H324" s="12" t="inlineStr">
         <is>
-          <t>B Souhrnná technická zpráva 11/2023, str. 22</t>
+          <t>B Souhrnná technická zpráva 11/2023, str. 22 / PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
         </is>
       </c>
       <c r="O324" s="13" t="n"/>
@@ -7203,10 +7211,14 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="G325" s="13" t="n"/>
+      <c r="G325" s="13" t="inlineStr">
+        <is>
+          <t>Podlaha na terénu je podle PENB zateplena foukanou izolací Climatizer tloušťky 220 mm a minerální vatou tloušťky 20 mm.</t>
+        </is>
+      </c>
       <c r="H325" s="12" t="inlineStr">
         <is>
-          <t>B Souhrnná technická zpráva 11/2023, str. 22</t>
+          <t>B Souhrnná technická zpráva 11/2023, str. 22 / PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
         </is>
       </c>
       <c r="O325" s="13" t="n"/>
@@ -7224,10 +7236,22 @@
           <t>Jaké jsou tepelněizolační parametry obvodových stěn?</t>
         </is>
       </c>
-      <c r="E326" s="13" t="n"/>
-      <c r="F326" s="11" t="n"/>
+      <c r="E326" s="13" t="inlineStr">
+        <is>
+          <t>PENB uvádí součinitel prostupu tepla obvodových stěn U = 0,177 a 0,173 W/(m²·K) podle části obvodového pláště.</t>
+        </is>
+      </c>
+      <c r="F326" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G326" s="13" t="n"/>
-      <c r="H326" s="13" t="n"/>
+      <c r="H326" s="13" t="inlineStr">
+        <is>
+          <t>PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
+        </is>
+      </c>
       <c r="O326" s="13" t="n"/>
     </row>
     <row r="327" ht="15.75" customHeight="1" s="15">
@@ -7243,10 +7267,22 @@
           <t>Jaké jsou tepelněizolační parametry střechy?</t>
         </is>
       </c>
-      <c r="E327" s="13" t="n"/>
-      <c r="F327" s="11" t="n"/>
+      <c r="E327" s="13" t="inlineStr">
+        <is>
+          <t>PENB uvádí pro střechu součinitel prostupu tepla U = 0,166 W/(m²·K).</t>
+        </is>
+      </c>
+      <c r="F327" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G327" s="13" t="n"/>
-      <c r="H327" s="13" t="n"/>
+      <c r="H327" s="13" t="inlineStr">
+        <is>
+          <t>PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
+        </is>
+      </c>
       <c r="O327" s="13" t="n"/>
     </row>
     <row r="328" ht="15.75" customHeight="1" s="15">
@@ -7262,10 +7298,22 @@
           <t>Jaké jsou tepelněizolační parametry oken?</t>
         </is>
       </c>
-      <c r="E328" s="13" t="n"/>
-      <c r="F328" s="11" t="n"/>
+      <c r="E328" s="13" t="inlineStr">
+        <is>
+          <t>PENB počítá u oken s izolačními trojskly a součinitelem prostupu tepla Uw = 0,5 W/(m²·K).</t>
+        </is>
+      </c>
+      <c r="F328" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G328" s="13" t="n"/>
-      <c r="H328" s="13" t="n"/>
+      <c r="H328" s="13" t="inlineStr">
+        <is>
+          <t>PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
+        </is>
+      </c>
       <c r="O328" s="13" t="n"/>
     </row>
     <row r="329" ht="15.75" customHeight="1" s="15">
@@ -7476,10 +7524,22 @@
           <t>Čím lze doložit skutečné tepelněizolační vlastnosti tohoto domu?</t>
         </is>
       </c>
-      <c r="E338" s="13" t="n"/>
-      <c r="F338" s="11" t="n"/>
+      <c r="E338" s="13" t="inlineStr">
+        <is>
+          <t>Tepelněizolační vlastnosti jsou doloženy mimo jiné PENB, který obsahuje vypočtené součinitele prostupu tepla jednotlivých částí obálky budovy.</t>
+        </is>
+      </c>
+      <c r="F338" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G338" s="13" t="n"/>
-      <c r="H338" s="13" t="n"/>
+      <c r="H338" s="13" t="inlineStr">
+        <is>
+          <t>PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
+        </is>
+      </c>
       <c r="O338" s="13" t="n"/>
     </row>
     <row r="339" ht="15.75" customHeight="1" s="15">
@@ -7531,7 +7591,7 @@
           <t>Jakou požární odolnost mají stěny a další konstrukce domu?</t>
         </is>
       </c>
-      <c r="E341" t="inlineStr">
+      <c r="E341" s="0" t="inlineStr">
         <is>
           <t>PBŘ uvádí pro obvodovou nosnou stěnu požární odolnost REI 45 z vnitřní strany. Požární stěna technické místnosti a požární stropy mají požadavek EI 15 a požární dveře mezi požárními úseky EW 15 DP3.</t>
         </is>
@@ -7542,7 +7602,7 @@
         </is>
       </c>
       <c r="G341" s="13" t="n"/>
-      <c r="H341" t="inlineStr">
+      <c r="H341" s="0" t="inlineStr">
         <is>
           <t>PBŘ SO 2.1 / Ing. Jan Kabot / 08-2023</t>
         </is>
@@ -13618,10 +13678,14 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="G637" s="13" t="n"/>
+      <c r="G637" s="13" t="inlineStr">
+        <is>
+          <t>PENB hodnotí primární energii z neobnovitelných zdrojů ve třídě A – mimořádně úsporná; hodnota je 26 kWh/(m²·rok).</t>
+        </is>
+      </c>
       <c r="H637" s="12" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
         </is>
       </c>
       <c r="O637" s="13" t="n"/>

</xml_diff>

<commit_message>
docs(knowledge): complete grounded Bungalov 4KK safety answers
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 02.xlsx
+++ b/docs/knowledge/znalostní báze – mustr 02.xlsx
@@ -7572,10 +7572,22 @@
           <t>Jak je dům chráněný proti požáru?</t>
         </is>
       </c>
-      <c r="E340" s="13" t="n"/>
-      <c r="F340" s="11" t="n"/>
+      <c r="E340" s="13" t="inlineStr">
+        <is>
+          <t>Požární bezpečnost je řešena kombinací požárně dělicích konstrukcí a uzávěrů, rozdělením domu do dvou požárních úseků, bezpečnou únikovou cestou, autonomní detekcí požáru a přenosnými hasicími přístroji.</t>
+        </is>
+      </c>
+      <c r="F340" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G340" s="13" t="n"/>
-      <c r="H340" s="13" t="n"/>
+      <c r="H340" s="13" t="inlineStr">
+        <is>
+          <t>PBŘ SO 2.1 / Ing. Jan Kabot / 08-2023</t>
+        </is>
+      </c>
       <c r="O340" s="13" t="n"/>
     </row>
     <row r="341" ht="15.75" customHeight="1" s="15">
@@ -7641,10 +7653,22 @@
           <t>Jak je řešený bezpečný únik z domu při požáru?</t>
         </is>
       </c>
-      <c r="E343" s="13" t="n"/>
-      <c r="F343" s="11" t="n"/>
+      <c r="E343" s="13" t="inlineStr">
+        <is>
+          <t>Evakuace je zajištěna po nechráněné únikové cestě přímo na volné prostranství. PBŘ uvádí minimální šířku únikové cesty 0,9 m a šířku dveří 0,8 m.</t>
+        </is>
+      </c>
+      <c r="F343" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G343" s="13" t="n"/>
-      <c r="H343" s="13" t="n"/>
+      <c r="H343" s="13" t="inlineStr">
+        <is>
+          <t>PBŘ SO 2.1 / Ing. Jan Kabot / 08-2023</t>
+        </is>
+      </c>
       <c r="O343" s="13" t="n"/>
     </row>
     <row r="344" ht="15.75" customHeight="1" s="15">
@@ -7729,10 +7753,22 @@
           <t>Jak dům odolává silnému větru?</t>
         </is>
       </c>
-      <c r="E347" s="13" t="n"/>
-      <c r="F347" s="11" t="n"/>
+      <c r="E347" s="13" t="inlineStr">
+        <is>
+          <t>Dům je staticky posouzen na zatížení větrem pro II. větrnou zónu a II. kategorii terénu. Stabilitu proti bočnímu tlaku větru zajišťují ztužující stěny a křížové zavětrování ocelovými táhly.</t>
+        </is>
+      </c>
+      <c r="F347" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G347" s="13" t="n"/>
-      <c r="H347" s="13" t="n"/>
+      <c r="H347" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O347" s="13" t="n"/>
     </row>
     <row r="348" ht="15.75" customHeight="1" s="15">
@@ -7748,10 +7784,22 @@
           <t>Jak dům odolává vysokému zatížení sněhem?</t>
         </is>
       </c>
-      <c r="E348" s="13" t="n"/>
-      <c r="F348" s="11" t="n"/>
+      <c r="E348" s="13" t="inlineStr">
+        <is>
+          <t>Nosná konstrukce je staticky posouzena také na zatížení sněhem. Výpočet uvažuje charakteristické zatížení sněhem sk = 1,00 kN/m² a výsledné návrhové zatížení střechy 0,80 kN/m².</t>
+        </is>
+      </c>
+      <c r="F348" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G348" s="13" t="n"/>
-      <c r="H348" s="13" t="n"/>
+      <c r="H348" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O348" s="13" t="n"/>
     </row>
     <row r="349" ht="15.75" customHeight="1" s="15">
@@ -7919,10 +7967,22 @@
           <t>Jaké bezpečnostní kontroly se provádějí před předáním domu?</t>
         </is>
       </c>
-      <c r="E357" s="13" t="n"/>
-      <c r="F357" s="11" t="n"/>
+      <c r="E357" s="13" t="inlineStr">
+        <is>
+          <t>Před užíváním musí být doloženo správné provedení požárně bezpečnostních konstrukcí a zařízení podle příslušných certifikátů a dokumentace; správnost elektroinstalace se dokládá revizní zprávou. Požární stěny, stropy a uzávěry musí být provedeny a doloženy v souladu s PBŘ.</t>
+        </is>
+      </c>
+      <c r="F357" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G357" s="13" t="n"/>
-      <c r="H357" s="13" t="n"/>
+      <c r="H357" s="13" t="inlineStr">
+        <is>
+          <t>PBŘ SO 2.1 / Ing. Jan Kabot / 08-2023</t>
+        </is>
+      </c>
       <c r="O357" s="13" t="n"/>
     </row>
     <row r="358" ht="15.75" customHeight="1" s="15">
@@ -7938,8 +7998,22 @@
           <t>Splňuje dům všechny požadované požární a bezpečnostní normy?</t>
         </is>
       </c>
-      <c r="F358" s="11" t="n"/>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>PBŘ uzavírá, že při respektování všech jeho ustanovení novostavba vyhoví požadavkům na požární bezpečnost. Statický posudek současně uvádí, že navržené konstrukce vyhovují požadavkům na únosnost, použitelnost a stabilitu podle příslušných ČSN EN.</t>
+        </is>
+      </c>
+      <c r="F358" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G358" s="13" t="n"/>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>PBŘ SO 2.1 / Ing. Jan Kabot / 08-2023 / Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O358" s="13" t="n"/>
     </row>
     <row r="359" ht="15.75" customHeight="1" s="15">
@@ -7955,10 +8029,22 @@
           <t>Jakými dokumenty lze bezpečnost a odolnost domu doložit?</t>
         </is>
       </c>
-      <c r="E359" s="13" t="n"/>
-      <c r="F359" s="11" t="n"/>
+      <c r="E359" s="13" t="inlineStr">
+        <is>
+          <t>Požární bezpečnost je doložena samostatným Požárně bezpečnostním řešením a mechanická odolnost a stabilita Statickým posudkem. Při dokončení se příslušné instalace a požárně bezpečnostní prvky dokládají také revizemi, certifikáty a dokumentací o správném provedení.</t>
+        </is>
+      </c>
+      <c r="F359" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G359" s="13" t="n"/>
-      <c r="H359" s="13" t="n"/>
+      <c r="H359" s="13" t="inlineStr">
+        <is>
+          <t>PBŘ SO 2.1 / Ing. Jan Kabot / 08-2023 / Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O359" s="13" t="n"/>
     </row>
     <row r="360" ht="15.75" customHeight="1" s="15">

</xml_diff>

<commit_message>
docs(knowledge): extend grounded Bungalov 4KK structural answers
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 02.xlsx
+++ b/docs/knowledge/znalostní báze – mustr 02.xlsx
@@ -5271,10 +5271,22 @@
           <t>Jaké zatížení unese střecha?</t>
         </is>
       </c>
-      <c r="E240" s="13" t="n"/>
-      <c r="F240" s="11" t="n"/>
+      <c r="E240" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek neurčuje jednu univerzální maximální únosnost střechy, ale ověřuje ji pro konkrétní kombinace zatížení. Ve výpočtu je uvažována skladba střechy 0,25 kN/m², FVE 0,20 kN/m² a zatížení sněhem 0,80 kN/m²; navržená konstrukce těmto kombinacím vyhovuje.</t>
+        </is>
+      </c>
+      <c r="F240" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G240" s="13" t="n"/>
-      <c r="H240" s="13" t="n"/>
+      <c r="H240" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O240" s="13" t="n"/>
     </row>
     <row r="241" ht="15.75" customHeight="1" s="15">
@@ -5290,10 +5302,22 @@
           <t>Je konstrukce navržená individuálně pro konkrétní místo stavby?</t>
         </is>
       </c>
-      <c r="E241" s="13" t="n"/>
-      <c r="F241" s="11" t="n"/>
+      <c r="E241" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Statický posudek je zpracován přímo pro tento rodinný dům v Krásném Poli a návrh zohledňuje konkrétní klimatické zatížení lokality, zejména sníh a vítr.</t>
+        </is>
+      </c>
+      <c r="F241" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G241" s="13" t="n"/>
-      <c r="H241" s="13" t="n"/>
+      <c r="H241" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O241" s="13" t="n"/>
     </row>
     <row r="242" ht="15.75" customHeight="1" s="15">
@@ -5309,10 +5333,22 @@
           <t>Jak se statika přizpůsobuje sněhové oblasti, kde bude dům stát?</t>
         </is>
       </c>
-      <c r="E242" s="13" t="n"/>
-      <c r="F242" s="11" t="n"/>
+      <c r="E242" s="13" t="inlineStr">
+        <is>
+          <t>Statický návrh používá klimatické zatížení podle aktuální sněhové mapy ČR pro konkrétní lokalitu. Pro tento dům je uvažováno charakteristické zatížení sněhem sk = 1,00 kN/m² a zatížení střechy sněhem 0,80 kN/m².</t>
+        </is>
+      </c>
+      <c r="F242" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G242" s="13" t="n"/>
-      <c r="H242" s="13" t="n"/>
+      <c r="H242" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O242" s="13" t="n"/>
     </row>
     <row r="243" ht="15.75" customHeight="1" s="15">
@@ -5416,10 +5452,22 @@
           <t>Jsou v domě nosné vnitřní stěny?</t>
         </is>
       </c>
-      <c r="E247" s="13" t="n"/>
-      <c r="F247" s="11" t="n"/>
+      <c r="E247" s="13" t="inlineStr">
+        <is>
+          <t>Některé vnitřní stěny mají statickou ztužující funkci. Statický posudek uvádí vnitřní stěny z OSB desek, které zajišťují stabilitu konstrukce proti bočnímu tlaku větru.</t>
+        </is>
+      </c>
+      <c r="F247" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G247" s="13" t="n"/>
-      <c r="H247" s="13" t="n"/>
+      <c r="H247" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O247" s="13" t="n"/>
     </row>
     <row r="248" ht="15.75" customHeight="1" s="15">
@@ -5435,10 +5483,22 @@
           <t>Které stěny lze později odstranit nebo posunout?</t>
         </is>
       </c>
-      <c r="E248" s="13" t="n"/>
-      <c r="F248" s="11" t="n"/>
+      <c r="E248" s="13" t="inlineStr">
+        <is>
+          <t>Nelze obecně předpokládat, že lze libovolnou stěnu odstranit nebo posunout, protože některé vnitřní stěny mají ztužující statickou funkci. Statický posudek požaduje při jakékoli odchylce od projektu konzultaci se statikem.</t>
+        </is>
+      </c>
+      <c r="F248" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G248" s="13" t="n"/>
-      <c r="H248" s="13" t="n"/>
+      <c r="H248" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O248" s="13" t="n"/>
     </row>
     <row r="249" ht="15.75" customHeight="1" s="15">
@@ -5454,10 +5514,22 @@
           <t>Lze do nosných stěn později dělat nové otvory?</t>
         </is>
       </c>
-      <c r="E249" s="13" t="n"/>
-      <c r="F249" s="11" t="n"/>
+      <c r="E249" s="13" t="inlineStr">
+        <is>
+          <t>Nové otvory v konstrukčně významných stěnách nelze provádět bez statického posouzení. Statický posudek výslovně požaduje konzultaci statika při jakémkoli odchýlení od projektu.</t>
+        </is>
+      </c>
+      <c r="F249" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G249" s="13" t="n"/>
-      <c r="H249" s="13" t="n"/>
+      <c r="H249" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O249" s="13" t="n"/>
     </row>
     <row r="250" ht="15.75" customHeight="1" s="15">
@@ -5948,10 +6020,22 @@
           <t>Jak je řešený detail kolem oken a dveří?</t>
         </is>
       </c>
-      <c r="E269" s="13" t="n"/>
-      <c r="F269" s="11" t="n"/>
+      <c r="E269" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek uvádí u okenních otvorů výztuhy z profilů 40 × 240 mm C22. Konkrétní konstrukční detail kolem dveřních otvorů tento statický posudek samostatně nepopisuje.</t>
+        </is>
+      </c>
+      <c r="F269" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G269" s="13" t="n"/>
-      <c r="H269" s="13" t="n"/>
+      <c r="H269" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O269" s="13" t="n"/>
     </row>
     <row r="270" ht="15.75" customHeight="1" s="15">
@@ -6005,10 +6089,22 @@
           <t>Jak je možné ověřit správnost provedení konstrukčních skladeb?</t>
         </is>
       </c>
-      <c r="E272" s="13" t="n"/>
-      <c r="F272" s="11" t="n"/>
+      <c r="E272" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek je zpracován ve stupni DSP a výslovně uvádí, že pro realizaci se předpokládá navazující stupeň projektové dokumentace. Při jakékoli odchylce provádění od projektu má být přizván statik ke konzultaci.</t>
+        </is>
+      </c>
+      <c r="F272" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G272" s="13" t="n"/>
-      <c r="H272" s="13" t="n"/>
+      <c r="H272" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O272" s="13" t="n"/>
     </row>
     <row r="273" ht="15.75" customHeight="1" s="15">
@@ -7998,7 +8094,7 @@
           <t>Splňuje dům všechny požadované požární a bezpečnostní normy?</t>
         </is>
       </c>
-      <c r="E358" t="inlineStr">
+      <c r="E358" s="0" t="inlineStr">
         <is>
           <t>PBŘ uzavírá, že při respektování všech jeho ustanovení novostavba vyhoví požadavkům na požární bezpečnost. Statický posudek současně uvádí, že navržené konstrukce vyhovují požadavkům na únosnost, použitelnost a stabilitu podle příslušných ČSN EN.</t>
         </is>
@@ -8009,7 +8105,7 @@
         </is>
       </c>
       <c r="G358" s="13" t="n"/>
-      <c r="H358" t="inlineStr">
+      <c r="H358" s="0" t="inlineStr">
         <is>
           <t>PBŘ SO 2.1 / Ing. Jan Kabot / 08-2023 / Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
         </is>

</xml_diff>

<commit_message>
docs(knowledge): extend grounded Bungalov 4KK thermal comfort answers
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 02.xlsx
+++ b/docs/knowledge/znalostní báze – mustr 02.xlsx
@@ -7151,10 +7151,22 @@
           <t>Jak dobře je dům zateplený?</t>
         </is>
       </c>
-      <c r="E319" s="13" t="n"/>
-      <c r="F319" s="11" t="n"/>
+      <c r="E319" s="13" t="inlineStr">
+        <is>
+          <t>PENB hodnotí tepelnou obálku domu průměrným součinitelem prostupu tepla 0,21 W/(m²·K). Měrná potřeba tepla na vytápění je 52 kWh/(m²·rok) a požadavky na novou budovu jsou podle průkazu splněny.</t>
+        </is>
+      </c>
+      <c r="F319" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G319" s="13" t="n"/>
-      <c r="H319" s="13" t="n"/>
+      <c r="H319" s="13" t="inlineStr">
+        <is>
+          <t>PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
+        </is>
+      </c>
       <c r="O319" s="13" t="n"/>
     </row>
     <row r="320" ht="15.75" customHeight="1" s="15">
@@ -7189,10 +7201,22 @@
           <t>Jak dům udržuje teplo v zimě?</t>
         </is>
       </c>
-      <c r="E321" s="13" t="n"/>
-      <c r="F321" s="11" t="n"/>
+      <c r="E321" s="13" t="inlineStr">
+        <is>
+          <t>PENB dokládá tepelně kvalitní obálku: obvodové stěny mají U = 0,177 až 0,173 W/(m²·K), střecha U = 0,166 W/(m²·K) a okna s trojskly Uw = 0,5 W/(m²·K). Tyto parametry omezují tepelné ztráty obálkou domu.</t>
+        </is>
+      </c>
+      <c r="F321" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G321" s="13" t="n"/>
-      <c r="H321" s="13" t="n"/>
+      <c r="H321" s="13" t="inlineStr">
+        <is>
+          <t>PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
+        </is>
+      </c>
       <c r="O321" s="13" t="n"/>
     </row>
     <row r="322" ht="15.75" customHeight="1" s="15">
@@ -7425,10 +7449,22 @@
           <t>Jakou roli při letním komfortu hraje venkovní stínění?</t>
         </is>
       </c>
-      <c r="E329" s="13" t="n"/>
-      <c r="F329" s="11" t="n"/>
+      <c r="E329" s="13" t="inlineStr">
+        <is>
+          <t>Studie u štítových oken a oken směrem k terase počítá s přípravou pro elektricky ovládané venkovní žaluzie. Konkrétní snížení letní teploty nebo přehřívání však dostupná studie nevyčísluje.</t>
+        </is>
+      </c>
+      <c r="F329" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G329" s="13" t="n"/>
-      <c r="H329" s="13" t="n"/>
+      <c r="H329" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O329" s="13" t="n"/>
     </row>
     <row r="330" ht="15.75" customHeight="1" s="15">
@@ -7563,10 +7599,22 @@
           <t>Jak orientace domu ovlivňuje jeho tepelný komfort?</t>
         </is>
       </c>
-      <c r="E335" s="13" t="n"/>
-      <c r="F335" s="11" t="n"/>
+      <c r="E335" s="13" t="inlineStr">
+        <is>
+          <t>Studie orientuje hlavní zahradní stranu domu s velkým prosklením a terasou na jihovýchod. Konkrétní kvantitativní dopad této orientace na zimní nebo letní tepelný komfort však dostupné podklady samostatně nevyhodnocují.</t>
+        </is>
+      </c>
+      <c r="F335" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G335" s="13" t="n"/>
-      <c r="H335" s="13" t="n"/>
+      <c r="H335" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O335" s="13" t="n"/>
     </row>
     <row r="336" ht="15.75" customHeight="1" s="15">
@@ -7582,10 +7630,22 @@
           <t>Jak velký vliv mají velká okna na teplotu uvnitř domu?</t>
         </is>
       </c>
-      <c r="E336" s="13" t="n"/>
-      <c r="F336" s="11" t="n"/>
+      <c r="E336" s="13" t="inlineStr">
+        <is>
+          <t>PENB uvádí podíl průsvitných konstrukcí 18,6 % plochy svislých konstrukcí a u oken počítá s trojskly Uw = 0,5 W/(m²·K). Konkrétní vliv velkých oken na letní vnitřní teplotu ale PENB samostatně nevyčísluje.</t>
+        </is>
+      </c>
+      <c r="F336" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G336" s="13" t="n"/>
-      <c r="H336" s="13" t="n"/>
+      <c r="H336" s="13" t="inlineStr">
+        <is>
+          <t>PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
+        </is>
+      </c>
       <c r="O336" s="13" t="n"/>
     </row>
     <row r="337" ht="15.75" customHeight="1" s="15">
@@ -7601,10 +7661,22 @@
           <t>Je tepelný komfort dřevostavby jiný než u zděného domu?</t>
         </is>
       </c>
-      <c r="E337" s="13" t="n"/>
-      <c r="F337" s="11" t="n"/>
+      <c r="E337" s="13" t="inlineStr">
+        <is>
+          <t>Ano, zejména tepelnou akumulací. E-book popisuje tuto dřevostavbu jako lehkou konstrukci s menší tepelnou akumulací než těžká zděná stavba, takže rychleji reaguje na změny vytápění i vnitřních tepelných podmínek.</t>
+        </is>
+      </c>
+      <c r="F337" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G337" s="13" t="n"/>
-      <c r="H337" s="13" t="n"/>
+      <c r="H337" s="13" t="inlineStr">
+        <is>
+          <t>E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O337" s="13" t="n"/>
     </row>
     <row r="338" ht="15.75" customHeight="1" s="15">

</xml_diff>

<commit_message>
docs(knowledge): extend grounded Bungalov 4KK installation answers
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 02.xlsx
+++ b/docs/knowledge/znalostní báze – mustr 02.xlsx
@@ -8394,10 +8394,22 @@
           <t>Je elektroinstalace připravená pro fotovoltaiku?</t>
         </is>
       </c>
-      <c r="E367" s="13" t="n"/>
-      <c r="F367" s="11" t="n"/>
+      <c r="E367" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Referenční realizace fotovoltaiku skutečně používá; fotovoltaická elektrárna je součástí elektroinstalace domu.</t>
+        </is>
+      </c>
+      <c r="F367" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G367" s="13" t="n"/>
-      <c r="H367" s="13" t="n"/>
+      <c r="H367" s="13" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
       <c r="O367" s="13" t="n"/>
     </row>
     <row r="368" ht="15.75" customHeight="1" s="15">
@@ -8536,10 +8548,22 @@
           <t>Jak dlouho se čeká na teplou vodu u vzdálenějších odběrných míst?</t>
         </is>
       </c>
-      <c r="E372" s="13" t="n"/>
-      <c r="F372" s="11" t="n"/>
+      <c r="E372" s="13" t="inlineStr">
+        <is>
+          <t>Rozvod teplé vody je vybaven cirkulací, která omezuje čekání na teplou vodu u vzdálenějších odběrných míst. Konkrétní dobu v sekundách dostupné podklady neuvádějí.</t>
+        </is>
+      </c>
+      <c r="F372" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G372" s="13" t="n"/>
-      <c r="H372" s="13" t="n"/>
+      <c r="H372" s="13" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
       <c r="O372" s="13" t="n"/>
     </row>
     <row r="373" ht="15.75" customHeight="1" s="15">
@@ -8681,8 +8705,22 @@
           <t>Které technické instalace vyžadují pravidelné revize?</t>
         </is>
       </c>
-      <c r="F379" s="11" t="n"/>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>Elektroinstalace patří mezi instalace, jejichž bezpečný stav se dokládá revizí. Konkrétní servisní a revizní intervaly jednotlivých technologií je nutné řídit dokumentací jejich výrobců a příslušnými předpisy.</t>
+        </is>
+      </c>
+      <c r="F379" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G379" s="13" t="n"/>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023</t>
+        </is>
+      </c>
       <c r="O379" s="13" t="n"/>
     </row>
     <row r="380" ht="15.75" customHeight="1" s="15">
@@ -8698,10 +8736,22 @@
           <t>Dostanu při předání dokumentaci skutečného provedení všech rozvodů?</t>
         </is>
       </c>
-      <c r="E380" s="13" t="n"/>
-      <c r="F380" s="11" t="n"/>
+      <c r="E380" s="13" t="inlineStr">
+        <is>
+          <t>Projektová dokumentace tvoří podklad pro provedení instalací; skutečné provedení a příslušné revizní či provozní doklady se dokládají v rámci dokončení a předání stavby. Dostupné podklady ale samostatně nepotvrzují přesný rozsah předávané dokumentace všech rozvodů.</t>
+        </is>
+      </c>
+      <c r="F380" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G380" s="13" t="n"/>
-      <c r="H380" s="13" t="n"/>
+      <c r="H380" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023</t>
+        </is>
+      </c>
       <c r="O380" s="13" t="n"/>
     </row>
     <row r="381" ht="15.75" customHeight="1" s="15">

</xml_diff>

<commit_message>
docs(knowledge): reconcile current Bungalov 4KK technologies
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 02.xlsx
+++ b/docs/knowledge/znalostní báze – mustr 02.xlsx
@@ -8705,7 +8705,7 @@
           <t>Které technické instalace vyžadují pravidelné revize?</t>
         </is>
       </c>
-      <c r="E379" t="inlineStr">
+      <c r="E379" s="0" t="inlineStr">
         <is>
           <t>Elektroinstalace patří mezi instalace, jejichž bezpečný stav se dokládá revizí. Konkrétní servisní a revizní intervaly jednotlivých technologií je nutné řídit dokumentací jejich výrobců a příslušnými předpisy.</t>
         </is>
@@ -8716,7 +8716,7 @@
         </is>
       </c>
       <c r="G379" s="13" t="n"/>
-      <c r="H379" t="inlineStr">
+      <c r="H379" s="0" t="inlineStr">
         <is>
           <t>B Souhrnná technická zpráva 11/2023</t>
         </is>
@@ -8791,13 +8791,17 @@
       </c>
       <c r="F382" s="11" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="G382" s="13" t="n"/>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G382" s="13" t="inlineStr">
+        <is>
+          <t>Krbové těleso bylo z aktuální klientské konfigurace vypuštěno. Dostupné CURRENT podklady zatím neumožňují bezpečně označit jediný hlavní systém vytápění.</t>
+        </is>
+      </c>
       <c r="H382" s="12" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
         </is>
       </c>
       <c r="O382" s="13" t="n"/>
@@ -8827,12 +8831,12 @@
       </c>
       <c r="G383" s="13" t="inlineStr">
         <is>
-          <t>Aktuální technologické řešení používá systém Zehnder ve výkonnější konfiguraci než původně uvažovaná varianta.</t>
+          <t>Krbové těleso bylo z aktuální klientské konfigurace vypuštěno. Zehnder je CURRENT řešení řízeného větrání/rekuperace; samotná informace o Zehnderu nedokládá hlavní systém vytápění. Hlavní systém vytápění je nutné ještě jednoznačně potvrdit.</t>
         </is>
       </c>
       <c r="H383" s="12" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / Validace autora domu / CURRENT / 2026-09-09</t>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / Validace autora domu / CURRENT / 2026-09-09 / Klientské změny č. 2 / Bungalov 4KK / 20.10.2023 / Validace autora domu / CURRENT / 2026-09-09</t>
         </is>
       </c>
       <c r="O383" s="13" t="n"/>
@@ -8852,22 +8856,18 @@
       </c>
       <c r="E384" s="12" t="inlineStr">
         <is>
-          <t>Pod dřevěnou třívrstvou podlahou jsou topné fólie (pod dlažbou rošty) jako rezervní zdroj tepla pro mrazivé dny (cca 25 dní v roce).</t>
+          <t>Ano. V aktuální konfiguraci jsou použity elektrické topné fólie. Pod dřevěnou podlahou slouží jako doplňkový / rezervní zdroj tepla pro chladné období.</t>
         </is>
       </c>
       <c r="F384" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G384" s="13" t="inlineStr">
-        <is>
-          <t>Ano. Aktuální klientská konfigurace používá elektrické topné fólie.</t>
-        </is>
-      </c>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G384" s="13" t="n"/>
       <c r="H384" s="12" t="inlineStr">
         <is>
-          <t>B Souhrnná technická zpráva 11/2023, str. 24 / Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
+          <t>B Souhrnná technická zpráva 11/2023, str. 24 / Klientské změny č. 2 / Bungalov 4KK / 20.10.2023 / Klientské změny č. 2 / Bungalov 4KK / 20.10.2023 / B Souhrnná technická zpráva 11/2023</t>
         </is>
       </c>
       <c r="O384" s="13" t="n"/>
@@ -8949,22 +8949,22 @@
       </c>
       <c r="E387" s="12" t="inlineStr">
         <is>
-          <t>Ano. Dům využívá rekuperaci tepla ze vzduchu a šedé vody.</t>
+          <t>Ano. Dům používá řízené větrání s rekuperací Zehnder ve výkonnější konfiguraci.</t>
         </is>
       </c>
       <c r="F387" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="G387" s="13" t="inlineStr">
         <is>
-          <t>Ano. Aktuální řešení používá systém řízeného větrání s rekuperací Zehnder ve výkonnější konfiguraci.</t>
+          <t>Ano. Aktuální řešení používá systém řízeného větrání s rekuperací Zehnder ve výkonnější konfiguraci. / HISTORICAL_UNVERIFIED: Ano. Dům využívá rekuperaci tepla ze vzduchu a šedé vody.</t>
         </is>
       </c>
       <c r="H387" s="12" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / Validace autora domu / CURRENT / 2026-09-09</t>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / Validace autora domu / CURRENT / 2026-09-09 / Validace autora domu / CURRENT / 2026-09-09</t>
         </is>
       </c>
       <c r="O387" s="13" t="n"/>
@@ -9082,10 +9082,22 @@
           <t>Jak je zajištěný dostatek čerstvého vzduchu v ložnicích?</t>
         </is>
       </c>
-      <c r="E392" s="13" t="n"/>
-      <c r="F392" s="11" t="n"/>
+      <c r="E392" s="13" t="inlineStr">
+        <is>
+          <t>Dostatek čerstvého vzduchu zajišťuje nucené řízené větrání s rekuperací, které přivádí čerstvý vzduch do obytných místností. Okna lze současně používat pro příležitostné přirozené větrání.</t>
+        </is>
+      </c>
+      <c r="F392" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G392" s="13" t="n"/>
-      <c r="H392" s="13" t="n"/>
+      <c r="H392" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023</t>
+        </is>
+      </c>
       <c r="O392" s="13" t="n"/>
     </row>
     <row r="393" ht="15.75" customHeight="1" s="15">

</xml_diff>

<commit_message>
docs(knowledge): extend grounded Bungalov 4KK energy answers
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 02.xlsx
+++ b/docs/knowledge/znalostní báze – mustr 02.xlsx
@@ -8801,7 +8801,7 @@
       </c>
       <c r="H382" s="12" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / Klientské změny č. 2 / 20.10.2023</t>
         </is>
       </c>
       <c r="O382" s="13" t="n"/>
@@ -8836,7 +8836,7 @@
       </c>
       <c r="H383" s="12" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / Validace autora domu / CURRENT / 2026-09-09 / Klientské změny č. 2 / Bungalov 4KK / 20.10.2023 / Validace autora domu / CURRENT / 2026-09-09</t>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / Validace autora domu / CURRENT / 2026-09-09 / Klientské změny č. 2 / 20.10.2023</t>
         </is>
       </c>
       <c r="O383" s="13" t="n"/>
@@ -8867,7 +8867,7 @@
       <c r="G384" s="13" t="n"/>
       <c r="H384" s="12" t="inlineStr">
         <is>
-          <t>B Souhrnná technická zpráva 11/2023, str. 24 / Klientské změny č. 2 / Bungalov 4KK / 20.10.2023 / Klientské změny č. 2 / Bungalov 4KK / 20.10.2023 / B Souhrnná technická zpráva 11/2023</t>
+          <t>B Souhrnná technická zpráva 11/2023, str. 24 / Klientské změny č. 2 / Bungalov 4KK / 20.10.2023 / B Souhrnná technická zpráva 11/2023</t>
         </is>
       </c>
       <c r="O384" s="13" t="n"/>
@@ -8964,7 +8964,7 @@
       </c>
       <c r="H387" s="12" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / Validace autora domu / CURRENT / 2026-09-09 / Validace autora domu / CURRENT / 2026-09-09</t>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / Validace autora domu / CURRENT / 2026-09-09</t>
         </is>
       </c>
       <c r="O387" s="13" t="n"/>

</xml_diff>

<commit_message>
docs(knowledge): extend grounded Bungalov 4KK acoustic answers
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 02.xlsx
+++ b/docs/knowledge/znalostní báze – mustr 02.xlsx
@@ -13682,10 +13682,22 @@
           <t>Je rekuperace při běžném provozu slyšet?</t>
         </is>
       </c>
-      <c r="E621" s="13" t="n"/>
-      <c r="F621" s="11" t="n"/>
+      <c r="E621" s="13" t="inlineStr">
+        <is>
+          <t>Řízené větrání je navrženo jako technické zařízení domu. Dostupné podklady ale neuvádějí konkrétní naměřenou hladinu hluku současné jednotky Zehnder, takže hlučnost v dB nelze z těchto dokumentů spolehlivě určit.</t>
+        </is>
+      </c>
+      <c r="F621" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G621" s="13" t="n"/>
-      <c r="H621" s="13" t="n"/>
+      <c r="H621" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-09</t>
+        </is>
+      </c>
       <c r="O621" s="13" t="n"/>
     </row>
     <row r="622" ht="15.75" customHeight="1" s="15">
@@ -13701,10 +13713,22 @@
           <t>Je v obytných místnostech slyšet tepelné čerpadlo?</t>
         </is>
       </c>
-      <c r="E622" s="13" t="n"/>
-      <c r="F622" s="11" t="n"/>
+      <c r="E622" s="13" t="inlineStr">
+        <is>
+          <t>Dostupné podklady neobsahují konkrétní měření hluku tepelných čerpadel v obytných místnostech, takže nelze bezpečně uvést konkrétní hladinu hluku ani tvrdit, že jsou za všech provozních stavů neslyšná.</t>
+        </is>
+      </c>
+      <c r="F622" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G622" s="13" t="n"/>
-      <c r="H622" s="13" t="n"/>
+      <c r="H622" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023</t>
+        </is>
+      </c>
       <c r="O622" s="13" t="n"/>
     </row>
     <row r="623" ht="15.75" customHeight="1" s="15">
@@ -13777,10 +13801,22 @@
           <t>Přenášejí se konstrukcí kroky nebo jiné vibrace?</t>
         </is>
       </c>
-      <c r="E626" s="13" t="n"/>
-      <c r="F626" s="11" t="n"/>
+      <c r="E626" s="13" t="inlineStr">
+        <is>
+          <t>Konstrukce je lehká rámová dřevostavba. Dostupné technické podklady ale neobsahují samostatné měření přenosu kročejového hluku nebo vibrací pro dokončený dům.</t>
+        </is>
+      </c>
+      <c r="F626" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G626" s="13" t="n"/>
-      <c r="H626" s="13" t="n"/>
+      <c r="H626" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023</t>
+        </is>
+      </c>
       <c r="O626" s="13" t="n"/>
     </row>
     <row r="627" ht="15.75" customHeight="1" s="15">
@@ -13872,10 +13908,22 @@
           <t>Jakými parametry lze akustické vlastnosti konstrukcí doložit?</t>
         </is>
       </c>
-      <c r="E631" s="13" t="n"/>
-      <c r="F631" s="11" t="n"/>
+      <c r="E631" s="13" t="inlineStr">
+        <is>
+          <t>Akustické vlastnosti konstrukcí lze doložit projektovými akustickými parametry jednotlivých skladeb a případně měřením dokončené stavby. Technická dokumentace tohoto domu obsahuje akustické parametry vybraných konstrukcí.</t>
+        </is>
+      </c>
+      <c r="F631" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G631" s="13" t="n"/>
-      <c r="H631" s="13" t="n"/>
+      <c r="H631" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023</t>
+        </is>
+      </c>
       <c r="O631" s="13" t="n"/>
     </row>
     <row r="632" ht="15.75" customHeight="1" s="15">

</xml_diff>

<commit_message>
docs(knowledge): extend Bungalov 4KK roof window maintenance answers
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 02.xlsx
+++ b/docs/knowledge/znalostní báze – mustr 02.xlsx
@@ -6194,10 +6194,22 @@
           <t>Jaká střešní krytina je na domě použitá?</t>
         </is>
       </c>
-      <c r="E277" s="13" t="n"/>
-      <c r="F277" s="11" t="n"/>
+      <c r="E277" s="13" t="inlineStr">
+        <is>
+          <t>Střešní krytina je BRATEX CLICK.</t>
+        </is>
+      </c>
+      <c r="F277" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G277" s="13" t="n"/>
-      <c r="H277" s="13" t="n"/>
+      <c r="H277" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O277" s="13" t="n"/>
     </row>
     <row r="278" ht="15.75" customHeight="1" s="15">
@@ -6389,10 +6401,22 @@
           <t>Je možné změnit barvu střechy?</t>
         </is>
       </c>
-      <c r="E286" s="13" t="n"/>
-      <c r="F286" s="11" t="n"/>
+      <c r="E286" s="13" t="inlineStr">
+        <is>
+          <t>Střecha je v antracitovém odstínu.</t>
+        </is>
+      </c>
+      <c r="F286" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G286" s="13" t="n"/>
-      <c r="H286" s="13" t="n"/>
+      <c r="H286" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O286" s="13" t="n"/>
     </row>
     <row r="287" ht="15.75" customHeight="1" s="15">

</xml_diff>

<commit_message>
docs(knowledge): complete grounded Bungalov 4KK envelope answers
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 02.xlsx
+++ b/docs/knowledge/znalostní báze – mustr 02.xlsx
@@ -6403,7 +6403,7 @@
       </c>
       <c r="E286" s="13" t="inlineStr">
         <is>
-          <t>Střecha je v antracitovém odstínu.</t>
+          <t>Aktuální referenční provedení má střechu v antracitovém odstínu. Dostupné podklady ale samostatně nepotvrzují, zda lze u tohoto domu v rámci objednávky zvolit jinou barvu střechy.</t>
         </is>
       </c>
       <c r="F286" s="11" t="inlineStr">
@@ -6451,10 +6451,22 @@
           <t>Jak je střecha zateplená?</t>
         </is>
       </c>
-      <c r="E288" s="13" t="n"/>
-      <c r="F288" s="11" t="n"/>
+      <c r="E288" s="13" t="inlineStr">
+        <is>
+          <t>Střešní konstrukce je zateplena foukanou celulózovou izolací Climatizer; PENB pracuje s tloušťkou izolace 220 mm.</t>
+        </is>
+      </c>
+      <c r="F288" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G288" s="13" t="n"/>
-      <c r="H288" s="13" t="n"/>
+      <c r="H288" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023 / PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
+        </is>
+      </c>
       <c r="O288" s="13" t="n"/>
     </row>
     <row r="289" ht="15.75" customHeight="1" s="15">
@@ -6470,10 +6482,22 @@
           <t>Jak je střecha odvětrávaná?</t>
         </is>
       </c>
-      <c r="E289" s="13" t="n"/>
-      <c r="F289" s="11" t="n"/>
+      <c r="E289" s="13" t="inlineStr">
+        <is>
+          <t>Střešní plášť je řešen jako difuzně otevřená skladba s difuzní fólií a odvětrávanou vrstvou pod vnějším pláštěm.</t>
+        </is>
+      </c>
+      <c r="F289" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G289" s="13" t="n"/>
-      <c r="H289" s="13" t="n"/>
+      <c r="H289" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023</t>
+        </is>
+      </c>
       <c r="O289" s="13" t="n"/>
     </row>
     <row r="290" ht="15.75" customHeight="1" s="15">
@@ -6551,10 +6575,22 @@
           <t>Jak střecha odolává silnému větru a sněhu?</t>
         </is>
       </c>
-      <c r="E292" s="13" t="n"/>
-      <c r="F292" s="11" t="n"/>
+      <c r="E292" s="13" t="inlineStr">
+        <is>
+          <t>Nosná konstrukce střechy je staticky posouzena na zatížení sněhem i větrem. Výpočet uvažuje charakteristické zatížení sněhem sk = 1,00 kN/m² a II. větrnou zónu, II. kategorii terénu.</t>
+        </is>
+      </c>
+      <c r="F292" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G292" s="13" t="n"/>
-      <c r="H292" s="13" t="n"/>
+      <c r="H292" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O292" s="13" t="n"/>
     </row>
     <row r="293" ht="15.75" customHeight="1" s="15">
@@ -6849,10 +6885,22 @@
           <t>Jsou součástí domu venkovní žaluzie nebo rolety?</t>
         </is>
       </c>
-      <c r="E303" s="13" t="n"/>
-      <c r="F303" s="11" t="n"/>
+      <c r="E303" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Aktuální provedení používá venkovní roletové žaluzie v antracitovém odstínu.</t>
+        </is>
+      </c>
+      <c r="F303" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G303" s="13" t="n"/>
-      <c r="H303" s="13" t="n"/>
+      <c r="H303" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O303" s="13" t="n"/>
     </row>
     <row r="304" ht="15.75" customHeight="1" s="15">
@@ -6868,10 +6916,22 @@
           <t>Jaké stínění je u tohoto domu navržené?</t>
         </is>
       </c>
-      <c r="E304" s="13" t="n"/>
-      <c r="F304" s="11" t="n"/>
+      <c r="E304" s="13" t="inlineStr">
+        <is>
+          <t>Venkovní stínění je řešeno roletovými žaluziemi.</t>
+        </is>
+      </c>
+      <c r="F304" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G304" s="13" t="n"/>
-      <c r="H304" s="13" t="n"/>
+      <c r="H304" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O304" s="13" t="n"/>
     </row>
     <row r="305" ht="15.75" customHeight="1" s="15">
@@ -6887,10 +6947,22 @@
           <t>Jakou barvu má venkovní stínění?</t>
         </is>
       </c>
-      <c r="E305" s="13" t="n"/>
-      <c r="F305" s="11" t="n"/>
+      <c r="E305" s="13" t="inlineStr">
+        <is>
+          <t>Venkovní roletové žaluzie jsou v antracitovém odstínu.</t>
+        </is>
+      </c>
+      <c r="F305" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G305" s="13" t="n"/>
-      <c r="H305" s="13" t="n"/>
+      <c r="H305" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O305" s="13" t="n"/>
     </row>
     <row r="306" ht="15.75" customHeight="1" s="15">
@@ -6906,10 +6978,22 @@
           <t>Jsou venkovní žaluzie nebo rolety elektricky ovládané?</t>
         </is>
       </c>
-      <c r="E306" s="13" t="n"/>
-      <c r="F306" s="11" t="n"/>
+      <c r="E306" s="13" t="inlineStr">
+        <is>
+          <t>Studie počítá u venkovního stínění s přípravou pro elektrické ovládání. Dostupná CURRENT validace potvrzuje roletové žaluzie, ale samostatně nepotvrzuje jejich výsledný způsob ovládání v dokončeném domě.</t>
+        </is>
+      </c>
+      <c r="F306" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G306" s="13" t="n"/>
-      <c r="H306" s="13" t="n"/>
+      <c r="H306" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022 / Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O306" s="13" t="n"/>
     </row>
     <row r="307" ht="15.75" customHeight="1" s="15">
@@ -7082,10 +7166,22 @@
           <t>Jak okna chrání interiér před přehříváním v létě?</t>
         </is>
       </c>
-      <c r="E314" s="13" t="n"/>
-      <c r="F314" s="11" t="n"/>
+      <c r="E314" s="13" t="inlineStr">
+        <is>
+          <t>Okna mají izolační trojskla a dům používá venkovní roletové žaluzie, které umožňují omezit přímé sluneční záření před zasklením. Konkrétní snížení letní vnitřní teploty dostupné podklady nevyčíslují.</t>
+        </is>
+      </c>
+      <c r="F314" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G314" s="13" t="n"/>
-      <c r="H314" s="13" t="n"/>
+      <c r="H314" s="13" t="inlineStr">
+        <is>
+          <t>PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023 / Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O314" s="13" t="n"/>
     </row>
     <row r="315" ht="15.75" customHeight="1" s="15">
@@ -14646,10 +14742,22 @@
           <t>Jak často je potřeba servisovat technologie domu?</t>
         </is>
       </c>
-      <c r="E661" s="13" t="n"/>
-      <c r="F661" s="11" t="n"/>
+      <c r="E661" s="13" t="inlineStr">
+        <is>
+          <t>Servisní intervaly technologií nejsou pro všechny prvky domu v dostupných podkladech jednotně stanoveny. Řídí se dokumentací a servisními požadavky konkrétních výrobců jednotlivých zařízení.</t>
+        </is>
+      </c>
+      <c r="F661" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G661" s="13" t="n"/>
-      <c r="H661" s="13" t="n"/>
+      <c r="H661" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023</t>
+        </is>
+      </c>
       <c r="O661" s="13" t="n"/>
     </row>
     <row r="662" ht="15.75" customHeight="1" s="15">

</xml_diff>

<commit_message>
docs(knowledge): globally harvest grounded Bungalov 4KK knowledge
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 02.xlsx
+++ b/docs/knowledge/znalostní báze – mustr 02.xlsx
@@ -576,10 +576,22 @@
           <t>Je tento dům vhodný pro rodinu s dětmi?</t>
         </is>
       </c>
-      <c r="E5" s="13" t="n"/>
-      <c r="F5" s="11" t="n"/>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Dům má dispozici 4+kk a tři samostatné pokoje vedle společného obytného prostoru; dispozičně tedy umožňuje běžné rodinné bydlení s dětmi.</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G5" s="13" t="n"/>
-      <c r="H5" s="13" t="n"/>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 14–15</t>
+        </is>
+      </c>
       <c r="O5" s="13" t="n"/>
     </row>
     <row r="6" ht="15.75" customHeight="1" s="15">
@@ -861,10 +873,22 @@
           <t>Počítá koncepce domu s prací z domova?</t>
         </is>
       </c>
-      <c r="E20" s="13" t="n"/>
-      <c r="F20" s="11" t="n"/>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Jeden ze samostatných pokojů lze využít jako pracovnu.</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G20" s="13" t="n"/>
-      <c r="H20" s="13" t="n"/>
+      <c r="H20" s="13" t="inlineStr">
+        <is>
+          <t>E-book Jak se staví Domy s energií / KOMPLET / Validace autora domu / CURRENT / 2026-09-09</t>
+        </is>
+      </c>
       <c r="O20" s="13" t="n"/>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="15">
@@ -960,10 +984,22 @@
           <t>Proč má dům právě dispozici 4+kk?</t>
         </is>
       </c>
-      <c r="E24" s="13" t="n"/>
-      <c r="F24" s="11" t="n"/>
+      <c r="E24" s="13" t="inlineStr">
+        <is>
+          <t>Dům je řešen jako 4+kk: společný obytný prostor s kuchyní doplňují tři samostatné pokoje.</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G24" s="13" t="n"/>
-      <c r="H24" s="13" t="n"/>
+      <c r="H24" s="13" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 14–15</t>
+        </is>
+      </c>
       <c r="O24" s="13" t="n"/>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="15">
@@ -1449,10 +1485,22 @@
           <t>Lze dům na pozemku otočit nebo zrcadlit?</t>
         </is>
       </c>
-      <c r="E49" s="13" t="n"/>
-      <c r="F49" s="11" t="n"/>
+      <c r="E49" s="13" t="inlineStr">
+        <is>
+          <t>Referenční pozemek je mírně svažitý a klesá směrem k jihovýchodu; při dokončovacích pracích se počítá s terénními úpravami a násypem.</t>
+        </is>
+      </c>
+      <c r="F49" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G49" s="13" t="n"/>
-      <c r="H49" s="13" t="n"/>
+      <c r="H49" s="13" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 1 a 26 / Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O49" s="13" t="n"/>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="15">
@@ -1563,10 +1611,22 @@
           <t>Jak poznám, jestli se tento dům na můj pozemek skutečně vejde?</t>
         </is>
       </c>
-      <c r="E55" s="13" t="n"/>
-      <c r="F55" s="11" t="n"/>
+      <c r="E55" s="13" t="inlineStr">
+        <is>
+          <t>Vhodnost konkrétního pozemku je nutné ověřit podle rozměrů domu, odstupů, orientace, přístupu a podmínek konkrétní parcely.</t>
+        </is>
+      </c>
+      <c r="F55" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G55" s="13" t="n"/>
-      <c r="H55" s="13" t="n"/>
+      <c r="H55" s="13" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 1 a 26 / Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O55" s="13" t="n"/>
     </row>
     <row r="56" ht="15.75" customHeight="1" s="15">
@@ -1601,10 +1661,22 @@
           <t>Jak umístění domu ovlivňují přípojky a inženýrské sítě?</t>
         </is>
       </c>
-      <c r="E57" s="13" t="n"/>
-      <c r="F57" s="11" t="n"/>
+      <c r="E57" s="13" t="inlineStr">
+        <is>
+          <t>Umístění domu musí respektovat možnosti napojení konkrétní parcely na technickou infrastrukturu a vedení přípojek.</t>
+        </is>
+      </c>
+      <c r="F57" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G57" s="13" t="n"/>
-      <c r="H57" s="13" t="n"/>
+      <c r="H57" s="13" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
       <c r="O57" s="13" t="n"/>
     </row>
     <row r="58" ht="15.75" customHeight="1" s="15">
@@ -1650,10 +1722,22 @@
           <t>Dá se k domu dobře přidat garáž nebo přístřešek pro auta?</t>
         </is>
       </c>
-      <c r="E59" s="13" t="n"/>
-      <c r="F59" s="11" t="n"/>
+      <c r="E59" s="13" t="inlineStr">
+        <is>
+          <t>Klientské změny doplnily dvě zásuvky v obývacím pokoji a tři zásuvky v exteriéru.</t>
+        </is>
+      </c>
+      <c r="F59" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G59" s="13" t="n"/>
-      <c r="H59" s="13" t="n"/>
+      <c r="H59" s="13" t="inlineStr">
+        <is>
+          <t>Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
+        </is>
+      </c>
       <c r="O59" s="13" t="n"/>
     </row>
     <row r="60" ht="15.75" customHeight="1" s="15">
@@ -1834,10 +1918,22 @@
           <t>Jaké jsou vnější rozměry domu?</t>
         </is>
       </c>
-      <c r="E67" s="13" t="n"/>
-      <c r="F67" s="11" t="n"/>
+      <c r="E67" s="13" t="inlineStr">
+        <is>
+          <t>Zastavěná plocha domu je 129 m².</t>
+        </is>
+      </c>
+      <c r="F67" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G67" s="13" t="n"/>
-      <c r="H67" s="13" t="n"/>
+      <c r="H67" s="13" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 2 a 14</t>
+        </is>
+      </c>
       <c r="O67" s="13" t="n"/>
     </row>
     <row r="68" ht="15.75" customHeight="1" s="15">
@@ -1853,10 +1949,22 @@
           <t>Jak velký je obývací pokoj s kuchyní?</t>
         </is>
       </c>
-      <c r="E68" s="13" t="n"/>
-      <c r="F68" s="11" t="n"/>
+      <c r="E68" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Z hlavního obytného prostoru je přímý vstup na terasu a zahradu.</t>
+        </is>
+      </c>
+      <c r="F68" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G68" s="13" t="n"/>
-      <c r="H68" s="13" t="n"/>
+      <c r="H68" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O68" s="13" t="n"/>
     </row>
     <row r="69" ht="15.75" customHeight="1" s="15">
@@ -1872,10 +1980,22 @@
           <t>Jak velké jsou jednotlivé dětské pokoje?</t>
         </is>
       </c>
-      <c r="E69" s="13" t="n"/>
-      <c r="F69" s="11" t="n"/>
+      <c r="E69" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Jeden z pokojů je koncipován flexibilně pro využití jako dětský pokoj nebo pracovna.</t>
+        </is>
+      </c>
+      <c r="F69" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G69" s="13" t="n"/>
-      <c r="H69" s="13" t="n"/>
+      <c r="H69" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O69" s="13" t="n"/>
     </row>
     <row r="70" ht="15.75" customHeight="1" s="15">
@@ -1891,10 +2011,22 @@
           <t>Jak velká je hlavní ložnice?</t>
         </is>
       </c>
-      <c r="E70" s="13" t="n"/>
-      <c r="F70" s="11" t="n"/>
+      <c r="E70" s="13" t="inlineStr">
+        <is>
+          <t>Ano. U ložnice je řešena integrovaná šatna bez sníženého podhledu.</t>
+        </is>
+      </c>
+      <c r="F70" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G70" s="13" t="n"/>
-      <c r="H70" s="13" t="n"/>
+      <c r="H70" s="13" t="inlineStr">
+        <is>
+          <t>Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
+        </is>
+      </c>
       <c r="O70" s="13" t="n"/>
     </row>
     <row r="71" ht="15.75" customHeight="1" s="15">
@@ -2161,10 +2293,22 @@
           <t>Kolik prostoru zabírá technické zázemí domu?</t>
         </is>
       </c>
-      <c r="E83" s="13" t="n"/>
-      <c r="F83" s="11" t="n"/>
+      <c r="E83" s="13" t="inlineStr">
+        <is>
+          <t>V technické místnosti je v nice boiler, vzadu pod stropem technologická jednotka a před nimi prostor pro rozvaděč.</t>
+        </is>
+      </c>
+      <c r="F83" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G83" s="13" t="n"/>
-      <c r="H83" s="13" t="n"/>
+      <c r="H83" s="13" t="inlineStr">
+        <is>
+          <t>Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
+        </is>
+      </c>
       <c r="O83" s="13" t="n"/>
     </row>
     <row r="84" ht="15.75" customHeight="1" s="15">
@@ -2254,10 +2398,22 @@
           <t>Jak je dům dispozičně řešený?</t>
         </is>
       </c>
-      <c r="E88" s="13" t="n"/>
-      <c r="F88" s="11" t="n"/>
+      <c r="E88" s="13" t="inlineStr">
+        <is>
+          <t>Projektová dokumentace uvádí vytápěnou užitnou plochu 112,9 m², nevytápěnou 53,8 m² a celkovou užitnou plochu 166,7 m².</t>
+        </is>
+      </c>
+      <c r="F88" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G88" s="13" t="n"/>
-      <c r="H88" s="13" t="n"/>
+      <c r="H88" s="13" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 14–15</t>
+        </is>
+      </c>
       <c r="O88" s="13" t="n"/>
     </row>
     <row r="89" ht="15.75" customHeight="1" s="15">
@@ -2418,10 +2574,22 @@
           <t>Kde je umístěná technická místnost?</t>
         </is>
       </c>
-      <c r="E96" s="13" t="n"/>
-      <c r="F96" s="11" t="n"/>
+      <c r="E96" s="13" t="inlineStr">
+        <is>
+          <t>V technické místnosti je v nice boiler, vzadu pod stropem technologická jednotka a před nimi prostor pro rozvaděč.</t>
+        </is>
+      </c>
+      <c r="F96" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G96" s="13" t="n"/>
-      <c r="H96" s="13" t="n"/>
+      <c r="H96" s="13" t="inlineStr">
+        <is>
+          <t>Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
+        </is>
+      </c>
       <c r="O96" s="13" t="n"/>
     </row>
     <row r="97" ht="15.75" customHeight="1" s="15">
@@ -2437,10 +2605,22 @@
           <t>Je z obytného prostoru přímý vstup na terasu?</t>
         </is>
       </c>
-      <c r="E97" s="13" t="n"/>
-      <c r="F97" s="11" t="n"/>
+      <c r="E97" s="13" t="inlineStr">
+        <is>
+          <t>Terasa přímo navazuje na hlavní obytný prostor; velké prosklení a přímý vstup vytvářejí intenzivní propojení interiéru se zahradou.</t>
+        </is>
+      </c>
+      <c r="F97" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G97" s="13" t="n"/>
-      <c r="H97" s="13" t="n"/>
+      <c r="H97" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O97" s="13" t="n"/>
     </row>
     <row r="98" ht="15.75" customHeight="1" s="15">
@@ -2475,10 +2655,22 @@
           <t>Lze některý z pokojů využít jako pracovnu?</t>
         </is>
       </c>
-      <c r="E99" s="13" t="n"/>
-      <c r="F99" s="11" t="n"/>
+      <c r="E99" s="13" t="inlineStr">
+        <is>
+          <t>Ano. V zádveří je dostatek prostoru pro běžný provoz rodiny.</t>
+        </is>
+      </c>
+      <c r="F99" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G99" s="13" t="n"/>
-      <c r="H99" s="13" t="n"/>
+      <c r="H99" s="13" t="inlineStr">
+        <is>
+          <t>E-book Jak se staví Domy s energií / KOMPLET / Validace autora domu / CURRENT / 2026-09-09</t>
+        </is>
+      </c>
       <c r="O99" s="13" t="n"/>
     </row>
     <row r="100" ht="15.75" customHeight="1" s="15">
@@ -2713,10 +2905,22 @@
           <t>Dá se změnit barva střechy?</t>
         </is>
       </c>
-      <c r="E111" s="13" t="n"/>
-      <c r="F111" s="11" t="n"/>
+      <c r="E111" s="13" t="inlineStr">
+        <is>
+          <t>Aktuální referenční provedení má střechu v antracitovém odstínu. Dostupné podklady ale samostatně nepotvrzují, zda lze u tohoto domu v rámci objednávky zvolit jinou barvu střechy.</t>
+        </is>
+      </c>
+      <c r="F111" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G111" s="13" t="n"/>
-      <c r="H111" s="13" t="n"/>
+      <c r="H111" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O111" s="13" t="n"/>
     </row>
     <row r="112" ht="15.75" customHeight="1" s="15">
@@ -2732,10 +2936,22 @@
           <t>Jaké materiály jsou použité na fasádě?</t>
         </is>
       </c>
-      <c r="E112" s="13" t="n"/>
-      <c r="F112" s="11" t="n"/>
+      <c r="E112" s="13" t="inlineStr">
+        <is>
+          <t>Vnější plášť je navržen z BRATEX CLICK – lakovaného pozinkovaného falcovaného plechu v antracitovém odstínu.</t>
+        </is>
+      </c>
+      <c r="F112" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G112" s="13" t="n"/>
-      <c r="H112" s="13" t="n"/>
+      <c r="H112" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 18 a 22</t>
+        </is>
+      </c>
       <c r="O112" s="13" t="n"/>
     </row>
     <row r="113" ht="15.75" customHeight="1" s="15">
@@ -3179,10 +3395,22 @@
           <t>Je možné dům zrcadlově otočit?</t>
         </is>
       </c>
-      <c r="E135" s="13" t="n"/>
-      <c r="F135" s="11" t="n"/>
+      <c r="E135" s="13" t="inlineStr">
+        <is>
+          <t>Referenční pozemek je mírně svažitý a klesá směrem k jihovýchodu; při dokončovacích pracích se počítá s terénními úpravami a násypem.</t>
+        </is>
+      </c>
+      <c r="F135" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G135" s="13" t="n"/>
-      <c r="H135" s="13" t="n"/>
+      <c r="H135" s="13" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 1 a 26 / Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O135" s="13" t="n"/>
     </row>
     <row r="136" ht="15.75" customHeight="1" s="15">
@@ -3198,10 +3426,22 @@
           <t>Dá se jeden z pokojů využít jako pracovna?</t>
         </is>
       </c>
-      <c r="E136" s="13" t="n"/>
-      <c r="F136" s="11" t="n"/>
+      <c r="E136" s="13" t="inlineStr">
+        <is>
+          <t>Ano. V zádveří je dostatek prostoru pro běžný provoz rodiny.</t>
+        </is>
+      </c>
+      <c r="F136" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G136" s="13" t="n"/>
-      <c r="H136" s="13" t="n"/>
+      <c r="H136" s="13" t="inlineStr">
+        <is>
+          <t>E-book Jak se staví Domy s energií / KOMPLET / Validace autora domu / CURRENT / 2026-09-09</t>
+        </is>
+      </c>
       <c r="O136" s="13" t="n"/>
     </row>
     <row r="137" ht="15.75" customHeight="1" s="15">
@@ -3255,10 +3495,22 @@
           <t>Je možné později přidat garáž nebo přístřešek?</t>
         </is>
       </c>
-      <c r="E139" s="13" t="n"/>
-      <c r="F139" s="11" t="n"/>
+      <c r="E139" s="13" t="inlineStr">
+        <is>
+          <t>Klientské změny doplnily dvě zásuvky v obývacím pokoji a tři zásuvky v exteriéru.</t>
+        </is>
+      </c>
+      <c r="F139" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G139" s="13" t="n"/>
-      <c r="H139" s="13" t="n"/>
+      <c r="H139" s="13" t="inlineStr">
+        <is>
+          <t>Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
+        </is>
+      </c>
       <c r="O139" s="13" t="n"/>
     </row>
     <row r="140" ht="15.75" customHeight="1" s="15">
@@ -4389,10 +4641,22 @@
           <t>Je potřeba radonový průzkum nebo měření?</t>
         </is>
       </c>
-      <c r="E199" s="13" t="n"/>
-      <c r="F199" s="11" t="n"/>
+      <c r="E199" s="13" t="inlineStr">
+        <is>
+          <t>Dům je staticky posouzen na zatížení větrem pro II. větrnou zónu a II. kategorii terénu. Stabilitu proti bočnímu tlaku větru zajišťují ztužující stěny a křížové zavětrování ocelovými táhly.</t>
+        </is>
+      </c>
+      <c r="F199" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G199" s="13" t="n"/>
-      <c r="H199" s="13" t="n"/>
+      <c r="H199" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O199" s="13" t="n"/>
     </row>
     <row r="200" ht="15.75" customHeight="1" s="15">
@@ -4633,10 +4897,22 @@
           <t>Jak se řeší drenáže a voda kolem domu?</t>
         </is>
       </c>
-      <c r="E210" s="13" t="n"/>
-      <c r="F210" s="11" t="n"/>
+      <c r="E210" s="13" t="inlineStr">
+        <is>
+          <t>Dešťová voda ze střechy je odváděna do retenčního systému a přebytek je zasakován. Konkrétní potřeba drenáže kolem domu závisí na podmínkách pozemku.</t>
+        </is>
+      </c>
+      <c r="F210" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G210" s="13" t="n"/>
-      <c r="H210" s="13" t="n"/>
+      <c r="H210" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 18 a 30–31</t>
+        </is>
+      </c>
       <c r="O210" s="13" t="n"/>
     </row>
     <row r="211" ht="15.75" customHeight="1" s="15">
@@ -5716,10 +5992,22 @@
           <t>Jak silné jsou obvodové stěny?</t>
         </is>
       </c>
-      <c r="E257" s="13" t="n"/>
-      <c r="F257" s="11" t="n"/>
+      <c r="E257" s="13" t="inlineStr">
+        <is>
+          <t>Koncepční skladba obvodového pláště je: sádrová omítka, Ekopanel, tepelná izolace Climatizer Plus mezi rámy, difuzní fólie, kontralatě, kotvící latě, odvětrávaná mezera a fasádní prvek.</t>
+        </is>
+      </c>
+      <c r="F257" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G257" s="13" t="n"/>
-      <c r="H257" s="13" t="n"/>
+      <c r="H257" s="13" t="inlineStr">
+        <is>
+          <t>E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O257" s="13" t="n"/>
     </row>
     <row r="258" ht="15.75" customHeight="1" s="15">
@@ -5735,10 +6023,22 @@
           <t>Z jakých vrstev se obvodová stěna skládá?</t>
         </is>
       </c>
-      <c r="E258" s="13" t="n"/>
-      <c r="F258" s="11" t="n"/>
+      <c r="E258" s="13" t="inlineStr">
+        <is>
+          <t>Koncepční skladba obvodového pláště je: sádrová omítka, Ekopanel, tepelná izolace Climatizer Plus mezi rámy, difuzní fólie, kontralatě, kotvící latě, odvětrávaná mezera a fasádní prvek.</t>
+        </is>
+      </c>
+      <c r="F258" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G258" s="13" t="n"/>
-      <c r="H258" s="13" t="n"/>
+      <c r="H258" s="13" t="inlineStr">
+        <is>
+          <t>E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O258" s="13" t="n"/>
     </row>
     <row r="259" ht="15.75" customHeight="1" s="15">
@@ -5754,10 +6054,22 @@
           <t>Z čeho jsou vnitřní nosné stěny?</t>
         </is>
       </c>
-      <c r="E259" s="13" t="n"/>
-      <c r="F259" s="11" t="n"/>
+      <c r="E259" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Bungalov 4KK je rámová difuzně otevřená dřevostavba.</t>
+        </is>
+      </c>
+      <c r="F259" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G259" s="13" t="n"/>
-      <c r="H259" s="13" t="n"/>
+      <c r="H259" s="13" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
       <c r="O259" s="13" t="n"/>
     </row>
     <row r="260" ht="15.75" customHeight="1" s="15">
@@ -5835,10 +6147,22 @@
           <t>Jak je řešená konstrukce podlahy?</t>
         </is>
       </c>
-      <c r="E262" s="13" t="n"/>
-      <c r="F262" s="11" t="n"/>
+      <c r="E262" s="13" t="inlineStr">
+        <is>
+          <t>Nosnou konstrukci střechy tvoří soustava dřevěných rámů z jehličnatých KVH hranolů pevnostní třídy C24.</t>
+        </is>
+      </c>
+      <c r="F262" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G262" s="13" t="n"/>
-      <c r="H262" s="13" t="n"/>
+      <c r="H262" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 22</t>
+        </is>
+      </c>
       <c r="O262" s="13" t="n"/>
     </row>
     <row r="263" ht="15.75" customHeight="1" s="15">
@@ -6158,10 +6482,22 @@
           <t>V čem se tento konstrukční systém liší od klasického zděného domu?</t>
         </is>
       </c>
-      <c r="E275" s="13" t="n"/>
-      <c r="F275" s="11" t="n"/>
+      <c r="E275" s="13" t="inlineStr">
+        <is>
+          <t>Dům je řešen jako rámová difuzně otevřená dřevostavba s vnitřní vestavbou z Ekopanelu, výplň tvoří celulóza Climatizer plus, z vnější strany opatřeno difůzní fólií a odvětrávanou fasádou.</t>
+        </is>
+      </c>
+      <c r="F275" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G275" s="13" t="n"/>
-      <c r="H275" s="13" t="n"/>
+      <c r="H275" s="13" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
       <c r="O275" s="13" t="n"/>
     </row>
     <row r="276" ht="15.75" customHeight="1" s="15">
@@ -6225,10 +6561,22 @@
           <t>Jakou barvu má střecha?</t>
         </is>
       </c>
-      <c r="E278" s="13" t="n"/>
-      <c r="F278" s="11" t="n"/>
+      <c r="E278" s="13" t="inlineStr">
+        <is>
+          <t>Střecha je v antracitovém odstínu.</t>
+        </is>
+      </c>
+      <c r="F278" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G278" s="13" t="n"/>
-      <c r="H278" s="13" t="n"/>
+      <c r="H278" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O278" s="13" t="n"/>
     </row>
     <row r="279" ht="15.75" customHeight="1" s="15">
@@ -6325,10 +6673,22 @@
           <t>Jaká je životnost střešní krytiny?</t>
         </is>
       </c>
-      <c r="E282" s="13" t="n"/>
-      <c r="F282" s="11" t="n"/>
+      <c r="E282" s="13" t="inlineStr">
+        <is>
+          <t>60 let a více.</t>
+        </is>
+      </c>
+      <c r="F282" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G282" s="13" t="n"/>
-      <c r="H282" s="13" t="n"/>
+      <c r="H282" s="13" t="inlineStr">
+        <is>
+          <t>Knowledge projection / 31.5</t>
+        </is>
+      </c>
       <c r="O282" s="13" t="n"/>
     </row>
     <row r="283" ht="15.75" customHeight="1" s="15">
@@ -6344,10 +6704,22 @@
           <t>Jakou údržbu střecha potřebuje?</t>
         </is>
       </c>
-      <c r="E283" s="13" t="n"/>
-      <c r="F283" s="11" t="n"/>
+      <c r="E283" s="13" t="inlineStr">
+        <is>
+          <t>Téměř žádnou, vyjma údržby dřevěných částí v exteriéru v intervalu 6-10 let.</t>
+        </is>
+      </c>
+      <c r="F283" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G283" s="13" t="n"/>
-      <c r="H283" s="13" t="n"/>
+      <c r="H283" s="13" t="inlineStr">
+        <is>
+          <t>Knowledge projection / 31.2</t>
+        </is>
+      </c>
       <c r="O283" s="13" t="n"/>
     </row>
     <row r="284" ht="15.75" customHeight="1" s="15">
@@ -6363,10 +6735,22 @@
           <t>Jakou údržbu potřebuje fasáda?</t>
         </is>
       </c>
-      <c r="E284" s="13" t="n"/>
-      <c r="F284" s="11" t="n"/>
+      <c r="E284" s="13" t="inlineStr">
+        <is>
+          <t>Pouze ošetření dřevěných částí v intervalu 6-10 let.</t>
+        </is>
+      </c>
+      <c r="F284" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G284" s="13" t="n"/>
-      <c r="H284" s="13" t="n"/>
+      <c r="H284" s="13" t="inlineStr">
+        <is>
+          <t>Knowledge projection / 31.6</t>
+        </is>
+      </c>
       <c r="O284" s="13" t="n"/>
     </row>
     <row r="285" ht="15.75" customHeight="1" s="15">
@@ -6432,10 +6816,22 @@
           <t>Lze na fasádě použít dřevo nebo jiný obklad?</t>
         </is>
       </c>
-      <c r="E287" s="13" t="n"/>
-      <c r="F287" s="11" t="n"/>
+      <c r="E287" s="13" t="inlineStr">
+        <is>
+          <t>Dřevěné obklady a nosné konstrukce přístřešků – tyto je nutné vždy ošetřit v intervalu 6-10 let.</t>
+        </is>
+      </c>
+      <c r="F287" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G287" s="13" t="n"/>
-      <c r="H287" s="13" t="n"/>
+      <c r="H287" s="13" t="inlineStr">
+        <is>
+          <t>Knowledge projection / 13.19</t>
+        </is>
+      </c>
       <c r="O287" s="13" t="n"/>
     </row>
     <row r="288" ht="15.75" customHeight="1" s="15">
@@ -6694,10 +7090,22 @@
           <t>Jaké jsou hlavní důvody pro volbu právě těchto materiálů střechy a fasády?</t>
         </is>
       </c>
-      <c r="E296" s="13" t="n"/>
-      <c r="F296" s="11" t="n"/>
+      <c r="E296" s="13" t="inlineStr">
+        <is>
+          <t>Použitý vnější plášť pracuje s lakovaným pozinkovaným plechem BRATEX CLICK; dostupné podklady popisují materiálové řešení, nikoli samostatné autorské zdůvodnění všech důvodů jeho volby.</t>
+        </is>
+      </c>
+      <c r="F296" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G296" s="13" t="n"/>
-      <c r="H296" s="13" t="n"/>
+      <c r="H296" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 18 a 22</t>
+        </is>
+      </c>
       <c r="O296" s="13" t="n"/>
     </row>
     <row r="297" ht="15.75" customHeight="1" s="15">
@@ -7009,10 +7417,22 @@
           <t>Jak jsou řešené dveře z obývacího prostoru na terasu?</t>
         </is>
       </c>
-      <c r="E307" s="13" t="n"/>
-      <c r="F307" s="11" t="n"/>
+      <c r="E307" s="13" t="inlineStr">
+        <is>
+          <t>Obytný prostor je propojen s terasou dveřmi; CURRENT validace zároveň potvrzuje, že terasové dveře nejsou řešeny jako posuvné.</t>
+        </is>
+      </c>
+      <c r="F307" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G307" s="13" t="n"/>
-      <c r="H307" s="13" t="n"/>
+      <c r="H307" s="13" t="inlineStr">
+        <is>
+          <t>E-book Jak se staví Domy s energií / KOMPLET / Validace autora domu / CURRENT / 2026-09-09</t>
+        </is>
+      </c>
       <c r="O307" s="13" t="n"/>
     </row>
     <row r="308" ht="15.75" customHeight="1" s="15">
@@ -7197,10 +7617,22 @@
           <t>Jak dobře okna tlumí hluk zvenčí?</t>
         </is>
       </c>
-      <c r="E315" s="13" t="n"/>
-      <c r="F315" s="11" t="n"/>
+      <c r="E315" s="13" t="inlineStr">
+        <is>
+          <t>Výborně, plastnová okna s troskly jsou špičkou v dané kategorii.</t>
+        </is>
+      </c>
+      <c r="F315" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G315" s="13" t="n"/>
-      <c r="H315" s="13" t="n"/>
+      <c r="H315" s="13" t="inlineStr">
+        <is>
+          <t>Knowledge projection / 29.7</t>
+        </is>
+      </c>
       <c r="O315" s="13" t="n"/>
     </row>
     <row r="316" ht="15.75" customHeight="1" s="15">
@@ -7302,10 +7734,22 @@
           <t>Nebude v domě v létě příliš horko?</t>
         </is>
       </c>
-      <c r="E320" s="13" t="n"/>
-      <c r="F320" s="11" t="n"/>
+      <c r="E320" s="13" t="inlineStr">
+        <is>
+          <t>Dům používá venkovní stínění a rekuperační jednotka umožňuje v létě chlazení. Tyto prvky omezují riziko letního přehřívání; konkrétní maximální vnitřní teplotu dostupné podklady neuvádějí.</t>
+        </is>
+      </c>
+      <c r="F320" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G320" s="13" t="n"/>
-      <c r="H320" s="13" t="n"/>
+      <c r="H320" s="13" t="inlineStr">
+        <is>
+          <t>PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
+        </is>
+      </c>
       <c r="O320" s="13" t="n"/>
     </row>
     <row r="321" ht="15.75" customHeight="1" s="15">
@@ -7352,10 +7796,22 @@
           <t>Jak dům chrání interiér před přehříváním?</t>
         </is>
       </c>
-      <c r="E322" s="13" t="n"/>
-      <c r="F322" s="11" t="n"/>
+      <c r="E322" s="13" t="inlineStr">
+        <is>
+          <t>Okna mají izolační trojskla a dům používá venkovní roletové žaluzie, které umožňují omezit přímé sluneční záření před zasklením. Konkrétní snížení letní vnitřní teploty dostupné podklady nevyčíslují.</t>
+        </is>
+      </c>
+      <c r="F322" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G322" s="13" t="n"/>
-      <c r="H322" s="13" t="n"/>
+      <c r="H322" s="13" t="inlineStr">
+        <is>
+          <t>PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023 / Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O322" s="13" t="n"/>
     </row>
     <row r="323" ht="15.75" customHeight="1" s="15">
@@ -8141,10 +8597,22 @@
           <t>Jak je řešená ochrana elektroinstalace proti poruchám?</t>
         </is>
       </c>
-      <c r="E351" s="13" t="n"/>
-      <c r="F351" s="11" t="n"/>
+      <c r="E351" s="13" t="inlineStr">
+        <is>
+          <t>Bezpečný stav elektroinstalace se dokládá příslušnou revizí; konkrétní ochranné prvky musí odpovídat projektové dokumentaci a příslušným předpisům.</t>
+        </is>
+      </c>
+      <c r="F351" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G351" s="13" t="n"/>
-      <c r="H351" s="13" t="n"/>
+      <c r="H351" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023</t>
+        </is>
+      </c>
       <c r="O351" s="13" t="n"/>
     </row>
     <row r="352" ht="15.75" customHeight="1" s="15">
@@ -8749,10 +9217,22 @@
           <t>Kudy jsou technické rozvody v konstrukci vedené?</t>
         </is>
       </c>
-      <c r="E375" s="13" t="n"/>
-      <c r="F375" s="11" t="n"/>
+      <c r="E375" s="13" t="inlineStr">
+        <is>
+          <t>Technické rozvody jsou provedeny podle projektové dokumentace. Přesné trasy jednotlivých vedení je nutné určovat podle dokumentace skutečného provedení a konkrétní realizace.</t>
+        </is>
+      </c>
+      <c r="F375" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G375" s="13" t="n"/>
-      <c r="H375" s="13" t="n"/>
+      <c r="H375" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023</t>
+        </is>
+      </c>
       <c r="O375" s="13" t="n"/>
     </row>
     <row r="376" ht="15.75" customHeight="1" s="15">
@@ -9295,10 +9775,22 @@
           <t>Jak hlučné jsou technologie domu?</t>
         </is>
       </c>
-      <c r="E395" s="13" t="n"/>
-      <c r="F395" s="11" t="n"/>
+      <c r="E395" s="13" t="inlineStr">
+        <is>
+          <t>Dům používá technická zařízení včetně řízeného větrání. Dostupné podklady ale neobsahují jednotné naměřené hodnoty hlučnosti všech technologií v dokončeném domě.</t>
+        </is>
+      </c>
+      <c r="F395" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G395" s="13" t="n"/>
-      <c r="H395" s="13" t="n"/>
+      <c r="H395" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-09</t>
+        </is>
+      </c>
       <c r="O395" s="13" t="n"/>
     </row>
     <row r="396" ht="15.75" customHeight="1" s="15">
@@ -9372,10 +9864,22 @@
           <t>Jak často je potřeba technologie servisovat?</t>
         </is>
       </c>
-      <c r="E398" s="13" t="n"/>
-      <c r="F398" s="11" t="n"/>
+      <c r="E398" s="13" t="inlineStr">
+        <is>
+          <t>Servisní intervaly technologií nejsou pro všechny prvky domu v dostupných podkladech jednotně stanoveny. Řídí se dokumentací a servisními požadavky konkrétních výrobců jednotlivých zařízení.</t>
+        </is>
+      </c>
+      <c r="F398" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G398" s="13" t="n"/>
-      <c r="H398" s="13" t="n"/>
+      <c r="H398" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023</t>
+        </is>
+      </c>
       <c r="O398" s="13" t="n"/>
     </row>
     <row r="399" ht="15.75" customHeight="1" s="15">
@@ -9609,10 +10113,22 @@
           <t>Je podlaha vhodná pro podlahové vytápění?</t>
         </is>
       </c>
-      <c r="E410" s="13" t="n"/>
-      <c r="F410" s="11" t="n"/>
+      <c r="E410" s="13" t="inlineStr">
+        <is>
+          <t>Aktuální konfigurace používá elektrické topné fólie pod dřevěnou podlahou, takže použitá podlahová skladba s tímto způsobem vytápění počítá.</t>
+        </is>
+      </c>
+      <c r="F410" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G410" s="13" t="n"/>
-      <c r="H410" s="13" t="n"/>
+      <c r="H410" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023, str. 24 / Klientské změny č. 2 / Bungalov 4KK / 20.10.2023 / B Souhrnná technická zpráva 11/2023</t>
+        </is>
+      </c>
       <c r="O410" s="13" t="n"/>
     </row>
     <row r="411" ht="15.75" customHeight="1" s="15">
@@ -9885,10 +10401,22 @@
           <t>Jak velký je obývací pokoj s kuchyní?</t>
         </is>
       </c>
-      <c r="E424" s="13" t="n"/>
-      <c r="F424" s="11" t="n"/>
+      <c r="E424" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Z hlavního obytného prostoru je přímý vstup na terasu a zahradu.</t>
+        </is>
+      </c>
+      <c r="F424" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G424" s="13" t="n"/>
-      <c r="H424" s="13" t="n"/>
+      <c r="H424" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O424" s="13" t="n"/>
     </row>
     <row r="425" ht="15.75" customHeight="1" s="15">
@@ -10030,10 +10558,22 @@
           <t>Jak je obytný prostor propojený se zahradou?</t>
         </is>
       </c>
-      <c r="E431" s="13" t="n"/>
-      <c r="F431" s="11" t="n"/>
+      <c r="E431" s="13" t="inlineStr">
+        <is>
+          <t>Terasa přímo navazuje na hlavní obytný prostor; velké prosklení a přímý vstup vytvářejí intenzivní propojení interiéru se zahradou.</t>
+        </is>
+      </c>
+      <c r="F431" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G431" s="13" t="n"/>
-      <c r="H431" s="13" t="n"/>
+      <c r="H431" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O431" s="13" t="n"/>
     </row>
     <row r="432" ht="15.75" customHeight="1" s="15">
@@ -10201,10 +10741,22 @@
           <t>Jak je v obývacím prostoru řešené stínění velkých oken?</t>
         </is>
       </c>
-      <c r="E440" s="13" t="n"/>
-      <c r="F440" s="11" t="n"/>
+      <c r="E440" s="13" t="inlineStr">
+        <is>
+          <t>Venkovní stínění je řešeno roletovými žaluziemi.</t>
+        </is>
+      </c>
+      <c r="F440" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G440" s="13" t="n"/>
-      <c r="H440" s="13" t="n"/>
+      <c r="H440" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O440" s="13" t="n"/>
     </row>
     <row r="441" ht="15.75" customHeight="1" s="15">
@@ -10220,10 +10772,22 @@
           <t>Nebude se obytný prostor kvůli velkému prosklení v létě přehřívat?</t>
         </is>
       </c>
-      <c r="E441" s="13" t="n"/>
-      <c r="F441" s="11" t="n"/>
+      <c r="E441" s="13" t="inlineStr">
+        <is>
+          <t>Dům používá venkovní stínění a rekuperační jednotka umožňuje v létě chlazení. Tyto prvky omezují riziko letního přehřívání; konkrétní maximální vnitřní teplotu dostupné podklady neuvádějí.</t>
+        </is>
+      </c>
+      <c r="F441" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G441" s="13" t="n"/>
-      <c r="H441" s="13" t="n"/>
+      <c r="H441" s="13" t="inlineStr">
+        <is>
+          <t>PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
+        </is>
+      </c>
       <c r="O441" s="13" t="n"/>
     </row>
     <row r="442" ht="15.75" customHeight="1" s="15">
@@ -10629,10 +11193,22 @@
           <t>Je z kuchyně dobře dostupná terasa pro venkovní stolování?</t>
         </is>
       </c>
-      <c r="E462" s="13" t="n"/>
-      <c r="F462" s="11" t="n"/>
+      <c r="E462" s="13" t="inlineStr">
+        <is>
+          <t>Terasa přímo navazuje na hlavní obytný prostor; velké prosklení a přímý vstup vytvářejí intenzivní propojení interiéru se zahradou.</t>
+        </is>
+      </c>
+      <c r="F462" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G462" s="13" t="n"/>
-      <c r="H462" s="13" t="n"/>
+      <c r="H462" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O462" s="13" t="n"/>
     </row>
     <row r="463" ht="15.75" customHeight="1" s="15">
@@ -10703,10 +11279,22 @@
           <t>Jak velká je hlavní ložnice?</t>
         </is>
       </c>
-      <c r="E466" s="13" t="n"/>
-      <c r="F466" s="11" t="n"/>
+      <c r="E466" s="13" t="inlineStr">
+        <is>
+          <t>Ano. U ložnice je řešena integrovaná šatna bez sníženého podhledu.</t>
+        </is>
+      </c>
+      <c r="F466" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G466" s="13" t="n"/>
-      <c r="H466" s="13" t="n"/>
+      <c r="H466" s="13" t="inlineStr">
+        <is>
+          <t>Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
+        </is>
+      </c>
       <c r="O466" s="13" t="n"/>
     </row>
     <row r="467" ht="15.75" customHeight="1" s="15">
@@ -10722,10 +11310,22 @@
           <t>Jak velké jsou dětské pokoje?</t>
         </is>
       </c>
-      <c r="E467" s="13" t="n"/>
-      <c r="F467" s="11" t="n"/>
+      <c r="E467" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Jeden z pokojů je koncipován flexibilně pro využití jako dětský pokoj nebo pracovna.</t>
+        </is>
+      </c>
+      <c r="F467" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G467" s="13" t="n"/>
-      <c r="H467" s="13" t="n"/>
+      <c r="H467" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O467" s="13" t="n"/>
     </row>
     <row r="468" ht="15.75" customHeight="1" s="15">
@@ -11031,10 +11631,22 @@
           <t>Jak se pokoje větrají a jak se v nich reguluje teplota?</t>
         </is>
       </c>
-      <c r="E482" s="13" t="n"/>
-      <c r="F482" s="11" t="n"/>
+      <c r="E482" s="13" t="inlineStr">
+        <is>
+          <t>Pokoje jsou větrány systémem nuceného řízeného větrání s rekuperací. Přesný způsob individuální regulace teploty v každém pokoji dostupné podklady samostatně nepotvrzují.</t>
+        </is>
+      </c>
+      <c r="F482" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G482" s="13" t="n"/>
-      <c r="H482" s="13" t="n"/>
+      <c r="H482" s="13" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
       <c r="O482" s="13" t="n"/>
     </row>
     <row r="483" ht="15.75" customHeight="1" s="15">
@@ -11050,10 +11662,22 @@
           <t>Lze pokoje zatemnit pro pohodlné spaní?</t>
         </is>
       </c>
-      <c r="E483" s="13" t="n"/>
-      <c r="F483" s="11" t="n"/>
+      <c r="E483" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Dům používá venkovní roletové žaluzie, které lze využít také pro omezení světla v pokojích.</t>
+        </is>
+      </c>
+      <c r="F483" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G483" s="13" t="n"/>
-      <c r="H483" s="13" t="n"/>
+      <c r="H483" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O483" s="13" t="n"/>
     </row>
     <row r="484" ht="15.75" customHeight="1" s="15">
@@ -11333,10 +11957,22 @@
           <t>Jak je koupelna větraná?</t>
         </is>
       </c>
-      <c r="E498" s="13" t="n"/>
-      <c r="F498" s="11" t="n"/>
+      <c r="E498" s="13" t="inlineStr">
+        <is>
+          <t>Dům využívá řízené větrání s rekuperací tepla.</t>
+        </is>
+      </c>
+      <c r="F498" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G498" s="13" t="n"/>
-      <c r="H498" s="13" t="n"/>
+      <c r="H498" s="13" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
       <c r="O498" s="13" t="n"/>
     </row>
     <row r="499" ht="15.75" customHeight="1" s="15">
@@ -11685,10 +12321,22 @@
           <t>Jak velká je technická místnost?</t>
         </is>
       </c>
-      <c r="E516" s="13" t="n"/>
-      <c r="F516" s="11" t="n"/>
+      <c r="E516" s="13" t="inlineStr">
+        <is>
+          <t>V technické místnosti je v nice boiler, vzadu pod stropem technologická jednotka a před nimi prostor pro rozvaděč.</t>
+        </is>
+      </c>
+      <c r="F516" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G516" s="13" t="n"/>
-      <c r="H516" s="13" t="n"/>
+      <c r="H516" s="13" t="inlineStr">
+        <is>
+          <t>Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
+        </is>
+      </c>
       <c r="O516" s="13" t="n"/>
     </row>
     <row r="517" ht="15.75" customHeight="1" s="15">
@@ -11735,10 +12383,22 @@
           <t>Je v technické místnosti místo pro pračku a sušičku?</t>
         </is>
       </c>
-      <c r="E518" s="13" t="n"/>
-      <c r="F518" s="11" t="n"/>
+      <c r="E518" s="13" t="inlineStr">
+        <is>
+          <t>Technická místnost soustřeďuje technické zázemí domu. Dostupné podklady ale samostatně nepotvrzují konkrétní finální umístění pračky a sušičky.</t>
+        </is>
+      </c>
+      <c r="F518" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G518" s="13" t="n"/>
-      <c r="H518" s="13" t="n"/>
+      <c r="H518" s="13" t="inlineStr">
+        <is>
+          <t>Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
+        </is>
+      </c>
       <c r="O518" s="13" t="n"/>
     </row>
     <row r="519" ht="15.75" customHeight="1" s="15">
@@ -12805,10 +13465,22 @@
           <t>Je z obývacího pokoje přímý výhled do zahrady?</t>
         </is>
       </c>
-      <c r="E574" s="13" t="n"/>
-      <c r="F574" s="11" t="n"/>
+      <c r="E574" s="13" t="inlineStr">
+        <is>
+          <t>Terasa přímo navazuje na hlavní obytný prostor; velké prosklení a přímý vstup vytvářejí intenzivní propojení interiéru se zahradou.</t>
+        </is>
+      </c>
+      <c r="F574" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G574" s="13" t="n"/>
-      <c r="H574" s="13" t="n"/>
+      <c r="H574" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O574" s="13" t="n"/>
     </row>
     <row r="575" ht="15.75" customHeight="1" s="15">
@@ -12824,10 +13496,22 @@
           <t>Jak je dům propojený se zahradou?</t>
         </is>
       </c>
-      <c r="E575" s="13" t="n"/>
-      <c r="F575" s="11" t="n"/>
+      <c r="E575" s="13" t="inlineStr">
+        <is>
+          <t>Terasa přímo navazuje na hlavní obytný prostor; velké prosklení a přímý vstup vytvářejí intenzivní propojení interiéru se zahradou.</t>
+        </is>
+      </c>
+      <c r="F575" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G575" s="13" t="n"/>
-      <c r="H575" s="13" t="n"/>
+      <c r="H575" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O575" s="13" t="n"/>
     </row>
     <row r="576" ht="15.75" customHeight="1" s="15">
@@ -13064,10 +13748,22 @@
           <t>Jak se řeší soukromí při velkém propojení interiéru se zahradou?</t>
         </is>
       </c>
-      <c r="E587" s="13" t="n"/>
-      <c r="F587" s="11" t="n"/>
+      <c r="E587" s="13" t="inlineStr">
+        <is>
+          <t>Soukromí u prosklených ploch lze podpořit venkovními roletovými žaluziemi.</t>
+        </is>
+      </c>
+      <c r="F587" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G587" s="13" t="n"/>
-      <c r="H587" s="13" t="n"/>
+      <c r="H587" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O587" s="13" t="n"/>
     </row>
     <row r="588" ht="15.75" customHeight="1" s="15">
@@ -13083,10 +13779,22 @@
           <t>Nezpůsobují velké prosklené plochy v létě přehřívání?</t>
         </is>
       </c>
-      <c r="E588" s="13" t="n"/>
-      <c r="F588" s="11" t="n"/>
+      <c r="E588" s="13" t="inlineStr">
+        <is>
+          <t>Dům používá venkovní stínění a rekuperační jednotka umožňuje v létě chlazení. Tyto prvky omezují riziko letního přehřívání; konkrétní maximální vnitřní teplotu dostupné podklady neuvádějí.</t>
+        </is>
+      </c>
+      <c r="F588" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G588" s="13" t="n"/>
-      <c r="H588" s="13" t="n"/>
+      <c r="H588" s="13" t="inlineStr">
+        <is>
+          <t>PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
+        </is>
+      </c>
       <c r="O588" s="13" t="n"/>
     </row>
     <row r="589" ht="15.75" customHeight="1" s="15">
@@ -13307,10 +14015,22 @@
           <t>Je z kuchyně dobře dostupná terasa pro venkovní stolování?</t>
         </is>
       </c>
-      <c r="E598" s="13" t="n"/>
-      <c r="F598" s="11" t="n"/>
+      <c r="E598" s="13" t="inlineStr">
+        <is>
+          <t>Terasa přímo navazuje na hlavní obytný prostor; velké prosklení a přímý vstup vytvářejí intenzivní propojení interiéru se zahradou.</t>
+        </is>
+      </c>
+      <c r="F598" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G598" s="13" t="n"/>
-      <c r="H598" s="13" t="n"/>
+      <c r="H598" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O598" s="13" t="n"/>
     </row>
     <row r="599" ht="15.75" customHeight="1" s="15">
@@ -13376,10 +14096,22 @@
           <t>Jak dům funguje při častém přecházení mezi interiérem a zahradou?</t>
         </is>
       </c>
-      <c r="E601" s="13" t="n"/>
-      <c r="F601" s="11" t="n"/>
+      <c r="E601" s="13" t="inlineStr">
+        <is>
+          <t>Terasa přímo navazuje na hlavní obytný prostor; velké prosklení a přímý vstup vytvářejí intenzivní propojení interiéru se zahradou.</t>
+        </is>
+      </c>
+      <c r="F601" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G601" s="13" t="n"/>
-      <c r="H601" s="13" t="n"/>
+      <c r="H601" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
+        </is>
+      </c>
       <c r="O601" s="13" t="n"/>
     </row>
     <row r="602" ht="15.75" customHeight="1" s="15">
@@ -13783,10 +14515,22 @@
           <t>Je v ložnici slyšet provoz technologií domu?</t>
         </is>
       </c>
-      <c r="E620" s="13" t="n"/>
-      <c r="F620" s="11" t="n"/>
+      <c r="E620" s="13" t="inlineStr">
+        <is>
+          <t>Dostupné podklady neobsahují konkrétní měření hluku technologií v ložnici, takže nelze bezpečně tvrdit, že jejich provoz není slyšet.</t>
+        </is>
+      </c>
+      <c r="F620" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G620" s="13" t="n"/>
-      <c r="H620" s="13" t="n"/>
+      <c r="H620" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-09</t>
+        </is>
+      </c>
       <c r="O620" s="13" t="n"/>
     </row>
     <row r="621" ht="15.75" customHeight="1" s="15">
@@ -13902,10 +14646,22 @@
           <t>Je v dřevostavbě větší hluk než ve zděném domě?</t>
         </is>
       </c>
-      <c r="E625" s="13" t="n"/>
-      <c r="F625" s="11" t="n"/>
+      <c r="E625" s="13" t="inlineStr">
+        <is>
+          <t>Samotný konstrukční princip dřevostavby nestačí k obecnému tvrzení, že je dům hlučnější než zděný. Akustické chování je nutné hodnotit podle konkrétních skladeb a jejich parametrů.</t>
+        </is>
+      </c>
+      <c r="F625" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G625" s="13" t="n"/>
-      <c r="H625" s="13" t="n"/>
+      <c r="H625" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023</t>
+        </is>
+      </c>
       <c r="O625" s="13" t="n"/>
     </row>
     <row r="626" ht="15.75" customHeight="1" s="15">
@@ -14301,10 +15057,22 @@
           <t>Jak spotřebu ovlivňuje rekuperace?</t>
         </is>
       </c>
-      <c r="E644" s="13" t="n"/>
-      <c r="F644" s="11" t="n"/>
+      <c r="E644" s="13" t="inlineStr">
+        <is>
+          <t>Rekuperace omezuje tepelné ztráty větráním tím, že využívá teplo odváděného vzduchu. Dostupné podklady ale samostatně nevyčíslují její podíl na celkové spotřebě tohoto domu.</t>
+        </is>
+      </c>
+      <c r="F644" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G644" s="13" t="n"/>
-      <c r="H644" s="13" t="n"/>
+      <c r="H644" s="13" t="inlineStr">
+        <is>
+          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+        </is>
+      </c>
       <c r="O644" s="13" t="n"/>
     </row>
     <row r="645" ht="15.75" customHeight="1" s="15">
@@ -15013,10 +15781,22 @@
           <t>Co můžu dělat, aby dům vydržel co nejdéle v dobrém stavu?</t>
         </is>
       </c>
-      <c r="E674" s="13" t="n"/>
-      <c r="F674" s="11" t="n"/>
+      <c r="E674" s="13" t="inlineStr">
+        <is>
+          <t>Pro dlouhou životnost domu je důležité provádět běžnou údržbu, zejména pravidelně ošetřovat exponované dřevěné části a dodržovat servisní požadavky použitých technologií.</t>
+        </is>
+      </c>
+      <c r="F674" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G674" s="13" t="n"/>
-      <c r="H674" s="13" t="n"/>
+      <c r="H674" s="13" t="inlineStr">
+        <is>
+          <t>Knowledge projection / 31.2</t>
+        </is>
+      </c>
       <c r="O674" s="13" t="n"/>
     </row>
     <row r="675" ht="15.75" customHeight="1" s="15">

</xml_diff>

<commit_message>
Revert "docs(knowledge): globally harvest grounded Bungalov 4KK knowledge"
This reverts commit 17b286a90ff01e352283697f6b2c87cbaa7f3051.
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 02.xlsx
+++ b/docs/knowledge/znalostní báze – mustr 02.xlsx
@@ -576,22 +576,10 @@
           <t>Je tento dům vhodný pro rodinu s dětmi?</t>
         </is>
       </c>
-      <c r="E5" s="13" t="inlineStr">
-        <is>
-          <t>Dům má dispozici 4+kk a tři samostatné pokoje vedle společného obytného prostoru; dispozičně tedy umožňuje běžné rodinné bydlení s dětmi.</t>
-        </is>
-      </c>
-      <c r="F5" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E5" s="13" t="n"/>
+      <c r="F5" s="11" t="n"/>
       <c r="G5" s="13" t="n"/>
-      <c r="H5" s="13" t="inlineStr">
-        <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 14–15</t>
-        </is>
-      </c>
+      <c r="H5" s="13" t="n"/>
       <c r="O5" s="13" t="n"/>
     </row>
     <row r="6" ht="15.75" customHeight="1" s="15">
@@ -873,22 +861,10 @@
           <t>Počítá koncepce domu s prací z domova?</t>
         </is>
       </c>
-      <c r="E20" s="13" t="inlineStr">
-        <is>
-          <t>Ano. Jeden ze samostatných pokojů lze využít jako pracovnu.</t>
-        </is>
-      </c>
-      <c r="F20" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E20" s="13" t="n"/>
+      <c r="F20" s="11" t="n"/>
       <c r="G20" s="13" t="n"/>
-      <c r="H20" s="13" t="inlineStr">
-        <is>
-          <t>E-book Jak se staví Domy s energií / KOMPLET / Validace autora domu / CURRENT / 2026-09-09</t>
-        </is>
-      </c>
+      <c r="H20" s="13" t="n"/>
       <c r="O20" s="13" t="n"/>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="15">
@@ -984,22 +960,10 @@
           <t>Proč má dům právě dispozici 4+kk?</t>
         </is>
       </c>
-      <c r="E24" s="13" t="inlineStr">
-        <is>
-          <t>Dům je řešen jako 4+kk: společný obytný prostor s kuchyní doplňují tři samostatné pokoje.</t>
-        </is>
-      </c>
-      <c r="F24" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E24" s="13" t="n"/>
+      <c r="F24" s="11" t="n"/>
       <c r="G24" s="13" t="n"/>
-      <c r="H24" s="13" t="inlineStr">
-        <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 14–15</t>
-        </is>
-      </c>
+      <c r="H24" s="13" t="n"/>
       <c r="O24" s="13" t="n"/>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="15">
@@ -1485,22 +1449,10 @@
           <t>Lze dům na pozemku otočit nebo zrcadlit?</t>
         </is>
       </c>
-      <c r="E49" s="13" t="inlineStr">
-        <is>
-          <t>Referenční pozemek je mírně svažitý a klesá směrem k jihovýchodu; při dokončovacích pracích se počítá s terénními úpravami a násypem.</t>
-        </is>
-      </c>
-      <c r="F49" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E49" s="13" t="n"/>
+      <c r="F49" s="11" t="n"/>
       <c r="G49" s="13" t="n"/>
-      <c r="H49" s="13" t="inlineStr">
-        <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 1 a 26 / Studie Bungalov 4KK / 01.11.2022</t>
-        </is>
-      </c>
+      <c r="H49" s="13" t="n"/>
       <c r="O49" s="13" t="n"/>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="15">
@@ -1611,22 +1563,10 @@
           <t>Jak poznám, jestli se tento dům na můj pozemek skutečně vejde?</t>
         </is>
       </c>
-      <c r="E55" s="13" t="inlineStr">
-        <is>
-          <t>Vhodnost konkrétního pozemku je nutné ověřit podle rozměrů domu, odstupů, orientace, přístupu a podmínek konkrétní parcely.</t>
-        </is>
-      </c>
-      <c r="F55" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E55" s="13" t="n"/>
+      <c r="F55" s="11" t="n"/>
       <c r="G55" s="13" t="n"/>
-      <c r="H55" s="13" t="inlineStr">
-        <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 1 a 26 / Studie Bungalov 4KK / 01.11.2022</t>
-        </is>
-      </c>
+      <c r="H55" s="13" t="n"/>
       <c r="O55" s="13" t="n"/>
     </row>
     <row r="56" ht="15.75" customHeight="1" s="15">
@@ -1661,22 +1601,10 @@
           <t>Jak umístění domu ovlivňují přípojky a inženýrské sítě?</t>
         </is>
       </c>
-      <c r="E57" s="13" t="inlineStr">
-        <is>
-          <t>Umístění domu musí respektovat možnosti napojení konkrétní parcely na technickou infrastrukturu a vedení přípojek.</t>
-        </is>
-      </c>
-      <c r="F57" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E57" s="13" t="n"/>
+      <c r="F57" s="11" t="n"/>
       <c r="G57" s="13" t="n"/>
-      <c r="H57" s="13" t="inlineStr">
-        <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
-        </is>
-      </c>
+      <c r="H57" s="13" t="n"/>
       <c r="O57" s="13" t="n"/>
     </row>
     <row r="58" ht="15.75" customHeight="1" s="15">
@@ -1722,22 +1650,10 @@
           <t>Dá se k domu dobře přidat garáž nebo přístřešek pro auta?</t>
         </is>
       </c>
-      <c r="E59" s="13" t="inlineStr">
-        <is>
-          <t>Klientské změny doplnily dvě zásuvky v obývacím pokoji a tři zásuvky v exteriéru.</t>
-        </is>
-      </c>
-      <c r="F59" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E59" s="13" t="n"/>
+      <c r="F59" s="11" t="n"/>
       <c r="G59" s="13" t="n"/>
-      <c r="H59" s="13" t="inlineStr">
-        <is>
-          <t>Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
-        </is>
-      </c>
+      <c r="H59" s="13" t="n"/>
       <c r="O59" s="13" t="n"/>
     </row>
     <row r="60" ht="15.75" customHeight="1" s="15">
@@ -1918,22 +1834,10 @@
           <t>Jaké jsou vnější rozměry domu?</t>
         </is>
       </c>
-      <c r="E67" s="13" t="inlineStr">
-        <is>
-          <t>Zastavěná plocha domu je 129 m².</t>
-        </is>
-      </c>
-      <c r="F67" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E67" s="13" t="n"/>
+      <c r="F67" s="11" t="n"/>
       <c r="G67" s="13" t="n"/>
-      <c r="H67" s="13" t="inlineStr">
-        <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 2 a 14</t>
-        </is>
-      </c>
+      <c r="H67" s="13" t="n"/>
       <c r="O67" s="13" t="n"/>
     </row>
     <row r="68" ht="15.75" customHeight="1" s="15">
@@ -1949,22 +1853,10 @@
           <t>Jak velký je obývací pokoj s kuchyní?</t>
         </is>
       </c>
-      <c r="E68" s="13" t="inlineStr">
-        <is>
-          <t>Ano. Z hlavního obytného prostoru je přímý vstup na terasu a zahradu.</t>
-        </is>
-      </c>
-      <c r="F68" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E68" s="13" t="n"/>
+      <c r="F68" s="11" t="n"/>
       <c r="G68" s="13" t="n"/>
-      <c r="H68" s="13" t="inlineStr">
-        <is>
-          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
-        </is>
-      </c>
+      <c r="H68" s="13" t="n"/>
       <c r="O68" s="13" t="n"/>
     </row>
     <row r="69" ht="15.75" customHeight="1" s="15">
@@ -1980,22 +1872,10 @@
           <t>Jak velké jsou jednotlivé dětské pokoje?</t>
         </is>
       </c>
-      <c r="E69" s="13" t="inlineStr">
-        <is>
-          <t>Ano. Jeden z pokojů je koncipován flexibilně pro využití jako dětský pokoj nebo pracovna.</t>
-        </is>
-      </c>
-      <c r="F69" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E69" s="13" t="n"/>
+      <c r="F69" s="11" t="n"/>
       <c r="G69" s="13" t="n"/>
-      <c r="H69" s="13" t="inlineStr">
-        <is>
-          <t>Studie Bungalov 4KK / 01.11.2022</t>
-        </is>
-      </c>
+      <c r="H69" s="13" t="n"/>
       <c r="O69" s="13" t="n"/>
     </row>
     <row r="70" ht="15.75" customHeight="1" s="15">
@@ -2011,22 +1891,10 @@
           <t>Jak velká je hlavní ložnice?</t>
         </is>
       </c>
-      <c r="E70" s="13" t="inlineStr">
-        <is>
-          <t>Ano. U ložnice je řešena integrovaná šatna bez sníženého podhledu.</t>
-        </is>
-      </c>
-      <c r="F70" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E70" s="13" t="n"/>
+      <c r="F70" s="11" t="n"/>
       <c r="G70" s="13" t="n"/>
-      <c r="H70" s="13" t="inlineStr">
-        <is>
-          <t>Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
-        </is>
-      </c>
+      <c r="H70" s="13" t="n"/>
       <c r="O70" s="13" t="n"/>
     </row>
     <row r="71" ht="15.75" customHeight="1" s="15">
@@ -2293,22 +2161,10 @@
           <t>Kolik prostoru zabírá technické zázemí domu?</t>
         </is>
       </c>
-      <c r="E83" s="13" t="inlineStr">
-        <is>
-          <t>V technické místnosti je v nice boiler, vzadu pod stropem technologická jednotka a před nimi prostor pro rozvaděč.</t>
-        </is>
-      </c>
-      <c r="F83" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E83" s="13" t="n"/>
+      <c r="F83" s="11" t="n"/>
       <c r="G83" s="13" t="n"/>
-      <c r="H83" s="13" t="inlineStr">
-        <is>
-          <t>Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
-        </is>
-      </c>
+      <c r="H83" s="13" t="n"/>
       <c r="O83" s="13" t="n"/>
     </row>
     <row r="84" ht="15.75" customHeight="1" s="15">
@@ -2398,22 +2254,10 @@
           <t>Jak je dům dispozičně řešený?</t>
         </is>
       </c>
-      <c r="E88" s="13" t="inlineStr">
-        <is>
-          <t>Projektová dokumentace uvádí vytápěnou užitnou plochu 112,9 m², nevytápěnou 53,8 m² a celkovou užitnou plochu 166,7 m².</t>
-        </is>
-      </c>
-      <c r="F88" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E88" s="13" t="n"/>
+      <c r="F88" s="11" t="n"/>
       <c r="G88" s="13" t="n"/>
-      <c r="H88" s="13" t="inlineStr">
-        <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 14–15</t>
-        </is>
-      </c>
+      <c r="H88" s="13" t="n"/>
       <c r="O88" s="13" t="n"/>
     </row>
     <row r="89" ht="15.75" customHeight="1" s="15">
@@ -2574,22 +2418,10 @@
           <t>Kde je umístěná technická místnost?</t>
         </is>
       </c>
-      <c r="E96" s="13" t="inlineStr">
-        <is>
-          <t>V technické místnosti je v nice boiler, vzadu pod stropem technologická jednotka a před nimi prostor pro rozvaděč.</t>
-        </is>
-      </c>
-      <c r="F96" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E96" s="13" t="n"/>
+      <c r="F96" s="11" t="n"/>
       <c r="G96" s="13" t="n"/>
-      <c r="H96" s="13" t="inlineStr">
-        <is>
-          <t>Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
-        </is>
-      </c>
+      <c r="H96" s="13" t="n"/>
       <c r="O96" s="13" t="n"/>
     </row>
     <row r="97" ht="15.75" customHeight="1" s="15">
@@ -2605,22 +2437,10 @@
           <t>Je z obytného prostoru přímý vstup na terasu?</t>
         </is>
       </c>
-      <c r="E97" s="13" t="inlineStr">
-        <is>
-          <t>Terasa přímo navazuje na hlavní obytný prostor; velké prosklení a přímý vstup vytvářejí intenzivní propojení interiéru se zahradou.</t>
-        </is>
-      </c>
-      <c r="F97" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E97" s="13" t="n"/>
+      <c r="F97" s="11" t="n"/>
       <c r="G97" s="13" t="n"/>
-      <c r="H97" s="13" t="inlineStr">
-        <is>
-          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
-        </is>
-      </c>
+      <c r="H97" s="13" t="n"/>
       <c r="O97" s="13" t="n"/>
     </row>
     <row r="98" ht="15.75" customHeight="1" s="15">
@@ -2655,22 +2475,10 @@
           <t>Lze některý z pokojů využít jako pracovnu?</t>
         </is>
       </c>
-      <c r="E99" s="13" t="inlineStr">
-        <is>
-          <t>Ano. V zádveří je dostatek prostoru pro běžný provoz rodiny.</t>
-        </is>
-      </c>
-      <c r="F99" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E99" s="13" t="n"/>
+      <c r="F99" s="11" t="n"/>
       <c r="G99" s="13" t="n"/>
-      <c r="H99" s="13" t="inlineStr">
-        <is>
-          <t>E-book Jak se staví Domy s energií / KOMPLET / Validace autora domu / CURRENT / 2026-09-09</t>
-        </is>
-      </c>
+      <c r="H99" s="13" t="n"/>
       <c r="O99" s="13" t="n"/>
     </row>
     <row r="100" ht="15.75" customHeight="1" s="15">
@@ -2905,22 +2713,10 @@
           <t>Dá se změnit barva střechy?</t>
         </is>
       </c>
-      <c r="E111" s="13" t="inlineStr">
-        <is>
-          <t>Aktuální referenční provedení má střechu v antracitovém odstínu. Dostupné podklady ale samostatně nepotvrzují, zda lze u tohoto domu v rámci objednávky zvolit jinou barvu střechy.</t>
-        </is>
-      </c>
-      <c r="F111" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E111" s="13" t="n"/>
+      <c r="F111" s="11" t="n"/>
       <c r="G111" s="13" t="n"/>
-      <c r="H111" s="13" t="inlineStr">
-        <is>
-          <t>Validace autora domu / CURRENT / 2026-09-10</t>
-        </is>
-      </c>
+      <c r="H111" s="13" t="n"/>
       <c r="O111" s="13" t="n"/>
     </row>
     <row r="112" ht="15.75" customHeight="1" s="15">
@@ -2936,22 +2732,10 @@
           <t>Jaké materiály jsou použité na fasádě?</t>
         </is>
       </c>
-      <c r="E112" s="13" t="inlineStr">
-        <is>
-          <t>Vnější plášť je navržen z BRATEX CLICK – lakovaného pozinkovaného falcovaného plechu v antracitovém odstínu.</t>
-        </is>
-      </c>
-      <c r="F112" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E112" s="13" t="n"/>
+      <c r="F112" s="11" t="n"/>
       <c r="G112" s="13" t="n"/>
-      <c r="H112" s="13" t="inlineStr">
-        <is>
-          <t>B Souhrnná technická zpráva 11/2023, str. 18 a 22</t>
-        </is>
-      </c>
+      <c r="H112" s="13" t="n"/>
       <c r="O112" s="13" t="n"/>
     </row>
     <row r="113" ht="15.75" customHeight="1" s="15">
@@ -3395,22 +3179,10 @@
           <t>Je možné dům zrcadlově otočit?</t>
         </is>
       </c>
-      <c r="E135" s="13" t="inlineStr">
-        <is>
-          <t>Referenční pozemek je mírně svažitý a klesá směrem k jihovýchodu; při dokončovacích pracích se počítá s terénními úpravami a násypem.</t>
-        </is>
-      </c>
-      <c r="F135" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E135" s="13" t="n"/>
+      <c r="F135" s="11" t="n"/>
       <c r="G135" s="13" t="n"/>
-      <c r="H135" s="13" t="inlineStr">
-        <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / B Souhrnná technická zpráva 11/2023, str. 1 a 26 / Studie Bungalov 4KK / 01.11.2022</t>
-        </is>
-      </c>
+      <c r="H135" s="13" t="n"/>
       <c r="O135" s="13" t="n"/>
     </row>
     <row r="136" ht="15.75" customHeight="1" s="15">
@@ -3426,22 +3198,10 @@
           <t>Dá se jeden z pokojů využít jako pracovna?</t>
         </is>
       </c>
-      <c r="E136" s="13" t="inlineStr">
-        <is>
-          <t>Ano. V zádveří je dostatek prostoru pro běžný provoz rodiny.</t>
-        </is>
-      </c>
-      <c r="F136" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E136" s="13" t="n"/>
+      <c r="F136" s="11" t="n"/>
       <c r="G136" s="13" t="n"/>
-      <c r="H136" s="13" t="inlineStr">
-        <is>
-          <t>E-book Jak se staví Domy s energií / KOMPLET / Validace autora domu / CURRENT / 2026-09-09</t>
-        </is>
-      </c>
+      <c r="H136" s="13" t="n"/>
       <c r="O136" s="13" t="n"/>
     </row>
     <row r="137" ht="15.75" customHeight="1" s="15">
@@ -3495,22 +3255,10 @@
           <t>Je možné později přidat garáž nebo přístřešek?</t>
         </is>
       </c>
-      <c r="E139" s="13" t="inlineStr">
-        <is>
-          <t>Klientské změny doplnily dvě zásuvky v obývacím pokoji a tři zásuvky v exteriéru.</t>
-        </is>
-      </c>
-      <c r="F139" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E139" s="13" t="n"/>
+      <c r="F139" s="11" t="n"/>
       <c r="G139" s="13" t="n"/>
-      <c r="H139" s="13" t="inlineStr">
-        <is>
-          <t>Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
-        </is>
-      </c>
+      <c r="H139" s="13" t="n"/>
       <c r="O139" s="13" t="n"/>
     </row>
     <row r="140" ht="15.75" customHeight="1" s="15">
@@ -4641,22 +4389,10 @@
           <t>Je potřeba radonový průzkum nebo měření?</t>
         </is>
       </c>
-      <c r="E199" s="13" t="inlineStr">
-        <is>
-          <t>Dům je staticky posouzen na zatížení větrem pro II. větrnou zónu a II. kategorii terénu. Stabilitu proti bočnímu tlaku větru zajišťují ztužující stěny a křížové zavětrování ocelovými táhly.</t>
-        </is>
-      </c>
-      <c r="F199" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E199" s="13" t="n"/>
+      <c r="F199" s="11" t="n"/>
       <c r="G199" s="13" t="n"/>
-      <c r="H199" s="13" t="inlineStr">
-        <is>
-          <t>Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
-        </is>
-      </c>
+      <c r="H199" s="13" t="n"/>
       <c r="O199" s="13" t="n"/>
     </row>
     <row r="200" ht="15.75" customHeight="1" s="15">
@@ -4897,22 +4633,10 @@
           <t>Jak se řeší drenáže a voda kolem domu?</t>
         </is>
       </c>
-      <c r="E210" s="13" t="inlineStr">
-        <is>
-          <t>Dešťová voda ze střechy je odváděna do retenčního systému a přebytek je zasakován. Konkrétní potřeba drenáže kolem domu závisí na podmínkách pozemku.</t>
-        </is>
-      </c>
-      <c r="F210" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E210" s="13" t="n"/>
+      <c r="F210" s="11" t="n"/>
       <c r="G210" s="13" t="n"/>
-      <c r="H210" s="13" t="inlineStr">
-        <is>
-          <t>B Souhrnná technická zpráva 11/2023, str. 18 a 30–31</t>
-        </is>
-      </c>
+      <c r="H210" s="13" t="n"/>
       <c r="O210" s="13" t="n"/>
     </row>
     <row r="211" ht="15.75" customHeight="1" s="15">
@@ -5992,22 +5716,10 @@
           <t>Jak silné jsou obvodové stěny?</t>
         </is>
       </c>
-      <c r="E257" s="13" t="inlineStr">
-        <is>
-          <t>Koncepční skladba obvodového pláště je: sádrová omítka, Ekopanel, tepelná izolace Climatizer Plus mezi rámy, difuzní fólie, kontralatě, kotvící latě, odvětrávaná mezera a fasádní prvek.</t>
-        </is>
-      </c>
-      <c r="F257" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E257" s="13" t="n"/>
+      <c r="F257" s="11" t="n"/>
       <c r="G257" s="13" t="n"/>
-      <c r="H257" s="13" t="inlineStr">
-        <is>
-          <t>E-book Jak se staví Domy s energií / KOMPLET</t>
-        </is>
-      </c>
+      <c r="H257" s="13" t="n"/>
       <c r="O257" s="13" t="n"/>
     </row>
     <row r="258" ht="15.75" customHeight="1" s="15">
@@ -6023,22 +5735,10 @@
           <t>Z jakých vrstev se obvodová stěna skládá?</t>
         </is>
       </c>
-      <c r="E258" s="13" t="inlineStr">
-        <is>
-          <t>Koncepční skladba obvodového pláště je: sádrová omítka, Ekopanel, tepelná izolace Climatizer Plus mezi rámy, difuzní fólie, kontralatě, kotvící latě, odvětrávaná mezera a fasádní prvek.</t>
-        </is>
-      </c>
-      <c r="F258" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E258" s="13" t="n"/>
+      <c r="F258" s="11" t="n"/>
       <c r="G258" s="13" t="n"/>
-      <c r="H258" s="13" t="inlineStr">
-        <is>
-          <t>E-book Jak se staví Domy s energií / KOMPLET</t>
-        </is>
-      </c>
+      <c r="H258" s="13" t="n"/>
       <c r="O258" s="13" t="n"/>
     </row>
     <row r="259" ht="15.75" customHeight="1" s="15">
@@ -6054,22 +5754,10 @@
           <t>Z čeho jsou vnitřní nosné stěny?</t>
         </is>
       </c>
-      <c r="E259" s="13" t="inlineStr">
-        <is>
-          <t>Ano. Bungalov 4KK je rámová difuzně otevřená dřevostavba.</t>
-        </is>
-      </c>
-      <c r="F259" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E259" s="13" t="n"/>
+      <c r="F259" s="11" t="n"/>
       <c r="G259" s="13" t="n"/>
-      <c r="H259" s="13" t="inlineStr">
-        <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
-        </is>
-      </c>
+      <c r="H259" s="13" t="n"/>
       <c r="O259" s="13" t="n"/>
     </row>
     <row r="260" ht="15.75" customHeight="1" s="15">
@@ -6147,22 +5835,10 @@
           <t>Jak je řešená konstrukce podlahy?</t>
         </is>
       </c>
-      <c r="E262" s="13" t="inlineStr">
-        <is>
-          <t>Nosnou konstrukci střechy tvoří soustava dřevěných rámů z jehličnatých KVH hranolů pevnostní třídy C24.</t>
-        </is>
-      </c>
-      <c r="F262" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E262" s="13" t="n"/>
+      <c r="F262" s="11" t="n"/>
       <c r="G262" s="13" t="n"/>
-      <c r="H262" s="13" t="inlineStr">
-        <is>
-          <t>B Souhrnná technická zpráva 11/2023, str. 22</t>
-        </is>
-      </c>
+      <c r="H262" s="13" t="n"/>
       <c r="O262" s="13" t="n"/>
     </row>
     <row r="263" ht="15.75" customHeight="1" s="15">
@@ -6482,22 +6158,10 @@
           <t>V čem se tento konstrukční systém liší od klasického zděného domu?</t>
         </is>
       </c>
-      <c r="E275" s="13" t="inlineStr">
-        <is>
-          <t>Dům je řešen jako rámová difuzně otevřená dřevostavba s vnitřní vestavbou z Ekopanelu, výplň tvoří celulóza Climatizer plus, z vnější strany opatřeno difůzní fólií a odvětrávanou fasádou.</t>
-        </is>
-      </c>
-      <c r="F275" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E275" s="13" t="n"/>
+      <c r="F275" s="11" t="n"/>
       <c r="G275" s="13" t="n"/>
-      <c r="H275" s="13" t="inlineStr">
-        <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
-        </is>
-      </c>
+      <c r="H275" s="13" t="n"/>
       <c r="O275" s="13" t="n"/>
     </row>
     <row r="276" ht="15.75" customHeight="1" s="15">
@@ -6561,22 +6225,10 @@
           <t>Jakou barvu má střecha?</t>
         </is>
       </c>
-      <c r="E278" s="13" t="inlineStr">
-        <is>
-          <t>Střecha je v antracitovém odstínu.</t>
-        </is>
-      </c>
-      <c r="F278" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E278" s="13" t="n"/>
+      <c r="F278" s="11" t="n"/>
       <c r="G278" s="13" t="n"/>
-      <c r="H278" s="13" t="inlineStr">
-        <is>
-          <t>Validace autora domu / CURRENT / 2026-09-10</t>
-        </is>
-      </c>
+      <c r="H278" s="13" t="n"/>
       <c r="O278" s="13" t="n"/>
     </row>
     <row r="279" ht="15.75" customHeight="1" s="15">
@@ -6673,22 +6325,10 @@
           <t>Jaká je životnost střešní krytiny?</t>
         </is>
       </c>
-      <c r="E282" s="13" t="inlineStr">
-        <is>
-          <t>60 let a více.</t>
-        </is>
-      </c>
-      <c r="F282" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E282" s="13" t="n"/>
+      <c r="F282" s="11" t="n"/>
       <c r="G282" s="13" t="n"/>
-      <c r="H282" s="13" t="inlineStr">
-        <is>
-          <t>Knowledge projection / 31.5</t>
-        </is>
-      </c>
+      <c r="H282" s="13" t="n"/>
       <c r="O282" s="13" t="n"/>
     </row>
     <row r="283" ht="15.75" customHeight="1" s="15">
@@ -6704,22 +6344,10 @@
           <t>Jakou údržbu střecha potřebuje?</t>
         </is>
       </c>
-      <c r="E283" s="13" t="inlineStr">
-        <is>
-          <t>Téměř žádnou, vyjma údržby dřevěných částí v exteriéru v intervalu 6-10 let.</t>
-        </is>
-      </c>
-      <c r="F283" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E283" s="13" t="n"/>
+      <c r="F283" s="11" t="n"/>
       <c r="G283" s="13" t="n"/>
-      <c r="H283" s="13" t="inlineStr">
-        <is>
-          <t>Knowledge projection / 31.2</t>
-        </is>
-      </c>
+      <c r="H283" s="13" t="n"/>
       <c r="O283" s="13" t="n"/>
     </row>
     <row r="284" ht="15.75" customHeight="1" s="15">
@@ -6735,22 +6363,10 @@
           <t>Jakou údržbu potřebuje fasáda?</t>
         </is>
       </c>
-      <c r="E284" s="13" t="inlineStr">
-        <is>
-          <t>Pouze ošetření dřevěných částí v intervalu 6-10 let.</t>
-        </is>
-      </c>
-      <c r="F284" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E284" s="13" t="n"/>
+      <c r="F284" s="11" t="n"/>
       <c r="G284" s="13" t="n"/>
-      <c r="H284" s="13" t="inlineStr">
-        <is>
-          <t>Knowledge projection / 31.6</t>
-        </is>
-      </c>
+      <c r="H284" s="13" t="n"/>
       <c r="O284" s="13" t="n"/>
     </row>
     <row r="285" ht="15.75" customHeight="1" s="15">
@@ -6816,22 +6432,10 @@
           <t>Lze na fasádě použít dřevo nebo jiný obklad?</t>
         </is>
       </c>
-      <c r="E287" s="13" t="inlineStr">
-        <is>
-          <t>Dřevěné obklady a nosné konstrukce přístřešků – tyto je nutné vždy ošetřit v intervalu 6-10 let.</t>
-        </is>
-      </c>
-      <c r="F287" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E287" s="13" t="n"/>
+      <c r="F287" s="11" t="n"/>
       <c r="G287" s="13" t="n"/>
-      <c r="H287" s="13" t="inlineStr">
-        <is>
-          <t>Knowledge projection / 13.19</t>
-        </is>
-      </c>
+      <c r="H287" s="13" t="n"/>
       <c r="O287" s="13" t="n"/>
     </row>
     <row r="288" ht="15.75" customHeight="1" s="15">
@@ -7090,22 +6694,10 @@
           <t>Jaké jsou hlavní důvody pro volbu právě těchto materiálů střechy a fasády?</t>
         </is>
       </c>
-      <c r="E296" s="13" t="inlineStr">
-        <is>
-          <t>Použitý vnější plášť pracuje s lakovaným pozinkovaným plechem BRATEX CLICK; dostupné podklady popisují materiálové řešení, nikoli samostatné autorské zdůvodnění všech důvodů jeho volby.</t>
-        </is>
-      </c>
-      <c r="F296" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E296" s="13" t="n"/>
+      <c r="F296" s="11" t="n"/>
       <c r="G296" s="13" t="n"/>
-      <c r="H296" s="13" t="inlineStr">
-        <is>
-          <t>B Souhrnná technická zpráva 11/2023, str. 18 a 22</t>
-        </is>
-      </c>
+      <c r="H296" s="13" t="n"/>
       <c r="O296" s="13" t="n"/>
     </row>
     <row r="297" ht="15.75" customHeight="1" s="15">
@@ -7417,22 +7009,10 @@
           <t>Jak jsou řešené dveře z obývacího prostoru na terasu?</t>
         </is>
       </c>
-      <c r="E307" s="13" t="inlineStr">
-        <is>
-          <t>Obytný prostor je propojen s terasou dveřmi; CURRENT validace zároveň potvrzuje, že terasové dveře nejsou řešeny jako posuvné.</t>
-        </is>
-      </c>
-      <c r="F307" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E307" s="13" t="n"/>
+      <c r="F307" s="11" t="n"/>
       <c r="G307" s="13" t="n"/>
-      <c r="H307" s="13" t="inlineStr">
-        <is>
-          <t>E-book Jak se staví Domy s energií / KOMPLET / Validace autora domu / CURRENT / 2026-09-09</t>
-        </is>
-      </c>
+      <c r="H307" s="13" t="n"/>
       <c r="O307" s="13" t="n"/>
     </row>
     <row r="308" ht="15.75" customHeight="1" s="15">
@@ -7617,22 +7197,10 @@
           <t>Jak dobře okna tlumí hluk zvenčí?</t>
         </is>
       </c>
-      <c r="E315" s="13" t="inlineStr">
-        <is>
-          <t>Výborně, plastnová okna s troskly jsou špičkou v dané kategorii.</t>
-        </is>
-      </c>
-      <c r="F315" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E315" s="13" t="n"/>
+      <c r="F315" s="11" t="n"/>
       <c r="G315" s="13" t="n"/>
-      <c r="H315" s="13" t="inlineStr">
-        <is>
-          <t>Knowledge projection / 29.7</t>
-        </is>
-      </c>
+      <c r="H315" s="13" t="n"/>
       <c r="O315" s="13" t="n"/>
     </row>
     <row r="316" ht="15.75" customHeight="1" s="15">
@@ -7734,22 +7302,10 @@
           <t>Nebude v domě v létě příliš horko?</t>
         </is>
       </c>
-      <c r="E320" s="13" t="inlineStr">
-        <is>
-          <t>Dům používá venkovní stínění a rekuperační jednotka umožňuje v létě chlazení. Tyto prvky omezují riziko letního přehřívání; konkrétní maximální vnitřní teplotu dostupné podklady neuvádějí.</t>
-        </is>
-      </c>
-      <c r="F320" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E320" s="13" t="n"/>
+      <c r="F320" s="11" t="n"/>
       <c r="G320" s="13" t="n"/>
-      <c r="H320" s="13" t="inlineStr">
-        <is>
-          <t>PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
-        </is>
-      </c>
+      <c r="H320" s="13" t="n"/>
       <c r="O320" s="13" t="n"/>
     </row>
     <row r="321" ht="15.75" customHeight="1" s="15">
@@ -7796,22 +7352,10 @@
           <t>Jak dům chrání interiér před přehříváním?</t>
         </is>
       </c>
-      <c r="E322" s="13" t="inlineStr">
-        <is>
-          <t>Okna mají izolační trojskla a dům používá venkovní roletové žaluzie, které umožňují omezit přímé sluneční záření před zasklením. Konkrétní snížení letní vnitřní teploty dostupné podklady nevyčíslují.</t>
-        </is>
-      </c>
-      <c r="F322" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E322" s="13" t="n"/>
+      <c r="F322" s="11" t="n"/>
       <c r="G322" s="13" t="n"/>
-      <c r="H322" s="13" t="inlineStr">
-        <is>
-          <t>PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023 / Validace autora domu / CURRENT / 2026-09-10</t>
-        </is>
-      </c>
+      <c r="H322" s="13" t="n"/>
       <c r="O322" s="13" t="n"/>
     </row>
     <row r="323" ht="15.75" customHeight="1" s="15">
@@ -8597,22 +8141,10 @@
           <t>Jak je řešená ochrana elektroinstalace proti poruchám?</t>
         </is>
       </c>
-      <c r="E351" s="13" t="inlineStr">
-        <is>
-          <t>Bezpečný stav elektroinstalace se dokládá příslušnou revizí; konkrétní ochranné prvky musí odpovídat projektové dokumentaci a příslušným předpisům.</t>
-        </is>
-      </c>
-      <c r="F351" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E351" s="13" t="n"/>
+      <c r="F351" s="11" t="n"/>
       <c r="G351" s="13" t="n"/>
-      <c r="H351" s="13" t="inlineStr">
-        <is>
-          <t>B Souhrnná technická zpráva 11/2023</t>
-        </is>
-      </c>
+      <c r="H351" s="13" t="n"/>
       <c r="O351" s="13" t="n"/>
     </row>
     <row r="352" ht="15.75" customHeight="1" s="15">
@@ -9217,22 +8749,10 @@
           <t>Kudy jsou technické rozvody v konstrukci vedené?</t>
         </is>
       </c>
-      <c r="E375" s="13" t="inlineStr">
-        <is>
-          <t>Technické rozvody jsou provedeny podle projektové dokumentace. Přesné trasy jednotlivých vedení je nutné určovat podle dokumentace skutečného provedení a konkrétní realizace.</t>
-        </is>
-      </c>
-      <c r="F375" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E375" s="13" t="n"/>
+      <c r="F375" s="11" t="n"/>
       <c r="G375" s="13" t="n"/>
-      <c r="H375" s="13" t="inlineStr">
-        <is>
-          <t>B Souhrnná technická zpráva 11/2023</t>
-        </is>
-      </c>
+      <c r="H375" s="13" t="n"/>
       <c r="O375" s="13" t="n"/>
     </row>
     <row r="376" ht="15.75" customHeight="1" s="15">
@@ -9775,22 +9295,10 @@
           <t>Jak hlučné jsou technologie domu?</t>
         </is>
       </c>
-      <c r="E395" s="13" t="inlineStr">
-        <is>
-          <t>Dům používá technická zařízení včetně řízeného větrání. Dostupné podklady ale neobsahují jednotné naměřené hodnoty hlučnosti všech technologií v dokončeném domě.</t>
-        </is>
-      </c>
-      <c r="F395" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E395" s="13" t="n"/>
+      <c r="F395" s="11" t="n"/>
       <c r="G395" s="13" t="n"/>
-      <c r="H395" s="13" t="inlineStr">
-        <is>
-          <t>Validace autora domu / CURRENT / 2026-09-09</t>
-        </is>
-      </c>
+      <c r="H395" s="13" t="n"/>
       <c r="O395" s="13" t="n"/>
     </row>
     <row r="396" ht="15.75" customHeight="1" s="15">
@@ -9864,22 +9372,10 @@
           <t>Jak často je potřeba technologie servisovat?</t>
         </is>
       </c>
-      <c r="E398" s="13" t="inlineStr">
-        <is>
-          <t>Servisní intervaly technologií nejsou pro všechny prvky domu v dostupných podkladech jednotně stanoveny. Řídí se dokumentací a servisními požadavky konkrétních výrobců jednotlivých zařízení.</t>
-        </is>
-      </c>
-      <c r="F398" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E398" s="13" t="n"/>
+      <c r="F398" s="11" t="n"/>
       <c r="G398" s="13" t="n"/>
-      <c r="H398" s="13" t="inlineStr">
-        <is>
-          <t>B Souhrnná technická zpráva 11/2023</t>
-        </is>
-      </c>
+      <c r="H398" s="13" t="n"/>
       <c r="O398" s="13" t="n"/>
     </row>
     <row r="399" ht="15.75" customHeight="1" s="15">
@@ -10113,22 +9609,10 @@
           <t>Je podlaha vhodná pro podlahové vytápění?</t>
         </is>
       </c>
-      <c r="E410" s="13" t="inlineStr">
-        <is>
-          <t>Aktuální konfigurace používá elektrické topné fólie pod dřevěnou podlahou, takže použitá podlahová skladba s tímto způsobem vytápění počítá.</t>
-        </is>
-      </c>
-      <c r="F410" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E410" s="13" t="n"/>
+      <c r="F410" s="11" t="n"/>
       <c r="G410" s="13" t="n"/>
-      <c r="H410" s="13" t="inlineStr">
-        <is>
-          <t>B Souhrnná technická zpráva 11/2023, str. 24 / Klientské změny č. 2 / Bungalov 4KK / 20.10.2023 / B Souhrnná technická zpráva 11/2023</t>
-        </is>
-      </c>
+      <c r="H410" s="13" t="n"/>
       <c r="O410" s="13" t="n"/>
     </row>
     <row r="411" ht="15.75" customHeight="1" s="15">
@@ -10401,22 +9885,10 @@
           <t>Jak velký je obývací pokoj s kuchyní?</t>
         </is>
       </c>
-      <c r="E424" s="13" t="inlineStr">
-        <is>
-          <t>Ano. Z hlavního obytného prostoru je přímý vstup na terasu a zahradu.</t>
-        </is>
-      </c>
-      <c r="F424" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E424" s="13" t="n"/>
+      <c r="F424" s="11" t="n"/>
       <c r="G424" s="13" t="n"/>
-      <c r="H424" s="13" t="inlineStr">
-        <is>
-          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
-        </is>
-      </c>
+      <c r="H424" s="13" t="n"/>
       <c r="O424" s="13" t="n"/>
     </row>
     <row r="425" ht="15.75" customHeight="1" s="15">
@@ -10558,22 +10030,10 @@
           <t>Jak je obytný prostor propojený se zahradou?</t>
         </is>
       </c>
-      <c r="E431" s="13" t="inlineStr">
-        <is>
-          <t>Terasa přímo navazuje na hlavní obytný prostor; velké prosklení a přímý vstup vytvářejí intenzivní propojení interiéru se zahradou.</t>
-        </is>
-      </c>
-      <c r="F431" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E431" s="13" t="n"/>
+      <c r="F431" s="11" t="n"/>
       <c r="G431" s="13" t="n"/>
-      <c r="H431" s="13" t="inlineStr">
-        <is>
-          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
-        </is>
-      </c>
+      <c r="H431" s="13" t="n"/>
       <c r="O431" s="13" t="n"/>
     </row>
     <row r="432" ht="15.75" customHeight="1" s="15">
@@ -10741,22 +10201,10 @@
           <t>Jak je v obývacím prostoru řešené stínění velkých oken?</t>
         </is>
       </c>
-      <c r="E440" s="13" t="inlineStr">
-        <is>
-          <t>Venkovní stínění je řešeno roletovými žaluziemi.</t>
-        </is>
-      </c>
-      <c r="F440" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E440" s="13" t="n"/>
+      <c r="F440" s="11" t="n"/>
       <c r="G440" s="13" t="n"/>
-      <c r="H440" s="13" t="inlineStr">
-        <is>
-          <t>Validace autora domu / CURRENT / 2026-09-10</t>
-        </is>
-      </c>
+      <c r="H440" s="13" t="n"/>
       <c r="O440" s="13" t="n"/>
     </row>
     <row r="441" ht="15.75" customHeight="1" s="15">
@@ -10772,22 +10220,10 @@
           <t>Nebude se obytný prostor kvůli velkému prosklení v létě přehřívat?</t>
         </is>
       </c>
-      <c r="E441" s="13" t="inlineStr">
-        <is>
-          <t>Dům používá venkovní stínění a rekuperační jednotka umožňuje v létě chlazení. Tyto prvky omezují riziko letního přehřívání; konkrétní maximální vnitřní teplotu dostupné podklady neuvádějí.</t>
-        </is>
-      </c>
-      <c r="F441" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E441" s="13" t="n"/>
+      <c r="F441" s="11" t="n"/>
       <c r="G441" s="13" t="n"/>
-      <c r="H441" s="13" t="inlineStr">
-        <is>
-          <t>PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
-        </is>
-      </c>
+      <c r="H441" s="13" t="n"/>
       <c r="O441" s="13" t="n"/>
     </row>
     <row r="442" ht="15.75" customHeight="1" s="15">
@@ -11193,22 +10629,10 @@
           <t>Je z kuchyně dobře dostupná terasa pro venkovní stolování?</t>
         </is>
       </c>
-      <c r="E462" s="13" t="inlineStr">
-        <is>
-          <t>Terasa přímo navazuje na hlavní obytný prostor; velké prosklení a přímý vstup vytvářejí intenzivní propojení interiéru se zahradou.</t>
-        </is>
-      </c>
-      <c r="F462" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E462" s="13" t="n"/>
+      <c r="F462" s="11" t="n"/>
       <c r="G462" s="13" t="n"/>
-      <c r="H462" s="13" t="inlineStr">
-        <is>
-          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
-        </is>
-      </c>
+      <c r="H462" s="13" t="n"/>
       <c r="O462" s="13" t="n"/>
     </row>
     <row r="463" ht="15.75" customHeight="1" s="15">
@@ -11279,22 +10703,10 @@
           <t>Jak velká je hlavní ložnice?</t>
         </is>
       </c>
-      <c r="E466" s="13" t="inlineStr">
-        <is>
-          <t>Ano. U ložnice je řešena integrovaná šatna bez sníženého podhledu.</t>
-        </is>
-      </c>
-      <c r="F466" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E466" s="13" t="n"/>
+      <c r="F466" s="11" t="n"/>
       <c r="G466" s="13" t="n"/>
-      <c r="H466" s="13" t="inlineStr">
-        <is>
-          <t>Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
-        </is>
-      </c>
+      <c r="H466" s="13" t="n"/>
       <c r="O466" s="13" t="n"/>
     </row>
     <row r="467" ht="15.75" customHeight="1" s="15">
@@ -11310,22 +10722,10 @@
           <t>Jak velké jsou dětské pokoje?</t>
         </is>
       </c>
-      <c r="E467" s="13" t="inlineStr">
-        <is>
-          <t>Ano. Jeden z pokojů je koncipován flexibilně pro využití jako dětský pokoj nebo pracovna.</t>
-        </is>
-      </c>
-      <c r="F467" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E467" s="13" t="n"/>
+      <c r="F467" s="11" t="n"/>
       <c r="G467" s="13" t="n"/>
-      <c r="H467" s="13" t="inlineStr">
-        <is>
-          <t>Studie Bungalov 4KK / 01.11.2022</t>
-        </is>
-      </c>
+      <c r="H467" s="13" t="n"/>
       <c r="O467" s="13" t="n"/>
     </row>
     <row r="468" ht="15.75" customHeight="1" s="15">
@@ -11631,22 +11031,10 @@
           <t>Jak se pokoje větrají a jak se v nich reguluje teplota?</t>
         </is>
       </c>
-      <c r="E482" s="13" t="inlineStr">
-        <is>
-          <t>Pokoje jsou větrány systémem nuceného řízeného větrání s rekuperací. Přesný způsob individuální regulace teploty v každém pokoji dostupné podklady samostatně nepotvrzují.</t>
-        </is>
-      </c>
-      <c r="F482" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E482" s="13" t="n"/>
+      <c r="F482" s="11" t="n"/>
       <c r="G482" s="13" t="n"/>
-      <c r="H482" s="13" t="inlineStr">
-        <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
-        </is>
-      </c>
+      <c r="H482" s="13" t="n"/>
       <c r="O482" s="13" t="n"/>
     </row>
     <row r="483" ht="15.75" customHeight="1" s="15">
@@ -11662,22 +11050,10 @@
           <t>Lze pokoje zatemnit pro pohodlné spaní?</t>
         </is>
       </c>
-      <c r="E483" s="13" t="inlineStr">
-        <is>
-          <t>Ano. Dům používá venkovní roletové žaluzie, které lze využít také pro omezení světla v pokojích.</t>
-        </is>
-      </c>
-      <c r="F483" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E483" s="13" t="n"/>
+      <c r="F483" s="11" t="n"/>
       <c r="G483" s="13" t="n"/>
-      <c r="H483" s="13" t="inlineStr">
-        <is>
-          <t>Validace autora domu / CURRENT / 2026-09-10</t>
-        </is>
-      </c>
+      <c r="H483" s="13" t="n"/>
       <c r="O483" s="13" t="n"/>
     </row>
     <row r="484" ht="15.75" customHeight="1" s="15">
@@ -11957,22 +11333,10 @@
           <t>Jak je koupelna větraná?</t>
         </is>
       </c>
-      <c r="E498" s="13" t="inlineStr">
-        <is>
-          <t>Dům využívá řízené větrání s rekuperací tepla.</t>
-        </is>
-      </c>
-      <c r="F498" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E498" s="13" t="n"/>
+      <c r="F498" s="11" t="n"/>
       <c r="G498" s="13" t="n"/>
-      <c r="H498" s="13" t="inlineStr">
-        <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
-        </is>
-      </c>
+      <c r="H498" s="13" t="n"/>
       <c r="O498" s="13" t="n"/>
     </row>
     <row r="499" ht="15.75" customHeight="1" s="15">
@@ -12321,22 +11685,10 @@
           <t>Jak velká je technická místnost?</t>
         </is>
       </c>
-      <c r="E516" s="13" t="inlineStr">
-        <is>
-          <t>V technické místnosti je v nice boiler, vzadu pod stropem technologická jednotka a před nimi prostor pro rozvaděč.</t>
-        </is>
-      </c>
-      <c r="F516" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E516" s="13" t="n"/>
+      <c r="F516" s="11" t="n"/>
       <c r="G516" s="13" t="n"/>
-      <c r="H516" s="13" t="inlineStr">
-        <is>
-          <t>Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
-        </is>
-      </c>
+      <c r="H516" s="13" t="n"/>
       <c r="O516" s="13" t="n"/>
     </row>
     <row r="517" ht="15.75" customHeight="1" s="15">
@@ -12383,22 +11735,10 @@
           <t>Je v technické místnosti místo pro pračku a sušičku?</t>
         </is>
       </c>
-      <c r="E518" s="13" t="inlineStr">
-        <is>
-          <t>Technická místnost soustřeďuje technické zázemí domu. Dostupné podklady ale samostatně nepotvrzují konkrétní finální umístění pračky a sušičky.</t>
-        </is>
-      </c>
-      <c r="F518" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E518" s="13" t="n"/>
+      <c r="F518" s="11" t="n"/>
       <c r="G518" s="13" t="n"/>
-      <c r="H518" s="13" t="inlineStr">
-        <is>
-          <t>Klientské změny č. 2 / Bungalov 4KK / 20.10.2023</t>
-        </is>
-      </c>
+      <c r="H518" s="13" t="n"/>
       <c r="O518" s="13" t="n"/>
     </row>
     <row r="519" ht="15.75" customHeight="1" s="15">
@@ -13465,22 +12805,10 @@
           <t>Je z obývacího pokoje přímý výhled do zahrady?</t>
         </is>
       </c>
-      <c r="E574" s="13" t="inlineStr">
-        <is>
-          <t>Terasa přímo navazuje na hlavní obytný prostor; velké prosklení a přímý vstup vytvářejí intenzivní propojení interiéru se zahradou.</t>
-        </is>
-      </c>
-      <c r="F574" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E574" s="13" t="n"/>
+      <c r="F574" s="11" t="n"/>
       <c r="G574" s="13" t="n"/>
-      <c r="H574" s="13" t="inlineStr">
-        <is>
-          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
-        </is>
-      </c>
+      <c r="H574" s="13" t="n"/>
       <c r="O574" s="13" t="n"/>
     </row>
     <row r="575" ht="15.75" customHeight="1" s="15">
@@ -13496,22 +12824,10 @@
           <t>Jak je dům propojený se zahradou?</t>
         </is>
       </c>
-      <c r="E575" s="13" t="inlineStr">
-        <is>
-          <t>Terasa přímo navazuje na hlavní obytný prostor; velké prosklení a přímý vstup vytvářejí intenzivní propojení interiéru se zahradou.</t>
-        </is>
-      </c>
-      <c r="F575" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E575" s="13" t="n"/>
+      <c r="F575" s="11" t="n"/>
       <c r="G575" s="13" t="n"/>
-      <c r="H575" s="13" t="inlineStr">
-        <is>
-          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
-        </is>
-      </c>
+      <c r="H575" s="13" t="n"/>
       <c r="O575" s="13" t="n"/>
     </row>
     <row r="576" ht="15.75" customHeight="1" s="15">
@@ -13748,22 +13064,10 @@
           <t>Jak se řeší soukromí při velkém propojení interiéru se zahradou?</t>
         </is>
       </c>
-      <c r="E587" s="13" t="inlineStr">
-        <is>
-          <t>Soukromí u prosklených ploch lze podpořit venkovními roletovými žaluziemi.</t>
-        </is>
-      </c>
-      <c r="F587" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E587" s="13" t="n"/>
+      <c r="F587" s="11" t="n"/>
       <c r="G587" s="13" t="n"/>
-      <c r="H587" s="13" t="inlineStr">
-        <is>
-          <t>Validace autora domu / CURRENT / 2026-09-10</t>
-        </is>
-      </c>
+      <c r="H587" s="13" t="n"/>
       <c r="O587" s="13" t="n"/>
     </row>
     <row r="588" ht="15.75" customHeight="1" s="15">
@@ -13779,22 +13083,10 @@
           <t>Nezpůsobují velké prosklené plochy v létě přehřívání?</t>
         </is>
       </c>
-      <c r="E588" s="13" t="inlineStr">
-        <is>
-          <t>Dům používá venkovní stínění a rekuperační jednotka umožňuje v létě chlazení. Tyto prvky omezují riziko letního přehřívání; konkrétní maximální vnitřní teplotu dostupné podklady neuvádějí.</t>
-        </is>
-      </c>
-      <c r="F588" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E588" s="13" t="n"/>
+      <c r="F588" s="11" t="n"/>
       <c r="G588" s="13" t="n"/>
-      <c r="H588" s="13" t="inlineStr">
-        <is>
-          <t>PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
-        </is>
-      </c>
+      <c r="H588" s="13" t="n"/>
       <c r="O588" s="13" t="n"/>
     </row>
     <row r="589" ht="15.75" customHeight="1" s="15">
@@ -14015,22 +13307,10 @@
           <t>Je z kuchyně dobře dostupná terasa pro venkovní stolování?</t>
         </is>
       </c>
-      <c r="E598" s="13" t="inlineStr">
-        <is>
-          <t>Terasa přímo navazuje na hlavní obytný prostor; velké prosklení a přímý vstup vytvářejí intenzivní propojení interiéru se zahradou.</t>
-        </is>
-      </c>
-      <c r="F598" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E598" s="13" t="n"/>
+      <c r="F598" s="11" t="n"/>
       <c r="G598" s="13" t="n"/>
-      <c r="H598" s="13" t="inlineStr">
-        <is>
-          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
-        </is>
-      </c>
+      <c r="H598" s="13" t="n"/>
       <c r="O598" s="13" t="n"/>
     </row>
     <row r="599" ht="15.75" customHeight="1" s="15">
@@ -14096,22 +13376,10 @@
           <t>Jak dům funguje při častém přecházení mezi interiérem a zahradou?</t>
         </is>
       </c>
-      <c r="E601" s="13" t="inlineStr">
-        <is>
-          <t>Terasa přímo navazuje na hlavní obytný prostor; velké prosklení a přímý vstup vytvářejí intenzivní propojení interiéru se zahradou.</t>
-        </is>
-      </c>
-      <c r="F601" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E601" s="13" t="n"/>
+      <c r="F601" s="11" t="n"/>
       <c r="G601" s="13" t="n"/>
-      <c r="H601" s="13" t="inlineStr">
-        <is>
-          <t>Studie Bungalov 4KK / 01.11.2022 / E-book Jak se staví Domy s energií / KOMPLET</t>
-        </is>
-      </c>
+      <c r="H601" s="13" t="n"/>
       <c r="O601" s="13" t="n"/>
     </row>
     <row r="602" ht="15.75" customHeight="1" s="15">
@@ -14515,22 +13783,10 @@
           <t>Je v ložnici slyšet provoz technologií domu?</t>
         </is>
       </c>
-      <c r="E620" s="13" t="inlineStr">
-        <is>
-          <t>Dostupné podklady neobsahují konkrétní měření hluku technologií v ložnici, takže nelze bezpečně tvrdit, že jejich provoz není slyšet.</t>
-        </is>
-      </c>
-      <c r="F620" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E620" s="13" t="n"/>
+      <c r="F620" s="11" t="n"/>
       <c r="G620" s="13" t="n"/>
-      <c r="H620" s="13" t="inlineStr">
-        <is>
-          <t>Validace autora domu / CURRENT / 2026-09-09</t>
-        </is>
-      </c>
+      <c r="H620" s="13" t="n"/>
       <c r="O620" s="13" t="n"/>
     </row>
     <row r="621" ht="15.75" customHeight="1" s="15">
@@ -14646,22 +13902,10 @@
           <t>Je v dřevostavbě větší hluk než ve zděném domě?</t>
         </is>
       </c>
-      <c r="E625" s="13" t="inlineStr">
-        <is>
-          <t>Samotný konstrukční princip dřevostavby nestačí k obecnému tvrzení, že je dům hlučnější než zděný. Akustické chování je nutné hodnotit podle konkrétních skladeb a jejich parametrů.</t>
-        </is>
-      </c>
-      <c r="F625" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E625" s="13" t="n"/>
+      <c r="F625" s="11" t="n"/>
       <c r="G625" s="13" t="n"/>
-      <c r="H625" s="13" t="inlineStr">
-        <is>
-          <t>B Souhrnná technická zpráva 11/2023</t>
-        </is>
-      </c>
+      <c r="H625" s="13" t="n"/>
       <c r="O625" s="13" t="n"/>
     </row>
     <row r="626" ht="15.75" customHeight="1" s="15">
@@ -15057,22 +14301,10 @@
           <t>Jak spotřebu ovlivňuje rekuperace?</t>
         </is>
       </c>
-      <c r="E644" s="13" t="inlineStr">
-        <is>
-          <t>Rekuperace omezuje tepelné ztráty větráním tím, že využívá teplo odváděného vzduchu. Dostupné podklady ale samostatně nevyčíslují její podíl na celkové spotřebě tohoto domu.</t>
-        </is>
-      </c>
-      <c r="F644" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E644" s="13" t="n"/>
+      <c r="F644" s="11" t="n"/>
       <c r="G644" s="13" t="n"/>
-      <c r="H644" s="13" t="inlineStr">
-        <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
-        </is>
-      </c>
+      <c r="H644" s="13" t="n"/>
       <c r="O644" s="13" t="n"/>
     </row>
     <row r="645" ht="15.75" customHeight="1" s="15">
@@ -15781,22 +15013,10 @@
           <t>Co můžu dělat, aby dům vydržel co nejdéle v dobrém stavu?</t>
         </is>
       </c>
-      <c r="E674" s="13" t="inlineStr">
-        <is>
-          <t>Pro dlouhou životnost domu je důležité provádět běžnou údržbu, zejména pravidelně ošetřovat exponované dřevěné části a dodržovat servisní požadavky použitých technologií.</t>
-        </is>
-      </c>
-      <c r="F674" s="11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
+      <c r="E674" s="13" t="n"/>
+      <c r="F674" s="11" t="n"/>
       <c r="G674" s="13" t="n"/>
-      <c r="H674" s="13" t="inlineStr">
-        <is>
-          <t>Knowledge projection / 31.2</t>
-        </is>
-      </c>
+      <c r="H674" s="13" t="n"/>
       <c r="O674" s="13" t="n"/>
     </row>
     <row r="675" ht="15.75" customHeight="1" s="15">

</xml_diff>

<commit_message>
docs(knowledge): complete grounded Bungalov 4KK source harvest
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 02.xlsx
+++ b/docs/knowledge/znalostní báze – mustr 02.xlsx
@@ -633,10 +633,22 @@
           <t>Jaká byla hlavní myšlenka při návrhu tohoto domu?</t>
         </is>
       </c>
-      <c r="E8" s="13" t="n"/>
-      <c r="F8" s="11" t="n"/>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>Koncepce vychází z principu „bytu v zahradě“: úsporný půdorys, maximální důraz na funkčnost a silné propojení obytných místností se zahradou.</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G8" s="13" t="n"/>
-      <c r="H8" s="13" t="n"/>
+      <c r="H8" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O8" s="13" t="n"/>
     </row>
     <row r="9" ht="15.75" customHeight="1" s="15">
@@ -728,10 +740,22 @@
           <t>Je dům koncipovaný spíš jako úsporné, nebo velkorysé bydlení?</t>
         </is>
       </c>
-      <c r="E13" s="13" t="n"/>
-      <c r="F13" s="11" t="n"/>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>Návrh pracuje s prostorově úsporným řešením a vysokou užitnou hodnotou plochy; studie výslovně uvádí maximální důraz na funkčnost.</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G13" s="13" t="n"/>
-      <c r="H13" s="13" t="n"/>
+      <c r="H13" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O13" s="13" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="15">
@@ -747,10 +771,22 @@
           <t>Je hlavní důraz na prostor, praktičnost, nebo vzhled?</t>
         </is>
       </c>
-      <c r="E14" s="13" t="n"/>
-      <c r="F14" s="11" t="n"/>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>Hlavní důraz je podle studie na funkčnost a efektivní využití vnitřního prostoru; velká okna a otevřenější obytný prostor zároveň podporují prostorový dojem.</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G14" s="13" t="n"/>
-      <c r="H14" s="13" t="n"/>
+      <c r="H14" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O14" s="13" t="n"/>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="15">
@@ -979,10 +1015,22 @@
           <t>Jak spolu souvisí velikost domu a jeho užitná hodnota?</t>
         </is>
       </c>
-      <c r="E25" s="13" t="n"/>
-      <c r="F25" s="11" t="n"/>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>Koncepce zdůrazňuje skutečnou užitnou hodnotu prostoru, tedy poměr mezi málo využitelnými místy a plochami s vysokou mírou využití.</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G25" s="13" t="n"/>
-      <c r="H25" s="13" t="n"/>
+      <c r="H25" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O25" s="13" t="n"/>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="15">
@@ -998,10 +1046,22 @@
           <t>Snaží se návrh minimalizovat nevyužité prostory?</t>
         </is>
       </c>
-      <c r="E26" s="13" t="n"/>
-      <c r="F26" s="11" t="n"/>
+      <c r="E26" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Studie popisuje vnitřní prostor jako úsporný a navržený s maximálním důrazem na funkčnost.</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G26" s="13" t="n"/>
-      <c r="H26" s="13" t="n"/>
+      <c r="H26" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O26" s="13" t="n"/>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="15">
@@ -1036,10 +1096,22 @@
           <t>Jak dům pracuje s propojením interiéru a zahrady?</t>
         </is>
       </c>
-      <c r="E28" s="13" t="n"/>
-      <c r="F28" s="11" t="n"/>
+      <c r="E28" s="13" t="inlineStr">
+        <is>
+          <t>Obytné místnosti jsou výrazně propojené se zahradní stranou domu; na jihovýchodní straně je velká krytá terasa a velké prosklené otvory.</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G28" s="13" t="n"/>
-      <c r="H28" s="13" t="n"/>
+      <c r="H28" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O28" s="13" t="n"/>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="15">
@@ -1262,10 +1334,22 @@
           <t>Je dům vhodný i na svažitý pozemek?</t>
         </is>
       </c>
-      <c r="E40" s="13" t="n"/>
-      <c r="F40" s="11" t="n"/>
+      <c r="E40" s="13" t="inlineStr">
+        <is>
+          <t>Studie uvádí, že dům lze dobře osadit do svahu na vrstevnici. Konkrétní vhodnost ale vždy závisí na podmínkách daného pozemku a založení.</t>
+        </is>
+      </c>
+      <c r="F40" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G40" s="13" t="n"/>
-      <c r="H40" s="13" t="n"/>
+      <c r="H40" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O40" s="13" t="n"/>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="15">
@@ -1335,10 +1419,22 @@
           <t>Jaká orientace pozemku ke světovým stranám je pro tento dům nejlepší?</t>
         </is>
       </c>
-      <c r="E43" s="13" t="n"/>
-      <c r="F43" s="11" t="n"/>
+      <c r="E43" s="13" t="inlineStr">
+        <is>
+          <t>Studie pracuje se vstupní „technickou“ stranou na severozápad a zahradní stranou s terasou na jihovýchod. Jde o koncepční orientaci studie, nikoli univerzální podmínku každého pozemku.</t>
+        </is>
+      </c>
+      <c r="F43" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G43" s="13" t="n"/>
-      <c r="H43" s="13" t="n"/>
+      <c r="H43" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O43" s="13" t="n"/>
     </row>
     <row r="44" ht="15.75" customHeight="1" s="15">
@@ -1354,10 +1450,22 @@
           <t>Kam je ideální orientovat obytnou část domu?</t>
         </is>
       </c>
-      <c r="E44" s="13" t="n"/>
-      <c r="F44" s="11" t="n"/>
+      <c r="E44" s="13" t="inlineStr">
+        <is>
+          <t>V koncepční studii je hlavní obytná a zahradní strana orientována na jihovýchod.</t>
+        </is>
+      </c>
+      <c r="F44" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G44" s="13" t="n"/>
-      <c r="H44" s="13" t="n"/>
+      <c r="H44" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O44" s="13" t="n"/>
     </row>
     <row r="45" ht="15.75" customHeight="1" s="15">
@@ -1373,10 +1481,22 @@
           <t>Kam je ideální orientovat terasu a zahradu?</t>
         </is>
       </c>
-      <c r="E45" s="13" t="n"/>
-      <c r="F45" s="11" t="n"/>
+      <c r="E45" s="13" t="inlineStr">
+        <is>
+          <t>Koncepční studie umisťuje velkou krytou terasu na jihovýchodní zahradní stranu domu.</t>
+        </is>
+      </c>
+      <c r="F45" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G45" s="13" t="n"/>
-      <c r="H45" s="13" t="n"/>
+      <c r="H45" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O45" s="13" t="n"/>
     </row>
     <row r="46" ht="15.75" customHeight="1" s="15">
@@ -1468,10 +1588,22 @@
           <t>Jak orientace domu ovlivní světlo uvnitř?</t>
         </is>
       </c>
-      <c r="E50" s="13" t="n"/>
-      <c r="F50" s="11" t="n"/>
+      <c r="E50" s="13" t="inlineStr">
+        <is>
+          <t>Orientace ovlivňuje přístup denního světla přes velká okna obytných místností; studie proto váže hlavní prosklení na zahradní stranu.</t>
+        </is>
+      </c>
+      <c r="F50" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G50" s="13" t="n"/>
-      <c r="H50" s="13" t="n"/>
+      <c r="H50" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O50" s="13" t="n"/>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="15">
@@ -1487,10 +1619,22 @@
           <t>Jak orientace domu ovlivní přehřívání v létě?</t>
         </is>
       </c>
-      <c r="E51" s="13" t="n"/>
-      <c r="F51" s="11" t="n"/>
+      <c r="E51" s="13" t="inlineStr">
+        <is>
+          <t>Studie počítá na štítových oknech a oknech ze strany terasy s přípravou pro venkovní žaluzie, které umožňují omezit solární zisky.</t>
+        </is>
+      </c>
+      <c r="F51" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G51" s="13" t="n"/>
-      <c r="H51" s="13" t="n"/>
+      <c r="H51" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O51" s="13" t="n"/>
     </row>
     <row r="52" ht="15.75" customHeight="1" s="15">
@@ -1582,10 +1726,22 @@
           <t>Co všechno je potřeba o pozemku znát před rozhodnutím o umístění domu?</t>
         </is>
       </c>
-      <c r="E56" s="13" t="n"/>
-      <c r="F56" s="11" t="n"/>
+      <c r="E56" s="13" t="inlineStr">
+        <is>
+          <t>Před konkrétním osazením je nutné znát zejména rozměry a sklon parcely, přístup, orientaci, možnosti založení a napojení na technickou infrastrukturu.</t>
+        </is>
+      </c>
+      <c r="F56" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G56" s="13" t="n"/>
-      <c r="H56" s="13" t="n"/>
+      <c r="H56" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023 / Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O56" s="13" t="n"/>
     </row>
     <row r="57" ht="15.75" customHeight="1" s="15">
@@ -1669,10 +1825,22 @@
           <t>Jak umístění domu ovlivní využitelnou část zahrady?</t>
         </is>
       </c>
-      <c r="E60" s="13" t="n"/>
-      <c r="F60" s="11" t="n"/>
+      <c r="E60" s="13" t="inlineStr">
+        <is>
+          <t>Koncepce pracuje s podélným domem a soustřeďuje hlavní obytnou vazbu na zahradní stranu s terasou; způsob osazení proto přímo ovlivňuje využitelnou zahradu.</t>
+        </is>
+      </c>
+      <c r="F60" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G60" s="13" t="n"/>
-      <c r="H60" s="13" t="n"/>
+      <c r="H60" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O60" s="13" t="n"/>
     </row>
     <row r="61" ht="15.75" customHeight="1" s="15">
@@ -1834,10 +2002,22 @@
           <t>Jaké jsou vnější rozměry domu?</t>
         </is>
       </c>
-      <c r="E67" s="13" t="n"/>
-      <c r="F67" s="11" t="n"/>
+      <c r="E67" s="13" t="inlineStr">
+        <is>
+          <t>Technická dokumentace uvádí půdorys obytné části přibližně 6,4 × 22,3 m. PENB pracuje s velmi blízkým rozměrem 6,44 × 22,66 m; jde o různé dokumentační podklady konkrétní realizace.</t>
+        </is>
+      </c>
+      <c r="F67" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G67" s="13" t="n"/>
-      <c r="H67" s="13" t="n"/>
+      <c r="H67" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023 / PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
+        </is>
+      </c>
       <c r="O67" s="13" t="n"/>
     </row>
     <row r="68" ht="15.75" customHeight="1" s="15">
@@ -1853,10 +2033,22 @@
           <t>Jak velký je obývací pokoj s kuchyní?</t>
         </is>
       </c>
-      <c r="E68" s="13" t="n"/>
-      <c r="F68" s="11" t="n"/>
+      <c r="E68" s="13" t="inlineStr">
+        <is>
+          <t>Studie uvádí kuchyň přibližně 12 m² a obývací pokoj přibližně 29 m²; společně tedy přibližně 41 m², bez započtení dalších navazujících ploch.</t>
+        </is>
+      </c>
+      <c r="F68" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G68" s="13" t="n"/>
-      <c r="H68" s="13" t="n"/>
+      <c r="H68" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O68" s="13" t="n"/>
     </row>
     <row r="69" ht="15.75" customHeight="1" s="15">
@@ -2180,10 +2372,22 @@
           <t>Působí dům uvnitř větší, nebo menší, než napovídá jeho plocha?</t>
         </is>
       </c>
-      <c r="E84" s="13" t="n"/>
-      <c r="F84" s="11" t="n"/>
+      <c r="E84" s="13" t="inlineStr">
+        <is>
+          <t>Studie uvádí, že díky menšímu rozponu, otevřenému prostoru a velkým oknům je dům uvnitř vnímán větší, než působí zvenčí.</t>
+        </is>
+      </c>
+      <c r="F84" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G84" s="13" t="n"/>
-      <c r="H84" s="13" t="n"/>
+      <c r="H84" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O84" s="13" t="n"/>
     </row>
     <row r="85" ht="15.75" customHeight="1" s="15">
@@ -2199,10 +2403,22 @@
           <t>Je plocha domu využitá efektivně, nebo jsou v něm hluchá místa?</t>
         </is>
       </c>
-      <c r="E85" s="13" t="n"/>
-      <c r="F85" s="11" t="n"/>
+      <c r="E85" s="13" t="inlineStr">
+        <is>
+          <t>Studie výslovně staví návrh na prostorové hospodárnosti a vysoké míře využití ploch; největší část je věnována hlavnímu obytnému prostoru.</t>
+        </is>
+      </c>
+      <c r="F85" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G85" s="13" t="n"/>
-      <c r="H85" s="13" t="n"/>
+      <c r="H85" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O85" s="13" t="n"/>
     </row>
     <row r="86" ht="15.75" customHeight="1" s="15">
@@ -2254,10 +2470,22 @@
           <t>Jak je dům dispozičně řešený?</t>
         </is>
       </c>
-      <c r="E88" s="13" t="n"/>
-      <c r="F88" s="11" t="n"/>
+      <c r="E88" s="13" t="inlineStr">
+        <is>
+          <t>Jde o přízemní 4+kk: hlavní společný prostor tvoří obývací pokoj, kuchyň a jídelna a doplňují jej tři samostatné pokoje a hygienické a technické zázemí.</t>
+        </is>
+      </c>
+      <c r="F88" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G88" s="13" t="n"/>
-      <c r="H88" s="13" t="n"/>
+      <c r="H88" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022 / B Souhrnná technická zpráva 11/2023</t>
+        </is>
+      </c>
       <c r="O88" s="13" t="n"/>
     </row>
     <row r="89" ht="15.75" customHeight="1" s="15">
@@ -2292,10 +2520,22 @@
           <t>Jak je oddělená denní a klidová část domu?</t>
         </is>
       </c>
-      <c r="E90" s="13" t="n"/>
-      <c r="F90" s="11" t="n"/>
+      <c r="E90" s="13" t="inlineStr">
+        <is>
+          <t>Dispozice soustřeďuje společný obytný prostor na jednu část domu a samostatné pokoje do klidovější části podél společné komunikace.</t>
+        </is>
+      </c>
+      <c r="F90" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G90" s="13" t="n"/>
-      <c r="H90" s="13" t="n"/>
+      <c r="H90" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O90" s="13" t="n"/>
     </row>
     <row r="91" ht="15.75" customHeight="1" s="15">
@@ -2437,10 +2677,22 @@
           <t>Je z obytného prostoru přímý vstup na terasu?</t>
         </is>
       </c>
-      <c r="E97" s="13" t="n"/>
-      <c r="F97" s="11" t="n"/>
+      <c r="E97" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Hlavní obytný prostor je přímo navázán na zahradní stranu a krytou terasu.</t>
+        </is>
+      </c>
+      <c r="F97" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G97" s="13" t="n"/>
-      <c r="H97" s="13" t="n"/>
+      <c r="H97" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O97" s="13" t="n"/>
     </row>
     <row r="98" ht="15.75" customHeight="1" s="15">
@@ -2475,10 +2727,22 @@
           <t>Lze některý z pokojů využít jako pracovnu?</t>
         </is>
       </c>
-      <c r="E99" s="13" t="n"/>
-      <c r="F99" s="11" t="n"/>
+      <c r="E99" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Samostatný pokoj lze dispozičně využít jako pracovnu; studie pracuje s volnou dispozicí umožněnou rámovým konstrukčním konceptem.</t>
+        </is>
+      </c>
+      <c r="F99" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G99" s="13" t="n"/>
-      <c r="H99" s="13" t="n"/>
+      <c r="H99" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O99" s="13" t="n"/>
     </row>
     <row r="100" ht="15.75" customHeight="1" s="15">
@@ -2563,10 +2827,22 @@
           <t>Proč jsou jednotlivé místnosti uspořádané právě tímto způsobem?</t>
         </is>
       </c>
-      <c r="E103" s="13" t="n"/>
-      <c r="F103" s="11" t="n"/>
+      <c r="E103" s="13" t="inlineStr">
+        <is>
+          <t>Uspořádání vychází z úsporného půdorysu, minimalizace nevyužitých ploch a přímého propojení hlavního obytného prostoru se zahradou.</t>
+        </is>
+      </c>
+      <c r="F103" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G103" s="13" t="n"/>
-      <c r="H103" s="13" t="n"/>
+      <c r="H103" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O103" s="13" t="n"/>
     </row>
     <row r="104" ht="15.75" customHeight="1" s="15">
@@ -2732,10 +3008,22 @@
           <t>Jaké materiály jsou použité na fasádě?</t>
         </is>
       </c>
-      <c r="E112" s="13" t="n"/>
-      <c r="F112" s="11" t="n"/>
+      <c r="E112" s="13" t="inlineStr">
+        <is>
+          <t>Technická dokumentace konkrétní realizace uvádí fasádní plášť z pozinkovaného falcovaného plechu v antracitovém odstínu; studie současně ukazuje i koncepční variantu s dřevěným obkladem.</t>
+        </is>
+      </c>
+      <c r="F112" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G112" s="13" t="n"/>
-      <c r="H112" s="13" t="n"/>
+      <c r="H112" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023 / Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O112" s="13" t="n"/>
     </row>
     <row r="113" ht="15.75" customHeight="1" s="15">
@@ -2953,10 +3241,22 @@
           <t>Lze použít dřevěný nebo jiný obklad části fasády?</t>
         </is>
       </c>
-      <c r="E123" s="13" t="n"/>
-      <c r="F123" s="11" t="n"/>
+      <c r="E123" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Studie obsahuje variantu WOOD s obkladem z dřevěných palubek ošetřených fasádním olejem a uvádí možnost více odstínů.</t>
+        </is>
+      </c>
+      <c r="F123" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G123" s="13" t="n"/>
-      <c r="H123" s="13" t="n"/>
+      <c r="H123" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O123" s="13" t="n"/>
     </row>
     <row r="124" ht="15.75" customHeight="1" s="15">
@@ -2991,10 +3291,22 @@
           <t>Proč má dům právě tento architektonický vzhled?</t>
         </is>
       </c>
-      <c r="E125" s="13" t="n"/>
-      <c r="F125" s="11" t="n"/>
+      <c r="E125" s="13" t="inlineStr">
+        <is>
+          <t>Architektura vychází z úzkého podélného bungalovu, jednoduché sedlové střechy, velkých otvorů do zahrady a důrazu na funkční využití prostoru.</t>
+        </is>
+      </c>
+      <c r="F125" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G125" s="13" t="n"/>
-      <c r="H125" s="13" t="n"/>
+      <c r="H125" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O125" s="13" t="n"/>
     </row>
     <row r="126" ht="15.75" customHeight="1" s="15">
@@ -3010,10 +3322,22 @@
           <t>Jaké prvky nejvíce určují charakter tohoto domu?</t>
         </is>
       </c>
-      <c r="E126" s="13" t="n"/>
-      <c r="F126" s="11" t="n"/>
+      <c r="E126" s="13" t="inlineStr">
+        <is>
+          <t>Charakter domu určují zejména podélná hmota, sedlová střecha, výrazné štítové prosklení, zahradní terasa a kombinace tmavého pláště s dřevěnými prvky.</t>
+        </is>
+      </c>
+      <c r="F126" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G126" s="13" t="n"/>
-      <c r="H126" s="13" t="n"/>
+      <c r="H126" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O126" s="13" t="n"/>
     </row>
     <row r="127" ht="15.75" customHeight="1" s="15">
@@ -3141,10 +3465,22 @@
           <t>Je možné změnit umístění příček?</t>
         </is>
       </c>
-      <c r="E133" s="13" t="n"/>
-      <c r="F133" s="11" t="n"/>
+      <c r="E133" s="13" t="inlineStr">
+        <is>
+          <t>Studie popisuje konstrukční koncept jako řešení umožňující velmi volnou dispozici; konkrétní změna příček ale musí respektovat skutečnou nosnou a ztužující funkci stěn podle realizační statiky.</t>
+        </is>
+      </c>
+      <c r="F133" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G133" s="13" t="n"/>
-      <c r="H133" s="13" t="n"/>
+      <c r="H133" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022 / Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O133" s="13" t="n"/>
     </row>
     <row r="134" ht="15.75" customHeight="1" s="15">
@@ -3198,10 +3534,22 @@
           <t>Dá se jeden z pokojů využít jako pracovna?</t>
         </is>
       </c>
-      <c r="E136" s="13" t="n"/>
-      <c r="F136" s="11" t="n"/>
+      <c r="E136" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Jeden ze samostatných pokojů lze využít jako pracovnu bez změny základního dispozičního principu.</t>
+        </is>
+      </c>
+      <c r="F136" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G136" s="13" t="n"/>
-      <c r="H136" s="13" t="n"/>
+      <c r="H136" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O136" s="13" t="n"/>
     </row>
     <row r="137" ht="15.75" customHeight="1" s="15">
@@ -3388,10 +3736,22 @@
           <t>Které změny jsou jednoduché a které už vyžadují zásah do konstrukce?</t>
         </is>
       </c>
-      <c r="E146" s="13" t="n"/>
-      <c r="F146" s="11" t="n"/>
+      <c r="E146" s="13" t="inlineStr">
+        <is>
+          <t>Nenostné dispoziční úpravy jsou principiálně jednodušší; zásahy do nosných nebo ztužujících stěn, otvorů a rámů musí být posouzeny statikem.</t>
+        </is>
+      </c>
+      <c r="F146" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G146" s="13" t="n"/>
-      <c r="H146" s="13" t="n"/>
+      <c r="H146" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O146" s="13" t="n"/>
     </row>
     <row r="147" ht="15.75" customHeight="1" s="15">
@@ -3407,10 +3767,22 @@
           <t>Které části dispozice by se naopak měnit neměly?</t>
         </is>
       </c>
-      <c r="E147" s="13" t="n"/>
-      <c r="F147" s="11" t="n"/>
+      <c r="E147" s="13" t="inlineStr">
+        <is>
+          <t>Bez statického posouzení se nemají měnit prvky s nosnou nebo ztužující funkcí ani otvory, které ovlivňují nosný rám.</t>
+        </is>
+      </c>
+      <c r="F147" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G147" s="13" t="n"/>
-      <c r="H147" s="13" t="n"/>
+      <c r="H147" s="13" t="inlineStr">
+        <is>
+          <t>Statický posudek RD Krásné Pole / Ing. Ondřej Kika / 04-2024</t>
+        </is>
+      </c>
       <c r="O147" s="13" t="n"/>
     </row>
     <row r="148" ht="15.75" customHeight="1" s="15">
@@ -4275,10 +4647,22 @@
           <t>Jaké základy tento dům potřebuje?</t>
         </is>
       </c>
-      <c r="E193" s="13" t="n"/>
-      <c r="F193" s="11" t="n"/>
+      <c r="E193" s="13" t="inlineStr">
+        <is>
+          <t>Konkrétní referenční projekt je založen na železobetonových základových pásech.</t>
+        </is>
+      </c>
+      <c r="F193" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G193" s="13" t="n"/>
-      <c r="H193" s="13" t="n"/>
+      <c r="H193" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023</t>
+        </is>
+      </c>
       <c r="O193" s="13" t="n"/>
     </row>
     <row r="194" ht="15.75" customHeight="1" s="15">
@@ -4527,10 +4911,22 @@
           <t>Jak vlastnosti podloží ovlivní způsob založení domu?</t>
         </is>
       </c>
-      <c r="E205" s="13" t="n"/>
-      <c r="F205" s="11" t="n"/>
+      <c r="E205" s="13" t="inlineStr">
+        <is>
+          <t>Způsob založení musí odpovídat konkrétním geotechnickým a terénním podmínkám; referenční projekt používá železobetonové základové pásy.</t>
+        </is>
+      </c>
+      <c r="F205" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G205" s="13" t="n"/>
-      <c r="H205" s="13" t="n"/>
+      <c r="H205" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023</t>
+        </is>
+      </c>
       <c r="O205" s="13" t="n"/>
     </row>
     <row r="206" ht="15.75" customHeight="1" s="15">
@@ -5716,10 +6112,22 @@
           <t>Jak silné jsou obvodové stěny?</t>
         </is>
       </c>
-      <c r="E257" s="13" t="n"/>
-      <c r="F257" s="11" t="n"/>
+      <c r="E257" s="13" t="inlineStr">
+        <is>
+          <t>PENB uvádí u obvodové sendvičové konstrukce foukanou izolaci Climatizer tloušťky 280 mm. Celkovou tloušťku celé hotové obvodové stěny tento údaj sám o sobě neurčuje.</t>
+        </is>
+      </c>
+      <c r="F257" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G257" s="13" t="n"/>
-      <c r="H257" s="13" t="n"/>
+      <c r="H257" s="13" t="inlineStr">
+        <is>
+          <t>PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
+        </is>
+      </c>
       <c r="O257" s="13" t="n"/>
     </row>
     <row r="258" ht="15.75" customHeight="1" s="15">
@@ -5735,10 +6143,22 @@
           <t>Z jakých vrstev se obvodová stěna skládá?</t>
         </is>
       </c>
-      <c r="E258" s="13" t="n"/>
-      <c r="F258" s="11" t="n"/>
+      <c r="E258" s="13" t="inlineStr">
+        <is>
+          <t>Obvodový plášť je dřevěná sendvičová rámová konstrukce s foukanou celulózovou izolací Climatizer a difuzně otevřeným řešením; jednotlivé vrstvy se řídí projektovou skladbou.</t>
+        </is>
+      </c>
+      <c r="F258" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G258" s="13" t="n"/>
-      <c r="H258" s="13" t="n"/>
+      <c r="H258" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023 / PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
+        </is>
+      </c>
       <c r="O258" s="13" t="n"/>
     </row>
     <row r="259" ht="15.75" customHeight="1" s="15">
@@ -6070,10 +6490,22 @@
           <t>Jak je konstrukce chráněná proti kondenzaci vlhkosti uvnitř skladby?</t>
         </is>
       </c>
-      <c r="E271" s="13" t="n"/>
-      <c r="F271" s="11" t="n"/>
+      <c r="E271" s="13" t="inlineStr">
+        <is>
+          <t>Konstrukce je řešena jako difuzně otevřená skladba; její vrstvy jsou navrženy tak, aby umožňovaly bezpečný transport vodní páry konstrukcí.</t>
+        </is>
+      </c>
+      <c r="F271" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G271" s="13" t="n"/>
-      <c r="H271" s="13" t="n"/>
+      <c r="H271" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023</t>
+        </is>
+      </c>
       <c r="O271" s="13" t="n"/>
     </row>
     <row r="272" ht="15.75" customHeight="1" s="15">
@@ -6225,10 +6657,22 @@
           <t>Jakou barvu má střecha?</t>
         </is>
       </c>
-      <c r="E278" s="13" t="n"/>
-      <c r="F278" s="11" t="n"/>
+      <c r="E278" s="13" t="inlineStr">
+        <is>
+          <t>Střecha je v antracitovém odstínu.</t>
+        </is>
+      </c>
+      <c r="F278" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G278" s="13" t="n"/>
-      <c r="H278" s="13" t="n"/>
+      <c r="H278" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O278" s="13" t="n"/>
     </row>
     <row r="279" ht="15.75" customHeight="1" s="15">
@@ -6363,10 +6807,22 @@
           <t>Jakou údržbu potřebuje fasáda?</t>
         </is>
       </c>
-      <c r="E284" s="13" t="n"/>
-      <c r="F284" s="11" t="n"/>
+      <c r="E284" s="13" t="inlineStr">
+        <is>
+          <t>Dřevěné venkovní prvky vyžadují pravidelné povrchové ošetření; u plechového pláště dostupné podklady nestanovují stejný obnovovací interval.</t>
+        </is>
+      </c>
+      <c r="F284" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G284" s="13" t="n"/>
-      <c r="H284" s="13" t="n"/>
+      <c r="H284" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O284" s="13" t="n"/>
     </row>
     <row r="285" ht="15.75" customHeight="1" s="15">
@@ -6432,10 +6888,22 @@
           <t>Lze na fasádě použít dřevo nebo jiný obklad?</t>
         </is>
       </c>
-      <c r="E287" s="13" t="n"/>
-      <c r="F287" s="11" t="n"/>
+      <c r="E287" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Studie obsahuje variantu fasády s dřevěnými palubkami ošetřenými fasádním olejem.</t>
+        </is>
+      </c>
+      <c r="F287" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G287" s="13" t="n"/>
-      <c r="H287" s="13" t="n"/>
+      <c r="H287" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O287" s="13" t="n"/>
     </row>
     <row r="288" ht="15.75" customHeight="1" s="15">
@@ -7009,10 +7477,22 @@
           <t>Jak jsou řešené dveře z obývacího prostoru na terasu?</t>
         </is>
       </c>
-      <c r="E307" s="13" t="n"/>
-      <c r="F307" s="11" t="n"/>
+      <c r="E307" s="13" t="inlineStr">
+        <is>
+          <t>Obytný prostor má přímé dveře na terasu. CURRENT validace potvrzuje, že terasové dveře nejsou posuvné.</t>
+        </is>
+      </c>
+      <c r="F307" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G307" s="13" t="n"/>
-      <c r="H307" s="13" t="n"/>
+      <c r="H307" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022 / Validace autora domu / CURRENT / 2026-09-09</t>
+        </is>
+      </c>
       <c r="O307" s="13" t="n"/>
     </row>
     <row r="308" ht="15.75" customHeight="1" s="15">
@@ -7059,10 +7539,22 @@
           <t>Jak velké jsou prosklené plochy v obytné části?</t>
         </is>
       </c>
-      <c r="E309" s="13" t="n"/>
-      <c r="F309" s="11" t="n"/>
+      <c r="E309" s="13" t="inlineStr">
+        <is>
+          <t>PENB uvádí podíl průsvitných konstrukcí 18,6 % z plochy svislých konstrukcí. Samostatnou plochu prosklení pouze v obytné části dokument nevyčísluje.</t>
+        </is>
+      </c>
+      <c r="F309" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G309" s="13" t="n"/>
-      <c r="H309" s="13" t="n"/>
+      <c r="H309" s="13" t="inlineStr">
+        <is>
+          <t>PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
+        </is>
+      </c>
       <c r="O309" s="13" t="n"/>
     </row>
     <row r="310" ht="15.75" customHeight="1" s="15">
@@ -7302,10 +7794,22 @@
           <t>Nebude v domě v létě příliš horko?</t>
         </is>
       </c>
-      <c r="E320" s="13" t="n"/>
-      <c r="F320" s="11" t="n"/>
+      <c r="E320" s="13" t="inlineStr">
+        <is>
+          <t>Dům má kvalitně izolovanou obálku a venkovní stínění. Dokumentace ale sama neurčuje konkrétní maximální letní vnitřní teplotu, takže nelze slíbit určitou teplotu bez provozních dat.</t>
+        </is>
+      </c>
+      <c r="F320" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G320" s="13" t="n"/>
-      <c r="H320" s="13" t="n"/>
+      <c r="H320" s="13" t="inlineStr">
+        <is>
+          <t>PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023 / Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O320" s="13" t="n"/>
     </row>
     <row r="321" ht="15.75" customHeight="1" s="15">
@@ -7352,10 +7856,22 @@
           <t>Jak dům chrání interiér před přehříváním?</t>
         </is>
       </c>
-      <c r="E322" s="13" t="n"/>
-      <c r="F322" s="11" t="n"/>
+      <c r="E322" s="13" t="inlineStr">
+        <is>
+          <t>Proti přehřívání pomáhá venkovní stínění prosklených ploch; energetická dokumentace zároveň pracuje s chlazením. Přesný účinek závisí na provozu a podmínkách.</t>
+        </is>
+      </c>
+      <c r="F322" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G322" s="13" t="n"/>
-      <c r="H322" s="13" t="n"/>
+      <c r="H322" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022 / PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
+        </is>
+      </c>
       <c r="O322" s="13" t="n"/>
     </row>
     <row r="323" ht="15.75" customHeight="1" s="15">
@@ -7662,10 +8178,22 @@
           <t>Jak se v jednotlivých místnostech udržuje příjemná teplota?</t>
         </is>
       </c>
-      <c r="E332" s="13" t="n"/>
-      <c r="F332" s="11" t="n"/>
+      <c r="E332" s="13" t="inlineStr">
+        <is>
+          <t>Tepelnou stabilitu podporuje tepelněizolační obálka a řízené větrání; historický PENB navíc pracuje s vytápěním a chlazením, ale konkrétní CURRENT regulaci jednotlivých místností je nutné oddělit od této historické konfigurace.</t>
+        </is>
+      </c>
+      <c r="F332" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G332" s="13" t="n"/>
-      <c r="H332" s="13" t="n"/>
+      <c r="H332" s="13" t="inlineStr">
+        <is>
+          <t>PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
+        </is>
+      </c>
       <c r="O332" s="13" t="n"/>
     </row>
     <row r="333" ht="15.75" customHeight="1" s="15">
@@ -8003,10 +8531,22 @@
           <t>Jak je dům chráněný proti vlhkosti?</t>
         </is>
       </c>
-      <c r="E345" s="13" t="n"/>
-      <c r="F345" s="11" t="n"/>
+      <c r="E345" s="13" t="inlineStr">
+        <is>
+          <t>Spodní konstrukce je chráněna hydroizolačními vrstvami a obvodový plášť je navržen jako difuzně otevřený. Konkrétní ochrana jednotlivých detailů vychází z projektové skladby.</t>
+        </is>
+      </c>
+      <c r="F345" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G345" s="13" t="n"/>
-      <c r="H345" s="13" t="n"/>
+      <c r="H345" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023</t>
+        </is>
+      </c>
       <c r="O345" s="13" t="n"/>
     </row>
     <row r="346" ht="15.75" customHeight="1" s="15">
@@ -8022,10 +8562,22 @@
           <t>Jak je konstrukce chráněná proti plísním a hnilobě?</t>
         </is>
       </c>
-      <c r="E346" s="13" t="n"/>
-      <c r="F346" s="11" t="n"/>
+      <c r="E346" s="13" t="inlineStr">
+        <is>
+          <t>Ochrana dřevěné konstrukce proti dlouhodobému působení vlhkosti vychází zejména ze správně provedené hydroizolace, difuzně otevřené skladby a ochrany konstrukce před zatékáním.</t>
+        </is>
+      </c>
+      <c r="F346" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G346" s="13" t="n"/>
-      <c r="H346" s="13" t="n"/>
+      <c r="H346" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023</t>
+        </is>
+      </c>
       <c r="O346" s="13" t="n"/>
     </row>
     <row r="347" ht="15.75" customHeight="1" s="15">
@@ -8236,10 +8788,22 @@
           <t>Jak konstrukce reaguje při dlouhodobém působení vody po havárii?</t>
         </is>
       </c>
-      <c r="E356" s="13" t="n"/>
-      <c r="F356" s="11" t="n"/>
+      <c r="E356" s="13" t="inlineStr">
+        <is>
+          <t>Dlouhodobé působení vody je pro dřevěnou konstrukci nežádoucí; po havárii je nutné odstranit zdroj vody, konstrukci vysušit a podle rozsahu prověřit dotčené vrstvy. Dokumentace neposkytuje univerzální scénář pro každou havárii.</t>
+        </is>
+      </c>
+      <c r="F356" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G356" s="13" t="n"/>
-      <c r="H356" s="13" t="n"/>
+      <c r="H356" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023</t>
+        </is>
+      </c>
       <c r="O356" s="13" t="n"/>
     </row>
     <row r="357" ht="15.75" customHeight="1" s="15">
@@ -10011,10 +10575,22 @@
           <t>Kolik denního světla je v obytném prostoru?</t>
         </is>
       </c>
-      <c r="E430" s="13" t="n"/>
-      <c r="F430" s="11" t="n"/>
+      <c r="E430" s="13" t="inlineStr">
+        <is>
+          <t>Hlavní obytný prostor využívá velké zahradní a štítové prosklení; studie jej popisuje jako výrazně propojený se světlem a zahradou.</t>
+        </is>
+      </c>
+      <c r="F430" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G430" s="13" t="n"/>
-      <c r="H430" s="13" t="n"/>
+      <c r="H430" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O430" s="13" t="n"/>
     </row>
     <row r="431" ht="15.75" customHeight="1" s="15">
@@ -10030,10 +10606,22 @@
           <t>Jak je obytný prostor propojený se zahradou?</t>
         </is>
       </c>
-      <c r="E431" s="13" t="n"/>
-      <c r="F431" s="11" t="n"/>
+      <c r="E431" s="13" t="inlineStr">
+        <is>
+          <t>Obytný prostor je přímo propojen se zahradní stranou a velkou krytou terasou.</t>
+        </is>
+      </c>
+      <c r="F431" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G431" s="13" t="n"/>
-      <c r="H431" s="13" t="n"/>
+      <c r="H431" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O431" s="13" t="n"/>
     </row>
     <row r="432" ht="15.75" customHeight="1" s="15">
@@ -10201,10 +10789,22 @@
           <t>Jak je v obývacím prostoru řešené stínění velkých oken?</t>
         </is>
       </c>
-      <c r="E440" s="13" t="n"/>
-      <c r="F440" s="11" t="n"/>
+      <c r="E440" s="13" t="inlineStr">
+        <is>
+          <t>Na zahradních a štítových oknech studie počítá s venkovním stíněním; CURRENT konfigurace potvrzuje antracitové roletové žaluzie.</t>
+        </is>
+      </c>
+      <c r="F440" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G440" s="13" t="n"/>
-      <c r="H440" s="13" t="n"/>
+      <c r="H440" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022 / Validace autora domu / CURRENT / 2026-09-09</t>
+        </is>
+      </c>
       <c r="O440" s="13" t="n"/>
     </row>
     <row r="441" ht="15.75" customHeight="1" s="15">
@@ -12805,10 +13405,22 @@
           <t>Je z obývacího pokoje přímý výhled do zahrady?</t>
         </is>
       </c>
-      <c r="E574" s="13" t="n"/>
-      <c r="F574" s="11" t="n"/>
+      <c r="E574" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Hlavní obytný prostor je orientován k zahradní straně a velkému prosklení.</t>
+        </is>
+      </c>
+      <c r="F574" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G574" s="13" t="n"/>
-      <c r="H574" s="13" t="n"/>
+      <c r="H574" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O574" s="13" t="n"/>
     </row>
     <row r="575" ht="15.75" customHeight="1" s="15">
@@ -12824,10 +13436,22 @@
           <t>Jak je dům propojený se zahradou?</t>
         </is>
       </c>
-      <c r="E575" s="13" t="n"/>
-      <c r="F575" s="11" t="n"/>
+      <c r="E575" s="13" t="inlineStr">
+        <is>
+          <t>Dům je koncipován jako „byt v zahradě“ a hlavní obytná část je přímo propojena s krytou terasou a zahradní stranou.</t>
+        </is>
+      </c>
+      <c r="F575" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G575" s="13" t="n"/>
-      <c r="H575" s="13" t="n"/>
+      <c r="H575" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O575" s="13" t="n"/>
     </row>
     <row r="576" ht="15.75" customHeight="1" s="15">
@@ -12900,10 +13524,22 @@
           <t>Jak velké jsou prosklené plochy směrem do zahrady?</t>
         </is>
       </c>
-      <c r="E579" s="13" t="n"/>
-      <c r="F579" s="11" t="n"/>
+      <c r="E579" s="13" t="inlineStr">
+        <is>
+          <t>Dům používá výrazné zahradní a štítové prosklení. PENB uvádí, že průsvitné konstrukce tvoří 18,6 % svislé obálky celé budovy; nejde však o plochu pouze zahradního prosklení.</t>
+        </is>
+      </c>
+      <c r="F579" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G579" s="13" t="n"/>
-      <c r="H579" s="13" t="n"/>
+      <c r="H579" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022 / PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
+        </is>
+      </c>
       <c r="O579" s="13" t="n"/>
     </row>
     <row r="580" ht="15.75" customHeight="1" s="15">
@@ -12995,10 +13631,22 @@
           <t>Je z kuchyně vidět na zahradu nebo terasu?</t>
         </is>
       </c>
-      <c r="E584" s="13" t="n"/>
-      <c r="F584" s="11" t="n"/>
+      <c r="E584" s="13" t="inlineStr">
+        <is>
+          <t>Kuchyň je součástí společného obytného prostoru orientovaného k zahradní straně domu.</t>
+        </is>
+      </c>
+      <c r="F584" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G584" s="13" t="n"/>
-      <c r="H584" s="13" t="n"/>
+      <c r="H584" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O584" s="13" t="n"/>
     </row>
     <row r="585" ht="15.75" customHeight="1" s="15">
@@ -13083,10 +13731,22 @@
           <t>Nezpůsobují velké prosklené plochy v létě přehřívání?</t>
         </is>
       </c>
-      <c r="E588" s="13" t="n"/>
-      <c r="F588" s="11" t="n"/>
+      <c r="E588" s="13" t="inlineStr">
+        <is>
+          <t>Velké prosklení zvyšuje význam venkovního stínění; studie proto u zahradních a štítových oken počítá s přípravou venkovních žaluzií.</t>
+        </is>
+      </c>
+      <c r="F588" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G588" s="13" t="n"/>
-      <c r="H588" s="13" t="n"/>
+      <c r="H588" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O588" s="13" t="n"/>
     </row>
     <row r="589" ht="15.75" customHeight="1" s="15">
@@ -13288,10 +13948,22 @@
           <t>Kam je nejlepší terasu orientovat?</t>
         </is>
       </c>
-      <c r="E597" s="13" t="n"/>
-      <c r="F597" s="11" t="n"/>
+      <c r="E597" s="13" t="inlineStr">
+        <is>
+          <t>Koncepční studie orientuje hlavní terasu na jihovýchodní zahradní stranu. U konkrétní parcely je ale nutné orientaci přizpůsobit osazení domu a okolí.</t>
+        </is>
+      </c>
+      <c r="F597" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G597" s="13" t="n"/>
-      <c r="H597" s="13" t="n"/>
+      <c r="H597" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O597" s="13" t="n"/>
     </row>
     <row r="598" ht="15.75" customHeight="1" s="15">
@@ -13307,10 +13979,22 @@
           <t>Je z kuchyně dobře dostupná terasa pro venkovní stolování?</t>
         </is>
       </c>
-      <c r="E598" s="13" t="n"/>
-      <c r="F598" s="11" t="n"/>
+      <c r="E598" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Kuchyň je součástí hlavního obytného prostoru přímo navázaného na zahradní terasu.</t>
+        </is>
+      </c>
+      <c r="F598" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G598" s="13" t="n"/>
-      <c r="H598" s="13" t="n"/>
+      <c r="H598" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O598" s="13" t="n"/>
     </row>
     <row r="599" ht="15.75" customHeight="1" s="15">
@@ -13376,10 +14060,22 @@
           <t>Jak dům funguje při častém přecházení mezi interiérem a zahradou?</t>
         </is>
       </c>
-      <c r="E601" s="13" t="n"/>
-      <c r="F601" s="11" t="n"/>
+      <c r="E601" s="13" t="inlineStr">
+        <is>
+          <t>Přímé propojení hlavního obytného prostoru s velkou krytou terasou podporuje častý pohyb mezi interiérem a zahradou.</t>
+        </is>
+      </c>
+      <c r="F601" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G601" s="13" t="n"/>
-      <c r="H601" s="13" t="n"/>
+      <c r="H601" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O601" s="13" t="n"/>
     </row>
     <row r="602" ht="15.75" customHeight="1" s="15">
@@ -13578,10 +14274,22 @@
           <t>Co je největší předností propojení tohoto domu se zahradou?</t>
         </is>
       </c>
-      <c r="E611" s="13" t="n"/>
-      <c r="F611" s="11" t="n"/>
+      <c r="E611" s="13" t="inlineStr">
+        <is>
+          <t>Hlavní předností koncepce je přímé propojení společného obytného prostoru s krytou terasou a zahradou – princip, který studie označuje jako „byt v zahradě“.</t>
+        </is>
+      </c>
+      <c r="F611" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G611" s="13" t="n"/>
-      <c r="H611" s="13" t="n"/>
+      <c r="H611" s="13" t="inlineStr">
+        <is>
+          <t>Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O611" s="13" t="n"/>
     </row>
     <row r="612" ht="15.75" customHeight="1" s="15">
@@ -14301,10 +15009,22 @@
           <t>Jak spotřebu ovlivňuje rekuperace?</t>
         </is>
       </c>
-      <c r="E644" s="13" t="n"/>
-      <c r="F644" s="11" t="n"/>
+      <c r="E644" s="13" t="inlineStr">
+        <is>
+          <t>Rekuperace zpětně využívá teplo z odváděného vzduchu a omezuje tak tepelné ztráty větráním. PENB pro nucené větrání počítá se zpětným získáváním tepla; přesný finanční přínos samostatně nevyčísluje.</t>
+        </is>
+      </c>
+      <c r="F644" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G644" s="13" t="n"/>
-      <c r="H644" s="13" t="n"/>
+      <c r="H644" s="13" t="inlineStr">
+        <is>
+          <t>PENB RD Krásné Pole / ev. č. 516981.0 / 30.06.2023</t>
+        </is>
+      </c>
       <c r="O644" s="13" t="n"/>
     </row>
     <row r="645" ht="15.75" customHeight="1" s="15">
@@ -15013,10 +15733,22 @@
           <t>Co můžu dělat, aby dům vydržel co nejdéle v dobrém stavu?</t>
         </is>
       </c>
-      <c r="E674" s="13" t="n"/>
-      <c r="F674" s="11" t="n"/>
+      <c r="E674" s="13" t="inlineStr">
+        <is>
+          <t>Pro dlouhou životnost je důležité chránit konstrukci před dlouhodobou vlhkostí, udržovat venkovní dřevěné prvky a provádět servis technických zařízení podle požadavků jejich výrobců.</t>
+        </is>
+      </c>
+      <c r="F674" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G674" s="13" t="n"/>
-      <c r="H674" s="13" t="n"/>
+      <c r="H674" s="13" t="inlineStr">
+        <is>
+          <t>B Souhrnná technická zpráva 11/2023 / Studie Bungalov 4KK / 01.11.2022</t>
+        </is>
+      </c>
       <c r="O674" s="13" t="n"/>
     </row>
     <row r="675" ht="15.75" customHeight="1" s="15">

</xml_diff>

<commit_message>
docs(knowledge): apply Bungalov 4KK author knowledge round 1
</commit_message>
<xml_diff>
--- a/docs/knowledge/znalostní báze – mustr 02.xlsx
+++ b/docs/knowledge/znalostní báze – mustr 02.xlsx
@@ -526,10 +526,22 @@
           <t>Pro koho je tento dům především navržený?</t>
         </is>
       </c>
-      <c r="E3" s="13" t="n"/>
-      <c r="F3" s="11" t="n"/>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>Bungalov 4+kk je optimálně navržený pro čtyřčlennou rodinu se dvěma dětmi. Vhodný je také pro rodinu s jedním dítětem nebo pro starší pár, který chce větší prostorový komfort.</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G3" s="13" t="n"/>
-      <c r="H3" s="13" t="n"/>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O3" s="13" t="n"/>
     </row>
     <row r="4" ht="15.75" customHeight="1" s="15">
@@ -576,10 +588,22 @@
           <t>Je tento dům vhodný pro rodinu s dětmi?</t>
         </is>
       </c>
-      <c r="E5" s="13" t="n"/>
-      <c r="F5" s="11" t="n"/>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Optimální využití je pro rodinu se dvěma dětmi. Děti mohou mít každý vlastní pokoj, nebo mohou sdílet jeden dětský pokoj a další místnost může sloužit jako pracovna.</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G5" s="13" t="n"/>
-      <c r="H5" s="13" t="n"/>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O5" s="13" t="n"/>
     </row>
     <row r="6" ht="15.75" customHeight="1" s="15">
@@ -595,10 +619,22 @@
           <t>Je dům navržený spíš pro mladou rodinu, nebo i pro starší pár?</t>
         </is>
       </c>
-      <c r="E6" s="13" t="n"/>
-      <c r="F6" s="11" t="n"/>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>Dům je vhodný jak pro rodinu s dětmi, tak pro starší pár, který má potřebu většího prostorového komfortu.</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G6" s="13" t="n"/>
-      <c r="H6" s="13" t="n"/>
+      <c r="H6" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O6" s="13" t="n"/>
     </row>
     <row r="7" ht="15.75" customHeight="1" s="15">
@@ -664,10 +700,22 @@
           <t>V čem se tento dům liší od běžného bungalovu 4+kk?</t>
         </is>
       </c>
-      <c r="E9" s="13" t="n"/>
-      <c r="F9" s="11" t="n"/>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>Dům je navržen s mimořádným důrazem na efektivní využití zastavěného prostoru a minimum nevyužitých zákoutí. Současně je jeho konstrukční a technologická koncepce podřízena minimalizaci energetických nákladů a maximalizaci využitelných energetických zisků.</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G9" s="13" t="n"/>
-      <c r="H9" s="13" t="n"/>
+      <c r="H9" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O9" s="13" t="n"/>
     </row>
     <row r="10" ht="15.75" customHeight="1" s="15">
@@ -683,10 +731,22 @@
           <t>Jaké jsou jeho hlavní přednosti?</t>
         </is>
       </c>
-      <c r="E10" s="13" t="n"/>
-      <c r="F10" s="11" t="n"/>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>Hlavními přednostmi jsou velmi efektivní využití zastavěného prostoru s minimem nevyužitých míst a energetická koncepce zaměřená na minimalizaci energetických nákladů a maximalizaci energetických zisků.</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G10" s="13" t="n"/>
-      <c r="H10" s="13" t="n"/>
+      <c r="H10" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O10" s="13" t="n"/>
     </row>
     <row r="11" ht="15.75" customHeight="1" s="15">
@@ -702,10 +762,22 @@
           <t>Jaké jsou naopak jeho hlavní kompromisy?</t>
         </is>
       </c>
-      <c r="E11" s="13" t="n"/>
-      <c r="F11" s="11" t="n"/>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>Největším kompromisem je podlouhlý tvar domu. Úzký konstrukční rozpon přibližně 5,6 m vede k větší celkové délce domu, přibližně 20 m, a tím i k větším vzdálenostem mezi jeho částmi.</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G11" s="13" t="n"/>
-      <c r="H11" s="13" t="n"/>
+      <c r="H11" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O11" s="13" t="n"/>
     </row>
     <row r="12" ht="15.75" customHeight="1" s="15">
@@ -721,10 +793,22 @@
           <t>Pro koho bych tento dům naopak nedoporučil?</t>
         </is>
       </c>
-      <c r="E12" s="13" t="n"/>
-      <c r="F12" s="11" t="n"/>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>Méně vhodný je pro rodinu se třemi dětmi, pokud každý člen domácnosti potřebuje samostatný pokoj a současně má zůstat zachována pracovna. Takové využití je možné, ale už prostorově stísněnější.</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G12" s="13" t="n"/>
-      <c r="H12" s="13" t="n"/>
+      <c r="H12" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O12" s="13" t="n"/>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="15">
@@ -802,10 +886,22 @@
           <t>Co je na tomto domě podle autora nejdůležitější?</t>
         </is>
       </c>
-      <c r="E15" s="13" t="n"/>
-      <c r="F15" s="11" t="n"/>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>Z pohledu autora jsou zásadní dvě věci: maximálně vytěžit užitnou hodnotu zastavěného prostoru a současně minimalizovat energetické náklady a maximalizovat energetické zisky.</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G15" s="13" t="n"/>
-      <c r="H15" s="13" t="n"/>
+      <c r="H15" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O15" s="13" t="n"/>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="15">
@@ -878,10 +974,22 @@
           <t>Nakolik je návrh domu univerzální pro různé životní situace?</t>
         </is>
       </c>
-      <c r="E19" s="13" t="n"/>
-      <c r="F19" s="11" t="n"/>
+      <c r="E19" s="13" t="inlineStr">
+        <is>
+          <t>Dispozice se dokáže přizpůsobit různým životním situacím zejména variabilitou bloku ložnice, dětského pokoje a pracovny. Posunem příček lze měnit velikost a využití těchto místností.</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G19" s="13" t="n"/>
-      <c r="H19" s="13" t="n"/>
+      <c r="H19" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O19" s="13" t="n"/>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="15">
@@ -897,10 +1005,22 @@
           <t>Počítá koncepce domu s prací z domova?</t>
         </is>
       </c>
-      <c r="E20" s="13" t="n"/>
-      <c r="F20" s="11" t="n"/>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Při variantě, kdy dvě děti sdílejí dětský pokoj, zůstává samostatná místnost využitelná jako pracovna.</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G20" s="13" t="n"/>
-      <c r="H20" s="13" t="n"/>
+      <c r="H20" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O20" s="13" t="n"/>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="15">
@@ -916,10 +1036,22 @@
           <t>Je dům vhodný i pro rodinu se třemi dětmi?</t>
         </is>
       </c>
-      <c r="E21" s="13" t="n"/>
-      <c r="F21" s="11" t="n"/>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>Ano, pětičlenná rodina se třemi dětmi v domě bydlet může, ale už jde o prostorově náročnější variantu. Jednou z možností je využít větší původní ložnici jako dětský pokoj a ložnici rodičů přesunout do prostoru jiného pokoje, případně na úkor pracovny.</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G21" s="13" t="n"/>
-      <c r="H21" s="13" t="n"/>
+      <c r="H21" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O21" s="13" t="n"/>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="15">
@@ -996,10 +1128,22 @@
           <t>Proč má dům právě dispozici 4+kk?</t>
         </is>
       </c>
-      <c r="E24" s="13" t="n"/>
-      <c r="F24" s="11" t="n"/>
+      <c r="E24" s="13" t="inlineStr">
+        <is>
+          <t>Dispozice 4+kk odpovídá optimálnímu využití pro čtyřčlennou rodinu: společný obytný prostor, ložnice rodičů a dva další pokoje, které lze využít jako dva dětské pokoje nebo jako společný dětský pokoj a pracovnu.</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G24" s="13" t="n"/>
-      <c r="H24" s="13" t="n"/>
+      <c r="H24" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O24" s="13" t="n"/>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="15">
@@ -1146,10 +1290,22 @@
           <t>Co bylo při návrhu důležitější než maximální počet metrů čtverečních?</t>
         </is>
       </c>
-      <c r="E30" s="13" t="n"/>
-      <c r="F30" s="11" t="n"/>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>Důležitější než maximalizovat počet metrů čtverečních bylo dosáhnout co nejvyšší užitné hodnoty zastavěného prostoru, s minimem nevyužitých zákoutí.</t>
+        </is>
+      </c>
+      <c r="F30" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G30" s="13" t="n"/>
-      <c r="H30" s="13" t="n"/>
+      <c r="H30" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O30" s="13" t="n"/>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="15">
@@ -1184,10 +1340,22 @@
           <t>Kdybych měl Bungalov 4KK pochopit ve třech větách, co bych o něm měl vědět?</t>
         </is>
       </c>
-      <c r="E32" s="13" t="n"/>
-      <c r="F32" s="11" t="n"/>
+      <c r="E32" s="13" t="inlineStr">
+        <is>
+          <t>Bungalov 4+kk je nejlépe využitelný jako efektivní bydlení pro čtyřčlennou rodinu. Je navržen tak, aby z minima zastavěného prostoru vytěžil maximum skutečně využitelné plochy. Konstrukce a technologie jsou současně podřízeny nízké energetické náročnosti a schopnosti rychle reagovat na aktuální potřebu tepla.</t>
+        </is>
+      </c>
+      <c r="F32" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G32" s="13" t="n"/>
-      <c r="H32" s="13" t="n"/>
+      <c r="H32" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O32" s="13" t="n"/>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="15">
@@ -1336,7 +1504,7 @@
       </c>
       <c r="E40" s="13" t="inlineStr">
         <is>
-          <t>Studie uvádí, že dům lze dobře osadit do svahu na vrstevnici. Konkrétní vhodnost ale vždy závisí na podmínkách daného pozemku a založení.</t>
+          <t>Ano. Ideální je rovina nebo mírný svah směrem k jihu, jihozápadu nebo východu. Dům lze realizovat i v prudším svahu, ale projeví se to ve vyšší ceně spodní stavby a může se zhoršit přístupnost terasy. Severní svah pro tento dům není příliš vhodný.</t>
         </is>
       </c>
       <c r="F40" s="11" t="inlineStr">
@@ -1347,7 +1515,7 @@
       <c r="G40" s="13" t="n"/>
       <c r="H40" s="13" t="inlineStr">
         <is>
-          <t>Studie Bungalov 4KK / 01.11.2022</t>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
         </is>
       </c>
       <c r="O40" s="13" t="n"/>
@@ -1421,7 +1589,7 @@
       </c>
       <c r="E43" s="13" t="inlineStr">
         <is>
-          <t>Studie pracuje se vstupní „technickou“ stranou na severozápad a zahradní stranou s terasou na jihovýchod. Jde o koncepční orientaci studie, nikoli univerzální podmínku každého pozemku.</t>
+          <t>Ideální je obdélníkový pozemek s příjezdem ze severu, západu nebo východu. Z hlediska terénu je vhodná rovina nebo mírný svah orientovaný k jihu, jihozápadu nebo východu.</t>
         </is>
       </c>
       <c r="F43" s="11" t="inlineStr">
@@ -1432,7 +1600,7 @@
       <c r="G43" s="13" t="n"/>
       <c r="H43" s="13" t="inlineStr">
         <is>
-          <t>Studie Bungalov 4KK / 01.11.2022</t>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
         </is>
       </c>
       <c r="O43" s="13" t="n"/>
@@ -1512,10 +1680,22 @@
           <t>Co když mám zahradu orientovanou na sever?</t>
         </is>
       </c>
-      <c r="E46" s="13" t="n"/>
-      <c r="F46" s="11" t="n"/>
+      <c r="E46" s="13" t="inlineStr">
+        <is>
+          <t>Severní orientace svahu není pro tento dům příliš vhodná. Konkrétní použitelnost ale závisí na osazení domu a podmínkách konkrétního pozemku.</t>
+        </is>
+      </c>
+      <c r="F46" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G46" s="13" t="n"/>
-      <c r="H46" s="13" t="n"/>
+      <c r="H46" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O46" s="13" t="n"/>
     </row>
     <row r="47" ht="15.75" customHeight="1" s="15">
@@ -1550,10 +1730,22 @@
           <t>Co když příjezd na pozemek vede ze severu?</t>
         </is>
       </c>
-      <c r="E48" s="13" t="n"/>
-      <c r="F48" s="11" t="n"/>
+      <c r="E48" s="13" t="inlineStr">
+        <is>
+          <t>Příjezd ze severu patří mezi ideální varianty. Vhodný je také příjezd ze západu nebo východu.</t>
+        </is>
+      </c>
+      <c r="F48" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G48" s="13" t="n"/>
-      <c r="H48" s="13" t="n"/>
+      <c r="H48" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O48" s="13" t="n"/>
     </row>
     <row r="49" ht="15.75" customHeight="1" s="15">
@@ -1906,10 +2098,22 @@
           <t>Jaké vlastnosti pozemku mohou způsobit, že tento dům nebude vhodnou volbou?</t>
         </is>
       </c>
-      <c r="E63" s="13" t="n"/>
-      <c r="F63" s="11" t="n"/>
+      <c r="E63" s="13" t="inlineStr">
+        <is>
+          <t>Problematický je zejména severní svah. Prudký svah realizaci nevylučuje, ale zvyšuje náklady na spodní stavbu a může zhoršit přístupnost terasy.</t>
+        </is>
+      </c>
+      <c r="F63" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G63" s="13" t="n"/>
-      <c r="H63" s="13" t="n"/>
+      <c r="H63" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O63" s="13" t="n"/>
     </row>
     <row r="64" ht="15.75" customHeight="1" s="15">
@@ -2132,10 +2336,22 @@
           <t>Je velikost domu dostatečná pro čtyřčlennou rodinu?</t>
         </is>
       </c>
-      <c r="E72" s="13" t="n"/>
-      <c r="F72" s="11" t="n"/>
+      <c r="E72" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Čtyřčlenná rodina se dvěma dětmi představuje pro tento dům optimální využití.</t>
+        </is>
+      </c>
+      <c r="F72" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G72" s="13" t="n"/>
-      <c r="H72" s="13" t="n"/>
+      <c r="H72" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O72" s="13" t="n"/>
     </row>
     <row r="73" ht="15.75" customHeight="1" s="15">
@@ -2227,10 +2443,22 @@
           <t>Bude dům dostatečně velký i pro pětičlennou rodinu?</t>
         </is>
       </c>
-      <c r="E77" s="13" t="n"/>
-      <c r="F77" s="11" t="n"/>
+      <c r="E77" s="13" t="inlineStr">
+        <is>
+          <t>Pětičlenná rodina se třemi dětmi dům využít může, ale už jde o prostorově stísněnější variantu a je vhodné upravit rozdělení bloku ložnice, dětského pokoje a pracovny.</t>
+        </is>
+      </c>
+      <c r="F77" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G77" s="13" t="n"/>
-      <c r="H77" s="13" t="n"/>
+      <c r="H77" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O77" s="13" t="n"/>
     </row>
     <row r="78" ht="15.75" customHeight="1" s="15">
@@ -2708,10 +2936,22 @@
           <t>Dá se dispozice domu změnit?</t>
         </is>
       </c>
-      <c r="E98" s="13" t="n"/>
-      <c r="F98" s="11" t="n"/>
+      <c r="E98" s="13" t="inlineStr">
+        <is>
+          <t>Ano, ale smysluplná variabilita se týká především bloku ložnice, dětského pokoje a pracovny. Zde lze měnit polohu příček a tím velikost a využití jednotlivých místností.</t>
+        </is>
+      </c>
+      <c r="F98" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G98" s="13" t="n"/>
-      <c r="H98" s="13" t="n"/>
+      <c r="H98" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O98" s="13" t="n"/>
     </row>
     <row r="99" ht="15.75" customHeight="1" s="15">
@@ -2808,10 +3048,22 @@
           <t>Dá se některý pokoj zvětšit na úkor jiného prostoru?</t>
         </is>
       </c>
-      <c r="E102" s="13" t="n"/>
-      <c r="F102" s="11" t="n"/>
+      <c r="E102" s="13" t="inlineStr">
+        <is>
+          <t>Ano. V bloku ložnice, dětského pokoje a pracovny lze posunem příček zvětšit jednu místnost na úkor druhé.</t>
+        </is>
+      </c>
+      <c r="F102" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G102" s="13" t="n"/>
-      <c r="H102" s="13" t="n"/>
+      <c r="H102" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O102" s="13" t="n"/>
     </row>
     <row r="103" ht="15.75" customHeight="1" s="15">
@@ -2915,10 +3167,22 @@
           <t>Jaké jsou hlavní kompromisy této dispozice?</t>
         </is>
       </c>
-      <c r="E107" s="13" t="n"/>
-      <c r="F107" s="11" t="n"/>
+      <c r="E107" s="13" t="inlineStr">
+        <is>
+          <t>Hlavním kompromisem dispozice je její podlouhlost. Úzký rozpon domu přibližně 5,6 m vede k délce okolo 20 m, takže vzdálenosti mezi jednotlivými částmi domu jsou větší.</t>
+        </is>
+      </c>
+      <c r="F107" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G107" s="13" t="n"/>
-      <c r="H107" s="13" t="n"/>
+      <c r="H107" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O107" s="13" t="n"/>
     </row>
     <row r="108" ht="15.75" customHeight="1" s="15">
@@ -3222,10 +3486,22 @@
           <t>Které prvky domu lze měnit bez zásahu do jeho základního konceptu?</t>
         </is>
       </c>
-      <c r="E122" s="13" t="n"/>
-      <c r="F122" s="11" t="n"/>
+      <c r="E122" s="13" t="inlineStr">
+        <is>
+          <t>Bez narušení základního konceptu dává největší smysl měnit dispozici bloku ložnice, dětského pokoje a pracovny pomocí posunu příček.</t>
+        </is>
+      </c>
+      <c r="F122" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G122" s="13" t="n"/>
-      <c r="H122" s="13" t="n"/>
+      <c r="H122" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O122" s="13" t="n"/>
     </row>
     <row r="123" ht="15.75" customHeight="1" s="15">
@@ -3353,10 +3629,22 @@
           <t>Jak daleko lze s individualizací zajít, aby dům stále fungoval tak, jak byl navržen?</t>
         </is>
       </c>
-      <c r="E127" s="13" t="n"/>
-      <c r="F127" s="11" t="n"/>
+      <c r="E127" s="13" t="inlineStr">
+        <is>
+          <t>Smysluplná individualizace je především v bloku ložnice, dětského pokoje a pracovny. Zásadnější změny ostatních částí domu už podle autora nedávají z hlediska původního konceptu příliš smysl.</t>
+        </is>
+      </c>
+      <c r="F127" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G127" s="13" t="n"/>
-      <c r="H127" s="13" t="n"/>
+      <c r="H127" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O127" s="13" t="n"/>
     </row>
     <row r="128" ht="15.75" customHeight="1" s="15">
@@ -3408,10 +3696,22 @@
           <t>Dá se dispozice domu upravit podle našich potřeb?</t>
         </is>
       </c>
-      <c r="E130" s="13" t="n"/>
-      <c r="F130" s="11" t="n"/>
+      <c r="E130" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Největší smysl má úprava bloku ložnice, dětského pokoje a pracovny, kde lze posouvat příčky a měnit velikost a funkci místností.</t>
+        </is>
+      </c>
+      <c r="F130" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G130" s="13" t="n"/>
-      <c r="H130" s="13" t="n"/>
+      <c r="H130" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O130" s="13" t="n"/>
     </row>
     <row r="131" ht="15.75" customHeight="1" s="15">
@@ -3427,10 +3727,22 @@
           <t>Jaké změny můžeme udělat před zahájením stavby?</t>
         </is>
       </c>
-      <c r="E131" s="13" t="n"/>
-      <c r="F131" s="11" t="n"/>
+      <c r="E131" s="13" t="inlineStr">
+        <is>
+          <t>Před stavbou lze smysluplně upravovat zejména polohu příček v bloku ložnice, dětského pokoje a pracovny.</t>
+        </is>
+      </c>
+      <c r="F131" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G131" s="13" t="n"/>
-      <c r="H131" s="13" t="n"/>
+      <c r="H131" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O131" s="13" t="n"/>
     </row>
     <row r="132" ht="15.75" customHeight="1" s="15">
@@ -3446,10 +3758,22 @@
           <t>Dá se některý pokoj zvětšit nebo zmenšit?</t>
         </is>
       </c>
-      <c r="E132" s="13" t="n"/>
-      <c r="F132" s="11" t="n"/>
+      <c r="E132" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Posunem příček lze měnit velikost místností zejména v bloku ložnice, dětského pokoje a pracovny.</t>
+        </is>
+      </c>
+      <c r="F132" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G132" s="13" t="n"/>
-      <c r="H132" s="13" t="n"/>
+      <c r="H132" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O132" s="13" t="n"/>
     </row>
     <row r="133" ht="15.75" customHeight="1" s="15">
@@ -3565,10 +3889,22 @@
           <t>Lze později změnit využití jednotlivých místností?</t>
         </is>
       </c>
-      <c r="E137" s="13" t="n"/>
-      <c r="F137" s="11" t="n"/>
+      <c r="E137" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Zejména blok ložnice, dětského pokoje a pracovny lze díky úpravám příček přizpůsobovat měnícím se potřebám rodiny.</t>
+        </is>
+      </c>
+      <c r="F137" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G137" s="13" t="n"/>
-      <c r="H137" s="13" t="n"/>
+      <c r="H137" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O137" s="13" t="n"/>
     </row>
     <row r="138" ht="15.75" customHeight="1" s="15">
@@ -3622,10 +3958,22 @@
           <t>Lze dům přizpůsobit pětičlenné rodině?</t>
         </is>
       </c>
-      <c r="E140" s="13" t="n"/>
-      <c r="F140" s="11" t="n"/>
+      <c r="E140" s="13" t="inlineStr">
+        <is>
+          <t>Ano, ale s kompromisem. Pro tři děti lze například větší původní ložnici využít jako dětský pokoj a ložnici rodičů přesunout do prostoru dalšího pokoje, případně tím obětovat samostatnou pracovnu.</t>
+        </is>
+      </c>
+      <c r="F140" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G140" s="13" t="n"/>
-      <c r="H140" s="13" t="n"/>
+      <c r="H140" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O140" s="13" t="n"/>
     </row>
     <row r="141" ht="15.75" customHeight="1" s="15">
@@ -3817,10 +4165,22 @@
           <t>Jak dobře se dům dokáže přizpůsobit změnám potřeb rodiny v průběhu života?</t>
         </is>
       </c>
-      <c r="E149" s="13" t="n"/>
-      <c r="F149" s="11" t="n"/>
+      <c r="E149" s="13" t="inlineStr">
+        <is>
+          <t>Dům se dokáže přizpůsobovat změnám potřeb rodiny především variabilitou bloku ložnice, dětského pokoje a pracovny, kde lze měnit polohu příček a využití jednotlivých místností.</t>
+        </is>
+      </c>
+      <c r="F149" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G149" s="13" t="n"/>
-      <c r="H149" s="13" t="n"/>
+      <c r="H149" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O149" s="13" t="n"/>
     </row>
     <row r="150" ht="15.75" customHeight="1" s="15">
@@ -3853,10 +4213,22 @@
           <t>Jakým způsobem se tento dům realizuje?</t>
         </is>
       </c>
-      <c r="E151" s="13" t="n"/>
-      <c r="F151" s="11" t="n"/>
+      <c r="E151" s="13" t="inlineStr">
+        <is>
+          <t>Standardním režimem je dodávka projektu, spodní stavby a hrubé stavby domu. Pokud už klient vlastní pozemek, dům se nejprve osadí na konkrétní parcelu ve studii a následně se zpracuje projektová dokumentace a realizace. Pro klienta bez pozemku lze pracovat s připravenými koncepty domu na konkrétních pozemcích.</t>
+        </is>
+      </c>
+      <c r="F151" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G151" s="13" t="n"/>
-      <c r="H151" s="13" t="n"/>
+      <c r="H151" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O151" s="13" t="n"/>
     </row>
     <row r="152" ht="15.75" customHeight="1" s="15">
@@ -3872,10 +4244,22 @@
           <t>Dodává se dům na klíč?</t>
         </is>
       </c>
-      <c r="E152" s="13" t="n"/>
-      <c r="F152" s="11" t="n"/>
+      <c r="E152" s="13" t="inlineStr">
+        <is>
+          <t>Dům lze dodat kompletně na klíč, ale standardně není klient nucen odebrat kompletní dokončení. Základní model umožňuje převzít hrubou stavbu a další technologie, interiéry a designové prvky řešit individuálně.</t>
+        </is>
+      </c>
+      <c r="F152" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G152" s="13" t="n"/>
-      <c r="H152" s="13" t="n"/>
+      <c r="H152" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O152" s="13" t="n"/>
     </row>
     <row r="153" ht="15.75" customHeight="1" s="15">
@@ -3891,10 +4275,22 @@
           <t>Co všechno je součástí dodávky domu?</t>
         </is>
       </c>
-      <c r="E153" s="13" t="n"/>
-      <c r="F153" s="11" t="n"/>
+      <c r="E153" s="13" t="inlineStr">
+        <is>
+          <t>Standardní dodávka zahrnuje projektovou dokumentaci, spodní stavbu a hrubou stavbu zakončenou fasádou a okny, připravenou pro navazující instalace a technologie. Část technického minima se provádí už během hrubé stavby.</t>
+        </is>
+      </c>
+      <c r="F153" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G153" s="13" t="n"/>
-      <c r="H153" s="13" t="n"/>
+      <c r="H153" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O153" s="13" t="n"/>
     </row>
     <row r="154" ht="15.75" customHeight="1" s="15">
@@ -4005,10 +4401,22 @@
           <t>Lze si vybrat, v jakém stupni dokončení dům převezmu?</t>
         </is>
       </c>
-      <c r="E159" s="13" t="n"/>
-      <c r="F159" s="11" t="n"/>
+      <c r="E159" s="13" t="inlineStr">
+        <is>
+          <t>Ano. Standardem je hrubá stavba připravená pro navazující instalace a technologie, ale je možné zajistit také kompletní realizaci na klíč. Klient tak nemusí povinně odebírat všechny dokončovací, designové a interiérové práce.</t>
+        </is>
+      </c>
+      <c r="F159" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G159" s="13" t="n"/>
-      <c r="H159" s="13" t="n"/>
+      <c r="H159" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O159" s="13" t="n"/>
     </row>
     <row r="160" ht="15.75" customHeight="1" s="15">
@@ -4269,10 +4677,22 @@
           <t>Co všechno je zahrnuté v ceně domu?</t>
         </is>
       </c>
-      <c r="E173" s="13" t="n"/>
-      <c r="F173" s="11" t="n"/>
+      <c r="E173" s="13" t="inlineStr">
+        <is>
+          <t>Ve standardním rozsahu dodávky jsou projektová dokumentace, spodní stavba a hrubá stavba zakončená fasádou a okny, připravená pro instalace a technologie. Část nezbytného technického minima vzniká už během hrubé stavby.</t>
+        </is>
+      </c>
+      <c r="F173" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G173" s="13" t="n"/>
-      <c r="H173" s="13" t="n"/>
+      <c r="H173" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O173" s="13" t="n"/>
     </row>
     <row r="174" ht="15.75" customHeight="1" s="15">
@@ -4288,10 +4708,22 @@
           <t>Co naopak v základní ceně není?</t>
         </is>
       </c>
-      <c r="E174" s="13" t="n"/>
-      <c r="F174" s="11" t="n"/>
+      <c r="E174" s="13" t="inlineStr">
+        <is>
+          <t>Standardní rozsah hrubé stavby automaticky neznamená kompletní dokončení interiéru a všech technologií na klíč. Tyto části lze řešit individuálně podle požadavků klienta.</t>
+        </is>
+      </c>
+      <c r="F174" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G174" s="13" t="n"/>
-      <c r="H174" s="13" t="n"/>
+      <c r="H174" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O174" s="13" t="n"/>
     </row>
     <row r="175" ht="15.75" customHeight="1" s="15">
@@ -8118,7 +8550,7 @@
       </c>
       <c r="E330" s="13" t="inlineStr">
         <is>
-          <t>Lehká konstrukce má menší tepelnou akumulaci, takže na změnu topného režimu reaguje rychleji než těžká zděná konstrukce.</t>
+          <t>Dům má relativně malou tepelnou setrvačnost, takže při změně provozního režimu reaguje na ztrátu tepla rychleji než těžká zděná stavba. Současně vnitřní Ekopanel 60 poskytuje určitou míru tepelné akumulace.</t>
         </is>
       </c>
       <c r="F330" s="11" t="inlineStr">
@@ -8129,7 +8561,7 @@
       <c r="G330" s="13" t="n"/>
       <c r="H330" s="13" t="inlineStr">
         <is>
-          <t>E-book Jak se staví Domy s energií / KOMPLET</t>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
         </is>
       </c>
       <c r="O330" s="13" t="n"/>
@@ -8149,7 +8581,7 @@
       </c>
       <c r="E331" s="13" t="inlineStr">
         <is>
-          <t>Díky lehké konstrukci s malou tepelnou akumulací lze dům po změně topného režimu znovu tepelně stabilizovat relativně rychle.</t>
+          <t>Díky relativně malé tepelné setrvačnosti dům reaguje na požadavek vytápění rychle. To umožňuje pružně měnit tepelnou pohodu podle toho, zda je dům právě využíván.</t>
         </is>
       </c>
       <c r="F331" s="11" t="inlineStr">
@@ -8160,7 +8592,7 @@
       <c r="G331" s="13" t="n"/>
       <c r="H331" s="13" t="inlineStr">
         <is>
-          <t>E-book Jak se staví Domy s energií / KOMPLET</t>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
         </is>
       </c>
       <c r="O331" s="13" t="n"/>
@@ -8311,7 +8743,7 @@
       </c>
       <c r="E337" s="13" t="inlineStr">
         <is>
-          <t>Ano, zejména tepelnou akumulací. E-book popisuje tuto dřevostavbu jako lehkou konstrukci s menší tepelnou akumulací než těžká zděná stavba, takže rychleji reaguje na změny vytápění i vnitřních tepelných podmínek.</t>
+          <t>Ano. Oproti těžké zděné stavbě má dům menší tepelnou setrvačnost a rychleji reaguje na změny vytápění. Současně Ekopanel 60 přináší určitou akumulaci, takže nejde o konstrukci zcela bez akumulační schopnosti.</t>
         </is>
       </c>
       <c r="F337" s="11" t="inlineStr">
@@ -8322,7 +8754,7 @@
       <c r="G337" s="13" t="n"/>
       <c r="H337" s="13" t="inlineStr">
         <is>
-          <t>E-book Jak se staví Domy s energií / KOMPLET</t>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
         </is>
       </c>
       <c r="O337" s="13" t="n"/>
@@ -9470,22 +9902,18 @@
       </c>
       <c r="E382" s="12" t="inlineStr">
         <is>
-          <t>Vytápění zajišťuje tepelné čerpadlo doplněné krbem s tepelným zásobníkem.</t>
+          <t>Hlavní vytápění zajišťuje cirkulační vzduchové vytápění prostřednictvím rekuperační jednotky Zehnder s klimatizačním modulem. Klimatizační modul v zimě vzduch ohřívá. V nejchladnějších dnech jej doplňuje elektrické podlahové vytápění topnými fóliemi.</t>
         </is>
       </c>
       <c r="F382" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G382" s="13" t="inlineStr">
-        <is>
-          <t>Krbové těleso bylo z aktuální klientské konfigurace vypuštěno. Dostupné CURRENT podklady zatím neumožňují bezpečně označit jediný hlavní systém vytápění.</t>
-        </is>
-      </c>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G382" s="13" t="inlineStr"/>
       <c r="H382" s="12" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / Klientské změny č. 2 / 20.10.2023</t>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
         </is>
       </c>
       <c r="O382" s="13" t="n"/>
@@ -9505,22 +9933,18 @@
       </c>
       <c r="E383" s="12" t="inlineStr">
         <is>
-          <t>Vytápění zajišťuje tepelné čerpadlo a dvouplášťový krb napojený na zásobník tepla.</t>
+          <t>Dům používá cirkulační vzduchové vytápění integrované do systému řízeného větrání Zehnder s klimatizačním modulem. Pro nejchladnější období je doplněno elektrickými topnými fóliemi v podlaze.</t>
         </is>
       </c>
       <c r="F383" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G383" s="13" t="inlineStr">
-        <is>
-          <t>Krbové těleso bylo z aktuální klientské konfigurace vypuštěno. Zehnder je CURRENT řešení řízeného větrání/rekuperace; samotná informace o Zehnderu nedokládá hlavní systém vytápění. Hlavní systém vytápění je nutné ještě jednoznačně potvrdit.</t>
-        </is>
-      </c>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G383" s="13" t="inlineStr"/>
       <c r="H383" s="12" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK / Validace autora domu / CURRENT / 2026-09-09 / Klientské změny č. 2 / 20.10.2023</t>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
         </is>
       </c>
       <c r="O383" s="13" t="n"/>
@@ -9668,7 +10092,7 @@
       </c>
       <c r="E388" s="12" t="inlineStr">
         <is>
-          <t>Ano. Tepelné čerpadlo v rekuperační jednotce funguje v létě také jako klimatizace.</t>
+          <t>Ano. Klimatizační modul rekuperační jednotky Zehnder v létě zajišťuje chlazení domu.</t>
         </is>
       </c>
       <c r="F388" s="11" t="inlineStr">
@@ -9679,7 +10103,7 @@
       <c r="G388" s="13" t="n"/>
       <c r="H388" s="12" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
         </is>
       </c>
       <c r="O388" s="13" t="n"/>
@@ -9699,7 +10123,7 @@
       </c>
       <c r="E389" s="12" t="inlineStr">
         <is>
-          <t>Tepelné čerpadlo v rekuperační jednotce funguje v létě také jako klimatizace.</t>
+          <t>Ano. Chlazení je integrováno do rekuperační jednotky Zehnder prostřednictvím klimatizačního modulu.</t>
         </is>
       </c>
       <c r="F389" s="11" t="inlineStr">
@@ -9710,7 +10134,7 @@
       <c r="G389" s="13" t="n"/>
       <c r="H389" s="12" t="inlineStr">
         <is>
-          <t>domysenergii.cz / DŮM 002 / Bungalov 4KK</t>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
         </is>
       </c>
       <c r="O389" s="13" t="n"/>
@@ -15464,7 +15888,7 @@
       </c>
       <c r="E661" s="13" t="inlineStr">
         <is>
-          <t>Servisní intervaly technologií nejsou pro všechny prvky domu v dostupných podkladech jednotně stanoveny. Řídí se dokumentací a servisními požadavky konkrétních výrobců jednotlivých zařízení.</t>
+          <t>Servis technologií se řídí požadavky konkrétního výrobce a dodavatele. Intervaly a podmínky jsou uvedeny v návodech, záručních listech a předávacích protokolech jednotlivých zařízení.</t>
         </is>
       </c>
       <c r="F661" s="11" t="inlineStr">
@@ -15475,7 +15899,7 @@
       <c r="G661" s="13" t="n"/>
       <c r="H661" s="13" t="inlineStr">
         <is>
-          <t>B Souhrnná technická zpráva 11/2023</t>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
         </is>
       </c>
       <c r="O661" s="13" t="n"/>
@@ -15493,10 +15917,22 @@
           <t>Kdo zajišťuje servis po předání domu?</t>
         </is>
       </c>
-      <c r="E662" s="13" t="n"/>
-      <c r="F662" s="11" t="n"/>
+      <c r="E662" s="13" t="inlineStr">
+        <is>
+          <t>Servis jednotlivých technologií zajišťuje jejich konkrétní dodavatel podle podmínek uvedených v záručních listech, předávacích protokolech a návodech.</t>
+        </is>
+      </c>
+      <c r="F662" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G662" s="13" t="n"/>
-      <c r="H662" s="13" t="n"/>
+      <c r="H662" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O662" s="13" t="n"/>
     </row>
     <row r="663" ht="15.75" customHeight="1" s="15">
@@ -15512,10 +15948,22 @@
           <t>Jak dlouhá je záruka na dům?</t>
         </is>
       </c>
-      <c r="E663" s="13" t="n"/>
-      <c r="F663" s="11" t="n"/>
+      <c r="E663" s="13" t="inlineStr">
+        <is>
+          <t>Na dům platí zákonná záruka v délce pěti let.</t>
+        </is>
+      </c>
+      <c r="F663" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G663" s="13" t="n"/>
-      <c r="H663" s="13" t="n"/>
+      <c r="H663" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O663" s="13" t="n"/>
     </row>
     <row r="664" ht="15.75" customHeight="1" s="15">
@@ -15531,10 +15979,22 @@
           <t>Jaké záruky platí na jednotlivé konstrukce a technologie?</t>
         </is>
       </c>
-      <c r="E664" s="13" t="n"/>
-      <c r="F664" s="11" t="n"/>
+      <c r="E664" s="13" t="inlineStr">
+        <is>
+          <t>Na samotný dům platí zákonná pětiletá záruka. U jednotlivých technologií se konkrétní záruční a servisní podmínky řídí jejich záručními listy, předávacími protokoly a dokumentací výrobce.</t>
+        </is>
+      </c>
+      <c r="F664" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G664" s="13" t="n"/>
-      <c r="H664" s="13" t="n"/>
+      <c r="H664" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O664" s="13" t="n"/>
     </row>
     <row r="665" ht="15.75" customHeight="1" s="15">
@@ -15735,7 +16195,7 @@
       </c>
       <c r="E674" s="13" t="inlineStr">
         <is>
-          <t>Pro dlouhou životnost je důležité chránit konstrukci před dlouhodobou vlhkostí, udržovat venkovní dřevěné prvky a provádět servis technických zařízení podle požadavků jejich výrobců.</t>
+          <t>Dům je koncipován pro minimální údržbu. Pravidelnou povrchovou údržbu vyžadují především venkovní dřevěné části, například konstrukce přístřešku, terasové dřevěné prvky a dřevěný obklad, obvykle v intervalu přibližně 6 až 10 let. Technologie se servisují podle požadavků jejich výrobců a dodavatelů.</t>
         </is>
       </c>
       <c r="F674" s="11" t="inlineStr">
@@ -15746,7 +16206,7 @@
       <c r="G674" s="13" t="n"/>
       <c r="H674" s="13" t="inlineStr">
         <is>
-          <t>B Souhrnná technická zpráva 11/2023 / Studie Bungalov 4KK / 01.11.2022</t>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
         </is>
       </c>
       <c r="O674" s="13" t="n"/>
@@ -15781,10 +16241,22 @@
           <t>Jaké jsou největší nevýhody tohoto domu?</t>
         </is>
       </c>
-      <c r="E676" s="13" t="n"/>
-      <c r="F676" s="11" t="n"/>
+      <c r="E676" s="13" t="inlineStr">
+        <is>
+          <t>Největší nevýhodou domu je jeho podlouhlý tvar. Úzký rozpon přibližně 5,6 m prodlužuje dům přibližně na 20 m a zvětšuje vzdálenosti mezi jeho jednotlivými částmi.</t>
+        </is>
+      </c>
+      <c r="F676" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G676" s="13" t="n"/>
-      <c r="H676" s="13" t="n"/>
+      <c r="H676" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O676" s="13" t="n"/>
     </row>
     <row r="677" ht="15.75" customHeight="1" s="15">
@@ -15819,10 +16291,22 @@
           <t>Jaké jsou hlavní kompromisy této dispozice?</t>
         </is>
       </c>
-      <c r="E678" s="13" t="n"/>
-      <c r="F678" s="11" t="n"/>
+      <c r="E678" s="13" t="inlineStr">
+        <is>
+          <t>Hlavním kompromisem je výměna velmi efektivního úzkého půdorysu za větší délku domu a delší komunikační vzdálenosti uvnitř.</t>
+        </is>
+      </c>
+      <c r="F678" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G678" s="13" t="n"/>
-      <c r="H678" s="13" t="n"/>
+      <c r="H678" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O678" s="13" t="n"/>
     </row>
     <row r="679" ht="15.75" customHeight="1" s="15">
@@ -15838,10 +16322,22 @@
           <t>Co bych měl o tomto domě vědět předtím, než se pro něj rozhodnu?</t>
         </is>
       </c>
-      <c r="E679" s="13" t="n"/>
-      <c r="F679" s="11" t="n"/>
+      <c r="E679" s="13" t="inlineStr">
+        <is>
+          <t>Před rozhodnutím je dobré vědět především to, že dům je záměrně úzký a podlouhlý. Díky tomu efektivně využívá prostor, ale při délce přibližně 20 m vznikají větší vzdálenosti mezi jednotlivými částmi domu.</t>
+        </is>
+      </c>
+      <c r="F679" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G679" s="13" t="n"/>
-      <c r="H679" s="13" t="n"/>
+      <c r="H679" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O679" s="13" t="n"/>
     </row>
     <row r="680" ht="15.75" customHeight="1" s="15">
@@ -15952,10 +16448,22 @@
           <t>Jaké vlastnosti pozemku mohou realizaci tohoto domu výrazně zkomplikovat?</t>
         </is>
       </c>
-      <c r="E685" s="13" t="n"/>
-      <c r="F685" s="11" t="n"/>
+      <c r="E685" s="13" t="inlineStr">
+        <is>
+          <t>Realizaci může výrazně zkomplikovat prudký svah, protože se promítá do ceny spodní stavby a přístupnosti terasy. Severní svah je pro tento koncept méně vhodný.</t>
+        </is>
+      </c>
+      <c r="F685" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G685" s="13" t="n"/>
-      <c r="H685" s="13" t="n"/>
+      <c r="H685" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O685" s="13" t="n"/>
     </row>
     <row r="686" ht="15.75" customHeight="1" s="15">
@@ -16085,10 +16593,22 @@
           <t>Které vlastnosti domu jsou věcí osobní preference a mohou někomu vadit?</t>
         </is>
       </c>
-      <c r="E692" s="13" t="n"/>
-      <c r="F692" s="11" t="n"/>
+      <c r="E692" s="13" t="inlineStr">
+        <is>
+          <t>Někomu může vadit podlouhlá dispozice domu a větší vzdálenosti mezi jeho jednotlivými částmi. Je to přímý důsledek úzkého konstrukčního rozponu a efektivního využití zastavěného prostoru.</t>
+        </is>
+      </c>
+      <c r="F692" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G692" s="13" t="n"/>
-      <c r="H692" s="13" t="n"/>
+      <c r="H692" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O692" s="13" t="n"/>
     </row>
     <row r="693" ht="15.75" customHeight="1" s="15">
@@ -16104,10 +16624,22 @@
           <t>Jaký kompromis dělá Bungalov 4KK výměnou za svou relativně kompaktní velikost?</t>
         </is>
       </c>
-      <c r="E693" s="13" t="n"/>
-      <c r="F693" s="11" t="n"/>
+      <c r="E693" s="13" t="inlineStr">
+        <is>
+          <t>Za prostorovou efektivitu a úzký rozpon dům platí větší celkovou délkou a delšími vzdálenostmi mezi jednotlivými částmi.</t>
+        </is>
+      </c>
+      <c r="F693" s="11" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
       <c r="G693" s="13" t="n"/>
-      <c r="H693" s="13" t="n"/>
+      <c r="H693" s="13" t="inlineStr">
+        <is>
+          <t>Validace autora domu / CURRENT / 2026-09-10</t>
+        </is>
+      </c>
       <c r="O693" s="13" t="n"/>
     </row>
     <row r="694" ht="15.75" customHeight="1" s="15">

</xml_diff>